<commit_message>
add histogram template drawer
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10FB4223-7B09-4ADD-8153-42D50F9B2751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730CCF94-B1EE-4245-B799-2C4A1F0AC561}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="180" formatCode="0.000000"/>
+    <numFmt numFmtId="176" formatCode="0.000000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -67,7 +67,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -356,180 +356,172 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>0</v>
+        <v>7.3980600000000001</v>
       </c>
       <c r="B1" s="1">
-        <v>0</v>
+        <v>3.3006820000000001</v>
       </c>
       <c r="C1" s="1">
-        <v>0</v>
+        <v>0.189438</v>
       </c>
       <c r="D1" s="1">
-        <v>0</v>
+        <v>3.5541999999999997E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>0</v>
+        <v>1.4352999999999999E-2</v>
       </c>
       <c r="F1" s="1">
-        <v>0</v>
+        <v>1.6746E-2</v>
       </c>
       <c r="G1" s="1">
         <v>0</v>
       </c>
       <c r="H1" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="I1" s="1">
         <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>0</v>
+        <v>8.7829000000000004E-2</v>
       </c>
       <c r="K1" s="1">
         <v>0</v>
       </c>
       <c r="L1" s="1">
-        <v>0</v>
+        <v>1.3669999999999999E-3</v>
       </c>
       <c r="M1" s="1">
-        <v>0</v>
+        <v>3.4169999999999999E-3</v>
       </c>
       <c r="N1" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="O1" s="1">
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>0</v>
+        <v>7.8899999999999999E-4</v>
       </c>
       <c r="Q1" s="1">
-        <v>0</v>
+        <v>0.37600099999999997</v>
       </c>
       <c r="R1" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="S1" s="1">
-        <v>0</v>
+        <v>3.3779000000000003E-2</v>
       </c>
       <c r="T1" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="U1" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="V1" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="W1" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="X1" s="1">
         <v>0</v>
       </c>
       <c r="Y1" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="Z1" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="AA1" s="1">
         <v>0</v>
       </c>
       <c r="AB1" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC1" s="1">
         <v>0</v>
       </c>
       <c r="AD1" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AE1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI1" s="1">
-        <v>0</v>
-      </c>
+        <v>0.26475500000000002</v>
+      </c>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>1.2849999999999999E-3</v>
+        <v>1.3500000000000001E-3</v>
       </c>
       <c r="B2" s="1">
-        <v>6.4267000000000005E-2</v>
+        <v>0.52445399999999998</v>
       </c>
       <c r="C2" s="1">
-        <v>0</v>
+        <v>1.804E-3</v>
       </c>
       <c r="D2" s="1">
-        <v>0.696658</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="E2" s="1">
-        <v>0</v>
+        <v>3.0760000000000002E-3</v>
       </c>
       <c r="F2" s="1">
-        <v>1.9279999999999999E-2</v>
+        <v>1.709E-3</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
       </c>
       <c r="H2" s="1">
-        <v>1.2849999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="I2" s="1">
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>0</v>
+        <v>3.1440999999999997E-2</v>
       </c>
       <c r="K2" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="L2" s="1">
-        <v>1.5424E-2</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="O2" s="1">
         <v>0</v>
       </c>
       <c r="P2" s="1">
-        <v>0</v>
+        <v>3.9500000000000001E-4</v>
       </c>
       <c r="Q2" s="1">
-        <v>0</v>
+        <v>2.9480000000000001E-3</v>
       </c>
       <c r="R2" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="S2" s="1">
-        <v>1.5424E-2</v>
+        <v>5.8599999999999998E-3</v>
       </c>
       <c r="T2" s="1">
         <v>0</v>
       </c>
       <c r="U2" s="1">
-        <v>1.0283E-2</v>
+        <v>0</v>
       </c>
       <c r="V2" s="1">
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>3.8560000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="X2" s="1">
         <v>0</v>
@@ -538,13 +530,13 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AA2" s="1">
         <v>0</v>
       </c>
       <c r="AB2" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC2" s="1">
         <v>0</v>
@@ -553,20 +545,12 @@
         <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="1">
-        <v>0.172237</v>
-      </c>
+        <v>2.0168999999999999E-2</v>
+      </c>
+      <c r="AF2" s="1"/>
+      <c r="AG2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
@@ -576,31 +560,31 @@
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>9.7825999999999996E-2</v>
+        <v>1.491061</v>
       </c>
       <c r="D3" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>0.87681200000000004</v>
+        <v>0.126447</v>
       </c>
       <c r="F3" s="1">
-        <v>7.2459999999999998E-3</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G3" s="1">
-        <v>3.6229999999999999E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="J3" s="1">
         <v>0</v>
       </c>
       <c r="K3" s="1">
-        <v>0</v>
+        <v>2.7339999999999999E-3</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -615,31 +599,31 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>0</v>
+        <v>3.947E-3</v>
       </c>
       <c r="Q3" s="1">
-        <v>0</v>
+        <v>2.0170000000000001E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>0</v>
+        <v>4.62E-3</v>
       </c>
       <c r="S3" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="T3" s="1">
-        <v>0</v>
+        <v>8.2719999999999998E-3</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
       </c>
       <c r="V3" s="1">
-        <v>0</v>
+        <v>4.1359999999999999E-3</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>3.6229999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="1">
         <v>0</v>
@@ -660,48 +644,40 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI3" s="1">
-        <v>1.0869999999999999E-2</v>
-      </c>
+        <v>7.1799999999999998E-3</v>
+      </c>
+      <c r="AF3" s="1"/>
+      <c r="AG3" s="1"/>
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="1"/>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
-        <v>2.5850000000000001E-3</v>
+        <v>4.4999999999999999E-4</v>
       </c>
       <c r="B4" s="1">
-        <v>3.6189999999999998E-3</v>
+        <v>1.804E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>5.1699999999999999E-4</v>
+        <v>7.2160000000000002E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>2.068E-3</v>
+        <v>0.58746500000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>0</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="F4" s="1">
-        <v>0.945191</v>
+        <v>0.169849</v>
       </c>
       <c r="G4" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="H4" s="1">
-        <v>4.6540000000000002E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="I4" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="J4" s="1">
         <v>0</v>
@@ -710,13 +686,13 @@
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>5.1699999999999999E-4</v>
+        <v>9.9109999999999997E-3</v>
       </c>
       <c r="M4" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="N4" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="O4" s="1">
         <v>0</v>
@@ -725,34 +701,34 @@
         <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <v>0</v>
+        <v>2.3442999999999999E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>3.1020000000000002E-3</v>
+        <v>4.8260000000000004E-3</v>
       </c>
       <c r="T4" s="1">
         <v>0</v>
       </c>
       <c r="U4" s="1">
-        <v>2.068E-3</v>
+        <v>3.447E-3</v>
       </c>
       <c r="V4" s="1">
         <v>0</v>
       </c>
       <c r="W4" s="1">
-        <v>2.4819000000000001E-2</v>
+        <v>1.379E-3</v>
       </c>
       <c r="X4" s="1">
-        <v>1.5510000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="1">
-        <v>3.1020000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="1">
-        <v>5.1699999999999999E-4</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AA4" s="1">
         <v>0</v>
@@ -767,60 +743,52 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI4" s="1">
-        <v>5.6880000000000003E-3</v>
-      </c>
+        <v>2.4278999999999998E-2</v>
+      </c>
+      <c r="AF4" s="1"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="1"/>
+      <c r="AI4" s="1"/>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="B5" s="1">
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>2.0500000000000002E-3</v>
       </c>
       <c r="F5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="G5" s="1">
-        <v>0.85833300000000001</v>
+        <v>0</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>5.5560000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="J5" s="1">
         <v>0</v>
       </c>
       <c r="K5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
       </c>
       <c r="M5" s="1">
-        <v>8.3330000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="N5" s="1">
         <v>0</v>
@@ -835,7 +803,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="S5" s="1">
         <v>0</v>
@@ -844,16 +812,16 @@
         <v>0</v>
       </c>
       <c r="U5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="W5" s="1">
-        <v>1.1110999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>3.0556E-2</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="1">
         <v>0</v>
@@ -868,57 +836,49 @@
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>5.5560000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="1">
-        <v>2.7780000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="1">
         <v>0</v>
       </c>
-      <c r="AF5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI5" s="1">
-        <v>6.1110999999999999E-2</v>
-      </c>
+      <c r="AF5" s="1"/>
+      <c r="AG5" s="1"/>
+      <c r="AH5" s="1"/>
+      <c r="AI5" s="1"/>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>0</v>
       </c>
       <c r="B6" s="1">
-        <v>4.4250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>4.4250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>3.0973000000000001E-2</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G6" s="1">
-        <v>4.4250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>0.73008799999999996</v>
+        <v>0</v>
       </c>
       <c r="I6" s="1">
         <v>0</v>
       </c>
       <c r="J6" s="1">
-        <v>8.8500000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
@@ -930,7 +890,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="1">
-        <v>3.5397999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="O6" s="1">
         <v>0</v>
@@ -957,19 +917,19 @@
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>2.6549E-2</v>
+        <v>0</v>
       </c>
       <c r="X6" s="1">
-        <v>4.4250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="1">
-        <v>4.4248000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="1">
-        <v>4.4250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="1">
-        <v>8.8500000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="AB6" s="1">
         <v>0</v>
@@ -978,23 +938,15 @@
         <v>0</v>
       </c>
       <c r="AD6" s="1">
-        <v>1.3273999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="1">
-        <v>4.4250000000000001E-3</v>
-      </c>
-      <c r="AF6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI6" s="1">
-        <v>7.5220999999999996E-2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AF6" s="1"/>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="1"/>
+      <c r="AI6" s="1"/>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
@@ -1010,25 +962,25 @@
         <v>0</v>
       </c>
       <c r="E7" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>3.2258000000000002E-2</v>
+        <v>3.7590000000000002E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>0.67741899999999999</v>
+        <v>1.709E-3</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>3.2258000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="L7" s="1">
         <v>0</v>
@@ -1055,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="U7" s="1">
         <v>0</v>
@@ -1067,13 +1019,13 @@
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>6.4516000000000004E-2</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="1">
         <v>0</v>
       </c>
       <c r="Z7" s="1">
-        <v>0.16128999999999999</v>
+        <v>0</v>
       </c>
       <c r="AA7" s="1">
         <v>0</v>
@@ -1088,20 +1040,12 @@
         <v>0</v>
       </c>
       <c r="AE7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI7" s="1">
-        <v>3.2258000000000002E-2</v>
-      </c>
+        <v>1.0250000000000001E-3</v>
+      </c>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="1"/>
+      <c r="AI7" s="1"/>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
@@ -1126,13 +1070,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>0</v>
+        <v>2.0500000000000002E-3</v>
       </c>
       <c r="I8" s="1">
         <v>0</v>
       </c>
       <c r="J8" s="1">
-        <v>0.57142899999999996</v>
+        <v>0</v>
       </c>
       <c r="K8" s="1">
         <v>0</v>
@@ -1177,7 +1121,7 @@
         <v>0</v>
       </c>
       <c r="Y8" s="1">
-        <v>0.42857099999999998</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="1">
         <v>0</v>
@@ -1195,20 +1139,12 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI8" s="1">
-        <v>0</v>
-      </c>
+        <v>2.0500000000000002E-3</v>
+      </c>
+      <c r="AF8" s="1"/>
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="1"/>
+      <c r="AI8" s="1"/>
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
@@ -1236,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -1304,43 +1240,35 @@
       <c r="AE9" s="1">
         <v>0</v>
       </c>
-      <c r="AF9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI9" s="1">
-        <v>0</v>
-      </c>
+      <c r="AF9" s="1"/>
+      <c r="AG9" s="1"/>
+      <c r="AH9" s="1"/>
+      <c r="AI9" s="1"/>
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>0</v>
       </c>
       <c r="B10" s="1">
-        <v>1.1364000000000001E-2</v>
+        <v>1.121E-3</v>
       </c>
       <c r="C10" s="1">
-        <v>3.7880000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>7.5760000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="E10" s="1">
-        <v>7.5760000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>4.1667000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="G10" s="1">
-        <v>7.5760000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="H10" s="1">
-        <v>3.7879000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="I10" s="1">
         <v>0</v>
@@ -1352,13 +1280,13 @@
         <v>0</v>
       </c>
       <c r="L10" s="1">
-        <v>0.48106100000000002</v>
+        <v>0</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>7.5760000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="O10" s="1">
         <v>0</v>
@@ -1379,16 +1307,16 @@
         <v>0</v>
       </c>
       <c r="U10" s="1">
-        <v>7.5760000000000003E-3</v>
+        <v>0</v>
       </c>
       <c r="V10" s="1">
         <v>0</v>
       </c>
       <c r="W10" s="1">
-        <v>6.0606E-2</v>
+        <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>1.1364000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="1">
         <v>0</v>
@@ -1409,20 +1337,12 @@
         <v>0</v>
       </c>
       <c r="AE10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI10" s="1">
-        <v>0.31439400000000001</v>
-      </c>
+        <v>6.8300000000000001E-4</v>
+      </c>
+      <c r="AF10" s="1"/>
+      <c r="AG10" s="1"/>
+      <c r="AH10" s="1"/>
+      <c r="AI10" s="1"/>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
@@ -1444,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="1">
-        <v>9.0909000000000004E-2</v>
+        <v>0</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
@@ -1456,13 +1376,13 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>9.0909000000000004E-2</v>
+        <v>0</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
       </c>
       <c r="M11" s="1">
-        <v>0.36363600000000001</v>
+        <v>0</v>
       </c>
       <c r="N11" s="1">
         <v>0</v>
@@ -1518,18 +1438,10 @@
       <c r="AE11" s="1">
         <v>0</v>
       </c>
-      <c r="AF11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI11" s="1">
-        <v>0.45454499999999998</v>
-      </c>
+      <c r="AF11" s="1"/>
+      <c r="AG11" s="1"/>
+      <c r="AH11" s="1"/>
+      <c r="AI11" s="1"/>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
@@ -1548,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -1572,7 +1484,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="O12" s="1">
         <v>0</v>
@@ -1599,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="W12" s="1">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="X12" s="1">
         <v>0</v>
@@ -1625,22 +1537,14 @@
       <c r="AE12" s="1">
         <v>0</v>
       </c>
-      <c r="AF12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="1">
-        <v>0</v>
-      </c>
+      <c r="AF12" s="1"/>
+      <c r="AG12" s="1"/>
+      <c r="AH12" s="1"/>
+      <c r="AI12" s="1"/>
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
-        <v>1.3889E-2</v>
+        <v>0</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
@@ -1649,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
@@ -1661,7 +1565,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="1">
-        <v>1.3889E-2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="1">
         <v>0</v>
@@ -1676,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>0</v>
+        <v>6.6641000000000006E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>0.95833299999999999</v>
+        <v>7.1770000000000002E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1724,7 +1628,7 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="AD13" s="1">
         <v>0</v>
@@ -1732,18 +1636,10 @@
       <c r="AE13" s="1">
         <v>0</v>
       </c>
-      <c r="AF13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="1">
-        <v>1.3889E-2</v>
-      </c>
+      <c r="AF13" s="1"/>
+      <c r="AG13" s="1"/>
+      <c r="AH13" s="1"/>
+      <c r="AI13" s="1"/>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
@@ -1786,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="O14" s="1">
         <v>0</v>
@@ -1837,20 +1733,12 @@
         <v>0</v>
       </c>
       <c r="AE14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI14" s="1">
-        <v>0</v>
-      </c>
+        <v>3.4200000000000002E-4</v>
+      </c>
+      <c r="AF14" s="1"/>
+      <c r="AG14" s="1"/>
+      <c r="AH14" s="1"/>
+      <c r="AI14" s="1"/>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
@@ -1946,34 +1834,26 @@
       <c r="AE15" s="1">
         <v>0</v>
       </c>
-      <c r="AF15" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG15" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH15" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI15" s="1">
-        <v>0</v>
-      </c>
+      <c r="AF15" s="1"/>
+      <c r="AG15" s="1"/>
+      <c r="AH15" s="1"/>
+      <c r="AI15" s="1"/>
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
-        <v>0</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="B16" s="1">
         <v>0</v>
       </c>
       <c r="C16" s="1">
-        <v>0</v>
+        <v>5.0495999999999999E-2</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>0</v>
+        <v>4.7840000000000001E-3</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -2006,25 +1886,25 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0</v>
+        <v>0.77945299999999995</v>
       </c>
       <c r="Q16" s="1">
-        <v>0</v>
+        <v>9.8299999999999993E-4</v>
       </c>
       <c r="R16" s="1">
-        <v>0</v>
+        <v>0.30542900000000001</v>
       </c>
       <c r="S16" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="T16" s="1">
-        <v>0</v>
+        <v>3.447E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
       </c>
       <c r="V16" s="1">
-        <v>0</v>
+        <v>1.034E-3</v>
       </c>
       <c r="W16" s="1">
         <v>0</v>
@@ -2033,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>0</v>
+        <v>6.5490000000000001E-3</v>
       </c>
       <c r="Z16" s="1">
         <v>0</v>
@@ -2051,57 +1931,49 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF16" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG16" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH16" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI16" s="1">
-        <v>0</v>
-      </c>
+        <v>2.9246999999999999E-2</v>
+      </c>
+      <c r="AF16" s="1"/>
+      <c r="AG16" s="1"/>
+      <c r="AH16" s="1"/>
+      <c r="AI16" s="1"/>
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>1.175E-3</v>
+        <v>1.5302E-2</v>
       </c>
       <c r="B17" s="1">
-        <v>3.5249999999999999E-3</v>
+        <v>1.2819000000000001E-2</v>
       </c>
       <c r="C17" s="1">
-        <v>1.175E-3</v>
+        <v>9.7040000000000008E-3</v>
       </c>
       <c r="D17" s="1">
-        <v>1.175E-3</v>
+        <v>3.6908999999999997E-2</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="F17" s="1">
-        <v>1.4101000000000001E-2</v>
+        <v>1.0593999999999999E-2</v>
       </c>
       <c r="G17" s="1">
         <v>0</v>
       </c>
       <c r="H17" s="1">
-        <v>2.3500000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="I17" s="1">
         <v>0</v>
       </c>
       <c r="J17" s="1">
-        <v>0</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="K17" s="1">
         <v>0</v>
       </c>
       <c r="L17" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="M17" s="1">
         <v>0</v>
@@ -2113,72 +1985,64 @@
         <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>0</v>
+        <v>4.7359999999999998E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>0</v>
+        <v>4.182321</v>
       </c>
       <c r="R17" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="S17" s="1">
-        <v>6.6979999999999998E-2</v>
+        <v>0.50117199999999995</v>
       </c>
       <c r="T17" s="1">
-        <v>0</v>
+        <v>2.137E-2</v>
       </c>
       <c r="U17" s="1">
-        <v>0.90011799999999997</v>
+        <v>5.8599999999999998E-3</v>
       </c>
       <c r="V17" s="1">
-        <v>0</v>
+        <v>5.8599999999999998E-3</v>
       </c>
       <c r="W17" s="1">
-        <v>7.051E-3</v>
+        <v>1.034E-3</v>
       </c>
       <c r="X17" s="1">
-        <v>1.175E-3</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="1">
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>0</v>
+        <v>2.2405000000000001E-2</v>
       </c>
       <c r="AA17" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AB17" s="1">
-        <v>0</v>
+        <v>3.7919999999999998E-3</v>
       </c>
       <c r="AC17" s="1">
         <v>0</v>
       </c>
       <c r="AD17" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="AE17" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF17" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG17" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH17" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI17" s="1">
-        <v>1.175E-3</v>
-      </c>
+        <v>2.239E-2</v>
+      </c>
+      <c r="AF17" s="1"/>
+      <c r="AG17" s="1"/>
+      <c r="AH17" s="1"/>
+      <c r="AI17" s="1"/>
     </row>
     <row r="18" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A18" s="1">
         <v>0</v>
       </c>
       <c r="B18" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="C18" s="1">
         <v>0</v>
@@ -2187,7 +2051,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>0</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2226,7 +2090,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="1">
-        <v>0</v>
+        <v>6.8551000000000001E-2</v>
       </c>
       <c r="S18" s="1">
         <v>0</v>
@@ -2235,10 +2099,10 @@
         <v>0</v>
       </c>
       <c r="U18" s="1">
-        <v>1.0989000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="V18" s="1">
-        <v>0.79120900000000005</v>
+        <v>0</v>
       </c>
       <c r="W18" s="1">
         <v>0</v>
@@ -2247,10 +2111,10 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>0</v>
+        <v>5.5149999999999999E-3</v>
       </c>
       <c r="Z18" s="1">
-        <v>1.0989000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="1">
         <v>0</v>
@@ -2259,51 +2123,43 @@
         <v>0</v>
       </c>
       <c r="AC18" s="1">
-        <v>1.0989000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="AD18" s="1">
         <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF18" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG18" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH18" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI18" s="1">
-        <v>0.17582400000000001</v>
-      </c>
+        <v>2.4099999999999998E-3</v>
+      </c>
+      <c r="AF18" s="1"/>
+      <c r="AG18" s="1"/>
+      <c r="AH18" s="1"/>
+      <c r="AI18" s="1"/>
     </row>
     <row r="19" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>0</v>
       </c>
       <c r="B19" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="C19" s="1">
-        <v>1.1310000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="D19" s="1">
-        <v>3.3939999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="E19" s="1">
         <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>2.6017999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="G19" s="1">
-        <v>5.6559999999999996E-3</v>
+        <v>0</v>
       </c>
       <c r="H19" s="1">
-        <v>5.6559999999999996E-3</v>
+        <v>0</v>
       </c>
       <c r="I19" s="1">
         <v>0</v>
@@ -2315,7 +2171,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>3.3939999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="M19" s="1">
         <v>0</v>
@@ -2336,25 +2192,25 @@
         <v>0</v>
       </c>
       <c r="S19" s="1">
-        <v>7.9190000000000007E-3</v>
+        <v>1.5855999999999999E-2</v>
       </c>
       <c r="T19" s="1">
         <v>0</v>
       </c>
       <c r="U19" s="1">
-        <v>4.5250000000000004E-3</v>
+        <v>0</v>
       </c>
       <c r="V19" s="1">
         <v>0</v>
       </c>
       <c r="W19" s="1">
-        <v>0.88009000000000004</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="X19" s="1">
-        <v>1.0181000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="Y19" s="1">
-        <v>9.0500000000000008E-3</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="1">
         <v>0</v>
@@ -2369,23 +2225,15 @@
         <v>0</v>
       </c>
       <c r="AD19" s="1">
-        <v>6.7869999999999996E-3</v>
+        <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF19" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG19" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH19" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI19" s="1">
-        <v>3.6199000000000002E-2</v>
-      </c>
+        <v>6.8599999999999998E-4</v>
+      </c>
+      <c r="AF19" s="1"/>
+      <c r="AG19" s="1"/>
+      <c r="AH19" s="1"/>
+      <c r="AI19" s="1"/>
     </row>
     <row r="20" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
@@ -2395,25 +2243,25 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>3.5839999999999999E-3</v>
+        <v>1.804E-3</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="F20" s="1">
-        <v>7.1679999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>1.0753E-2</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
       </c>
       <c r="I20" s="1">
-        <v>3.5839999999999999E-3</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="J20" s="1">
         <v>0</v>
@@ -2440,34 +2288,34 @@
         <v>0</v>
       </c>
       <c r="R20" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="S20" s="1">
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>0</v>
+        <v>6.4455999999999999E-2</v>
       </c>
       <c r="U20" s="1">
-        <v>3.5839999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>0</v>
+        <v>2.4128E-2</v>
       </c>
       <c r="W20" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="X20" s="1">
-        <v>0.88530500000000001</v>
+        <v>0</v>
       </c>
       <c r="Y20" s="1">
         <v>0</v>
       </c>
       <c r="Z20" s="1">
-        <v>7.1679999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AB20" s="1">
         <v>0</v>
@@ -2476,23 +2324,15 @@
         <v>0</v>
       </c>
       <c r="AD20" s="1">
-        <v>3.5839999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF20" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG20" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH20" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI20" s="1">
-        <v>7.5269000000000003E-2</v>
-      </c>
+        <v>1.7229999999999999E-3</v>
+      </c>
+      <c r="AF20" s="1"/>
+      <c r="AG20" s="1"/>
+      <c r="AH20" s="1"/>
+      <c r="AI20" s="1"/>
     </row>
     <row r="21" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A21" s="1">
@@ -2505,22 +2345,22 @@
         <v>0</v>
       </c>
       <c r="D21" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>2.7397000000000001E-2</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G21" s="1">
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>3.4247E-2</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="I21" s="1">
-        <v>6.8490000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="J21" s="1">
         <v>0</v>
@@ -2529,7 +2369,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="M21" s="1">
         <v>0</v>
@@ -2553,28 +2393,28 @@
         <v>0</v>
       </c>
       <c r="T21" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="U21" s="1">
-        <v>1.3698999999999999E-2</v>
+        <v>1.4821000000000001E-2</v>
       </c>
       <c r="V21" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="W21" s="1">
-        <v>1.3698999999999999E-2</v>
+        <v>9.9959999999999997E-3</v>
       </c>
       <c r="X21" s="1">
-        <v>6.8490000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="Y21" s="1">
-        <v>0.87671200000000005</v>
+        <v>0</v>
       </c>
       <c r="Z21" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AA21" s="1">
-        <v>1.3698999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="AB21" s="1">
         <v>0</v>
@@ -2586,20 +2426,12 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF21" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG21" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH21" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI21" s="1">
-        <v>6.8490000000000001E-3</v>
-      </c>
+        <v>3.0959999999999998E-3</v>
+      </c>
+      <c r="AF21" s="1"/>
+      <c r="AG21" s="1"/>
+      <c r="AH21" s="1"/>
+      <c r="AI21" s="1"/>
     </row>
     <row r="22" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A22" s="1">
@@ -2621,19 +2453,19 @@
         <v>0</v>
       </c>
       <c r="G22" s="1">
-        <v>0.115385</v>
+        <v>0</v>
       </c>
       <c r="H22" s="1">
         <v>0</v>
       </c>
       <c r="I22" s="1">
-        <v>3.8462000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="J22" s="1">
         <v>0</v>
       </c>
       <c r="K22" s="1">
-        <v>7.6923000000000005E-2</v>
+        <v>0</v>
       </c>
       <c r="L22" s="1">
         <v>0</v>
@@ -2672,19 +2504,19 @@
         <v>0</v>
       </c>
       <c r="X22" s="1">
-        <v>3.8462000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="Y22" s="1">
         <v>0</v>
       </c>
       <c r="Z22" s="1">
-        <v>0.57692299999999996</v>
+        <v>0</v>
       </c>
       <c r="AA22" s="1">
         <v>0</v>
       </c>
       <c r="AB22" s="1">
-        <v>3.8462000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="AC22" s="1">
         <v>0</v>
@@ -2693,20 +2525,12 @@
         <v>0</v>
       </c>
       <c r="AE22" s="1">
-        <v>3.8462000000000003E-2</v>
-      </c>
-      <c r="AF22" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG22" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH22" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI22" s="1">
-        <v>7.6923000000000005E-2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AF22" s="1"/>
+      <c r="AG22" s="1"/>
+      <c r="AH22" s="1"/>
+      <c r="AI22" s="1"/>
     </row>
     <row r="23" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A23" s="1">
@@ -2788,7 +2612,7 @@
         <v>0</v>
       </c>
       <c r="AA23" s="1">
-        <v>0.66666700000000001</v>
+        <v>0</v>
       </c>
       <c r="AB23" s="1">
         <v>0</v>
@@ -2802,18 +2626,10 @@
       <c r="AE23" s="1">
         <v>0</v>
       </c>
-      <c r="AF23" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG23" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH23" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI23" s="1">
-        <v>0.33333299999999999</v>
-      </c>
+      <c r="AF23" s="1"/>
+      <c r="AG23" s="1"/>
+      <c r="AH23" s="1"/>
+      <c r="AI23" s="1"/>
     </row>
     <row r="24" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A24" s="1">
@@ -2841,7 +2657,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="J24" s="1">
         <v>0</v>
@@ -2907,20 +2723,12 @@
         <v>0</v>
       </c>
       <c r="AE24" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF24" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG24" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH24" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI24" s="1">
-        <v>0</v>
-      </c>
+        <v>6.8900000000000005E-4</v>
+      </c>
+      <c r="AF24" s="1"/>
+      <c r="AG24" s="1"/>
+      <c r="AH24" s="1"/>
+      <c r="AI24" s="1"/>
     </row>
     <row r="25" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A25" s="1">
@@ -2936,13 +2744,13 @@
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
       </c>
       <c r="G25" s="1">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="H25" s="1">
         <v>0</v>
@@ -2990,7 +2798,7 @@
         <v>0</v>
       </c>
       <c r="W25" s="1">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="X25" s="1">
         <v>0</v>
@@ -3008,7 +2816,7 @@
         <v>0</v>
       </c>
       <c r="AC25" s="1">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AD25" s="1">
         <v>0</v>
@@ -3016,18 +2824,10 @@
       <c r="AE25" s="1">
         <v>0</v>
       </c>
-      <c r="AF25" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG25" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH25" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI25" s="1">
-        <v>0.44</v>
-      </c>
+      <c r="AF25" s="1"/>
+      <c r="AG25" s="1"/>
+      <c r="AH25" s="1"/>
+      <c r="AI25" s="1"/>
     </row>
     <row r="26" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
@@ -3046,13 +2846,13 @@
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>0.117647</v>
+        <v>0</v>
       </c>
       <c r="G26" s="1">
-        <v>5.8824000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="H26" s="1">
-        <v>0.17647099999999999</v>
+        <v>0</v>
       </c>
       <c r="I26" s="1">
         <v>0</v>
@@ -3109,7 +2909,7 @@
         <v>0</v>
       </c>
       <c r="AA26" s="1">
-        <v>5.8824000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="AB26" s="1">
         <v>0</v>
@@ -3118,23 +2918,15 @@
         <v>0</v>
       </c>
       <c r="AD26" s="1">
-        <v>0.352941</v>
+        <v>0</v>
       </c>
       <c r="AE26" s="1">
         <v>0</v>
       </c>
-      <c r="AF26" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG26" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH26" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI26" s="1">
-        <v>0.235294</v>
-      </c>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="1"/>
+      <c r="AH26" s="1"/>
+      <c r="AI26" s="1"/>
     </row>
     <row r="27" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
@@ -3230,18 +3022,10 @@
       <c r="AE27" s="1">
         <v>0</v>
       </c>
-      <c r="AF27" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG27" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH27" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI27" s="1">
-        <v>0</v>
-      </c>
+      <c r="AF27" s="1"/>
+      <c r="AG27" s="1"/>
+      <c r="AH27" s="1"/>
+      <c r="AI27" s="1"/>
     </row>
     <row r="28" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
@@ -3263,7 +3047,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="1">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H28" s="1">
         <v>0</v>
@@ -3326,29 +3110,21 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>0</v>
+        <v>7.2379999999999996E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
       </c>
       <c r="AD28" s="1">
-        <v>0</v>
+        <v>1.034E-3</v>
       </c>
       <c r="AE28" s="1">
         <v>0</v>
       </c>
-      <c r="AF28" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="AG28" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH28" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI28" s="1">
-        <v>0</v>
-      </c>
+      <c r="AF28" s="1"/>
+      <c r="AG28" s="1"/>
+      <c r="AH28" s="1"/>
+      <c r="AI28" s="1"/>
     </row>
     <row r="29" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
@@ -3436,26 +3212,18 @@
         <v>0</v>
       </c>
       <c r="AC29" s="1">
-        <v>0</v>
+        <v>2.068E-3</v>
       </c>
       <c r="AD29" s="1">
         <v>0</v>
       </c>
       <c r="AE29" s="1">
-        <v>0</v>
-      </c>
-      <c r="AF29" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG29" s="1">
-        <v>1</v>
-      </c>
-      <c r="AH29" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI29" s="1">
-        <v>0</v>
-      </c>
+        <v>6.8900000000000005E-4</v>
+      </c>
+      <c r="AF29" s="1"/>
+      <c r="AG29" s="1"/>
+      <c r="AH29" s="1"/>
+      <c r="AI29" s="1"/>
     </row>
     <row r="30" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
@@ -3551,18 +3319,10 @@
       <c r="AE30" s="1">
         <v>0</v>
       </c>
-      <c r="AF30" s="1">
-        <v>0</v>
-      </c>
-      <c r="AG30" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH30" s="1">
-        <v>0</v>
-      </c>
-      <c r="AI30" s="1">
-        <v>0</v>
-      </c>
+      <c r="AF30" s="1"/>
+      <c r="AG30" s="1"/>
+      <c r="AH30" s="1"/>
+      <c r="AI30" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>

<commit_message>
fix off-res and side band code
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25629"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9EF789-434D-4562-9E66-A3B59A1BC67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778C6265-66E0-48E5-A749-763387DEA370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,97 +356,97 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>8.3962900000000005</v>
+        <v>6.4349350000000003</v>
       </c>
       <c r="B1" s="1">
-        <v>4.8468939999999998</v>
+        <v>2.9306589999999999</v>
       </c>
       <c r="C1" s="1">
-        <v>0.280362</v>
+        <v>0.16438900000000001</v>
       </c>
       <c r="D1" s="1">
-        <v>5.6388000000000001E-2</v>
+        <v>3.6567000000000002E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>2.7681999999999998E-2</v>
+        <v>1.7087000000000001E-2</v>
       </c>
       <c r="F1" s="1">
-        <v>2.9389999999999999E-2</v>
+        <v>1.7429E-2</v>
       </c>
       <c r="G1" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="H1" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="I1" s="1">
         <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>0.158913</v>
+        <v>8.4070000000000006E-2</v>
       </c>
       <c r="K1" s="1">
         <v>1.0250000000000001E-3</v>
       </c>
       <c r="L1" s="1">
-        <v>3.4169999999999999E-3</v>
+        <v>1.709E-3</v>
       </c>
       <c r="M1" s="1">
-        <v>5.8100000000000001E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="N1" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="O1" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="P1" s="1">
         <v>1.1839999999999999E-3</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.55838900000000002</v>
+        <v>0.47580899999999998</v>
       </c>
       <c r="R1" s="1">
+        <v>2.9989999999999999E-3</v>
+      </c>
+      <c r="S1" s="1">
+        <v>4.0673000000000001E-2</v>
+      </c>
+      <c r="T1" s="1">
+        <v>2.068E-3</v>
+      </c>
+      <c r="U1" s="1">
+        <v>0</v>
+      </c>
+      <c r="V1" s="1">
+        <v>1.7229999999999999E-3</v>
+      </c>
+      <c r="W1" s="1">
+        <v>3.4499999999999998E-4</v>
+      </c>
+      <c r="X1" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>2.7569999999999999E-3</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB1" s="1">
         <v>1.379E-3</v>
       </c>
-      <c r="S1" s="1">
-        <v>7.1349999999999997E-2</v>
-      </c>
-      <c r="T1" s="1">
-        <v>2.4130000000000002E-3</v>
-      </c>
-      <c r="U1" s="1">
-        <v>1.379E-3</v>
-      </c>
-      <c r="V1" s="1">
-        <v>1.379E-3</v>
-      </c>
-      <c r="W1" s="1">
-        <v>1.034E-3</v>
-      </c>
-      <c r="X1" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y1" s="1">
-        <v>3.4499999999999998E-4</v>
-      </c>
-      <c r="Z1" s="1">
-        <v>3.1020000000000002E-3</v>
-      </c>
-      <c r="AA1" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB1" s="1">
-        <v>1.7229999999999999E-3</v>
-      </c>
       <c r="AC1" s="1">
         <v>0</v>
       </c>
       <c r="AD1" s="1">
-        <v>6.8900000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.463173</v>
+        <v>0.34468500000000002</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -455,89 +455,89 @@
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>2.2499999999999998E-3</v>
+        <v>0.31639099999999998</v>
       </c>
       <c r="B2" s="1">
-        <v>0.72534399999999999</v>
+        <v>3.534208</v>
       </c>
       <c r="C2" s="1">
-        <v>2.9250000000000001E-3</v>
+        <v>4.6864999999999997E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>1.4695E-2</v>
       </c>
       <c r="E2" s="1">
-        <v>5.1260000000000003E-3</v>
+        <v>2.3238999999999999E-2</v>
       </c>
       <c r="F2" s="1">
-        <v>3.7590000000000002E-3</v>
+        <v>1.3328E-2</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
       </c>
       <c r="H2" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="I2" s="1">
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>5.5021E-2</v>
+        <v>0.256994</v>
       </c>
       <c r="K2" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>2.392E-3</v>
       </c>
       <c r="L2" s="1">
-        <v>6.8300000000000001E-4</v>
+        <v>3.0760000000000002E-3</v>
       </c>
       <c r="M2" s="1">
         <v>3.4200000000000002E-4</v>
       </c>
       <c r="N2" s="1">
-        <v>6.8300000000000001E-4</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="O2" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="P2" s="1">
-        <v>3.9500000000000001E-4</v>
+        <v>1.5790000000000001E-3</v>
       </c>
       <c r="Q2" s="1">
-        <v>5.2579999999999997E-3</v>
+        <v>9.3701999999999994E-2</v>
       </c>
       <c r="R2" s="1">
-        <v>2.0170000000000001E-3</v>
+        <v>4.6709999999999998E-3</v>
       </c>
       <c r="S2" s="1">
-        <v>1.3098E-2</v>
+        <v>8.8238999999999998E-2</v>
       </c>
       <c r="T2" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="U2" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="V2" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="W2" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="X2" s="1">
         <v>0</v>
       </c>
       <c r="Y2" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="Z2" s="1">
+        <v>8.6169999999999997E-3</v>
+      </c>
+      <c r="AA2" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="1">
         <v>1.034E-3</v>
       </c>
-      <c r="AA2" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="1">
-        <v>3.4499999999999998E-4</v>
-      </c>
       <c r="AC2" s="1">
         <v>0</v>
       </c>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>4.5803000000000003E-2</v>
+        <v>0.30156699999999997</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -554,37 +554,37 @@
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
-        <v>4.4999999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="B3" s="1">
-        <v>0</v>
+        <v>1.121E-3</v>
       </c>
       <c r="C3" s="1">
-        <v>1.9504809999999999</v>
+        <v>1.731965</v>
       </c>
       <c r="D3" s="1">
         <v>1.0250000000000001E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>0.22452800000000001</v>
+        <v>0.178392</v>
       </c>
       <c r="F3" s="1">
+        <v>1.709E-3</v>
+      </c>
+      <c r="G3" s="1">
+        <v>3.0760000000000002E-3</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
         <v>3.4200000000000002E-4</v>
       </c>
-      <c r="G3" s="1">
-        <v>2.392E-3</v>
-      </c>
-      <c r="H3" s="1">
-        <v>0</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1.3669999999999999E-3</v>
-      </c>
       <c r="J3" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="K3" s="1">
-        <v>7.1770000000000002E-3</v>
+        <v>1.0593999999999999E-2</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -599,28 +599,28 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>5.9199999999999999E-3</v>
+        <v>6.3150000000000003E-3</v>
       </c>
       <c r="Q3" s="1">
-        <v>3.0509999999999999E-3</v>
+        <v>4.3270000000000001E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>7.326E-3</v>
+        <v>8.0669999999999995E-3</v>
       </c>
       <c r="S3" s="1">
         <v>6.8900000000000005E-4</v>
       </c>
       <c r="T3" s="1">
-        <v>1.6889999999999999E-2</v>
+        <v>1.8957999999999999E-2</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
       </c>
       <c r="V3" s="1">
-        <v>6.894E-3</v>
+        <v>5.5149999999999999E-3</v>
       </c>
       <c r="W3" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="X3" s="1">
         <v>0</v>
@@ -632,10 +632,10 @@
         <v>0</v>
       </c>
       <c r="AA3" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="AB3" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC3" s="1">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>1.5747000000000001E-2</v>
+        <v>1.6424000000000001E-2</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -653,40 +653,40 @@
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
-        <v>4.4999999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>2.9250000000000001E-3</v>
+        <v>6.0959999999999999E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>1.2437999999999999E-2</v>
+        <v>7.463E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>0.83557300000000001</v>
+        <v>0.77884299999999995</v>
       </c>
       <c r="E4" s="1">
-        <v>2.7339999999999999E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="F4" s="1">
-        <v>0.30073800000000001</v>
+        <v>0.26758900000000002</v>
       </c>
       <c r="G4" s="1">
-        <v>2.7339999999999999E-3</v>
+        <v>2.0500000000000002E-3</v>
       </c>
       <c r="H4" s="1">
-        <v>1.3669999999999999E-3</v>
+        <v>2.0500000000000002E-3</v>
       </c>
       <c r="I4" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>1.709E-3</v>
       </c>
       <c r="J4" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="K4" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>2.0847000000000001E-2</v>
+        <v>2.5631000000000001E-2</v>
       </c>
       <c r="M4" s="1">
         <v>3.4200000000000002E-4</v>
@@ -701,40 +701,40 @@
         <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <v>3.7852999999999998E-2</v>
+        <v>3.4165000000000001E-2</v>
       </c>
       <c r="R4" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>9.306E-3</v>
+        <v>1.2753E-2</v>
       </c>
       <c r="T4" s="1">
-        <v>1.034E-3</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="U4" s="1">
-        <v>1.103E-2</v>
+        <v>1.2753E-2</v>
       </c>
       <c r="V4" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>1.379E-3</v>
       </c>
       <c r="W4" s="1">
-        <v>5.8599999999999998E-3</v>
+        <v>6.2040000000000003E-3</v>
       </c>
       <c r="X4" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="Y4" s="1">
         <v>0</v>
       </c>
       <c r="Z4" s="1">
-        <v>6.8900000000000005E-4</v>
+        <v>1.379E-3</v>
       </c>
       <c r="AA4" s="1">
         <v>0</v>
       </c>
       <c r="AB4" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="1">
         <v>0</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>4.8892999999999999E-2</v>
+        <v>4.4454E-2</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -752,25 +752,25 @@
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
-        <v>0</v>
+        <v>4.4999999999999999E-4</v>
       </c>
       <c r="B5" s="1">
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>0</v>
+        <v>8.4526000000000004E-2</v>
       </c>
       <c r="D5" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="E5" s="1">
-        <v>4.1009999999999996E-3</v>
+        <v>0.16096299999999999</v>
       </c>
       <c r="F5" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G5" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
@@ -782,7 +782,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="1">
-        <v>1.709E-3</v>
+        <v>1.4695E-2</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -791,31 +791,31 @@
         <v>0</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="O5" s="1">
         <v>0</v>
       </c>
       <c r="P5" s="1">
-        <v>0</v>
+        <v>3.9500000000000001E-4</v>
       </c>
       <c r="Q5" s="1">
         <v>0</v>
       </c>
       <c r="R5" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>3.637E-3</v>
       </c>
       <c r="S5" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="T5" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="U5" s="1">
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>5.5149999999999999E-3</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
@@ -824,13 +824,13 @@
         <v>0</v>
       </c>
       <c r="Y5" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="Z5" s="1">
         <v>0</v>
       </c>
       <c r="AA5" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>1.2664999999999999E-2</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -854,37 +854,37 @@
         <v>0</v>
       </c>
       <c r="B6" s="1">
-        <v>0</v>
+        <v>1.804E-3</v>
       </c>
       <c r="C6" s="1">
-        <v>0</v>
+        <v>1.121E-3</v>
       </c>
       <c r="D6" s="1">
+        <v>2.2554999999999999E-2</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2.392E-3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.12508</v>
+      </c>
+      <c r="G6" s="1">
         <v>3.4200000000000002E-4</v>
       </c>
-      <c r="E6" s="1">
-        <v>0</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1.709E-3</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0</v>
-      </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="J6" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="K6" s="1">
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>0</v>
+        <v>2.2897000000000001E-2</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -899,34 +899,34 @@
         <v>0</v>
       </c>
       <c r="Q6" s="1">
-        <v>0</v>
+        <v>1.9650000000000002E-3</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>0</v>
+        <v>3.7919999999999998E-3</v>
       </c>
       <c r="T6" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="U6" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="V6" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="W6" s="1">
-        <v>0</v>
+        <v>4.4809999999999997E-3</v>
       </c>
       <c r="X6" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="Y6" s="1">
         <v>0</v>
       </c>
       <c r="Z6" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="AA6" s="1">
         <v>0</v>
@@ -938,10 +938,10 @@
         <v>0</v>
       </c>
       <c r="AD6" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AE6" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>1.95E-2</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -962,19 +962,19 @@
         <v>0</v>
       </c>
       <c r="E7" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>6.1510000000000002E-3</v>
+        <v>8.5439999999999995E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>3.7590000000000002E-3</v>
+        <v>3.0760000000000002E-3</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
@@ -1007,13 +1007,13 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="U7" s="1">
         <v>0</v>
       </c>
       <c r="V7" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="AE7" s="1">
-        <v>2.0530000000000001E-3</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
@@ -1064,13 +1064,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G8" s="1">
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>3.0760000000000002E-3</v>
+        <v>1.3669999999999999E-3</v>
       </c>
       <c r="I8" s="1">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>3.4169999999999999E-3</v>
+        <v>4.4429999999999999E-3</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="G9" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -1238,7 +1238,7 @@
         <v>0</v>
       </c>
       <c r="AE9" s="1">
-        <v>0</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="AF9" s="1"/>
       <c r="AG9" s="1"/>
@@ -1247,22 +1247,22 @@
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
-        <v>0</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>1.121E-3</v>
+        <v>0.112841</v>
       </c>
       <c r="C10" s="1">
-        <v>0</v>
+        <v>4.2919999999999998E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>2.7339999999999999E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>0</v>
+        <v>7.5180000000000004E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>0</v>
+        <v>3.4169999999999999E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,19 +1274,19 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>0</v>
+        <v>8.3727999999999997E-2</v>
       </c>
       <c r="K10" s="1">
         <v>0</v>
       </c>
       <c r="L10" s="1">
-        <v>0</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="O10" s="1">
         <v>0</v>
@@ -1295,22 +1295,22 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>0</v>
+        <v>3.9820000000000003E-3</v>
       </c>
       <c r="R10" s="1">
-        <v>0</v>
+        <v>1.3270000000000001E-3</v>
       </c>
       <c r="S10" s="1">
-        <v>0</v>
+        <v>9.9959999999999997E-3</v>
       </c>
       <c r="T10" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="U10" s="1">
         <v>0</v>
       </c>
       <c r="V10" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
@@ -1319,16 +1319,16 @@
         <v>0</v>
       </c>
       <c r="Y10" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="Z10" s="1">
-        <v>0</v>
+        <v>2.4130000000000002E-3</v>
       </c>
       <c r="AA10" s="1">
         <v>0</v>
       </c>
       <c r="AB10" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC10" s="1">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>9.8104999999999998E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1352,19 +1352,19 @@
         <v>0</v>
       </c>
       <c r="C11" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>0</v>
+        <v>5.8100000000000001E-3</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
       </c>
       <c r="G11" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>0</v>
+        <v>3.0760000000000002E-3</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -1409,10 +1409,10 @@
         <v>0</v>
       </c>
       <c r="V11" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="W11" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="X11" s="1">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="1">
-        <v>0</v>
+        <v>4.104E-3</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1454,13 +1454,13 @@
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="E12" s="1">
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>0</v>
+        <v>4.1009999999999996E-3</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="1">
-        <v>0</v>
+        <v>3.0760000000000002E-3</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
@@ -1535,7 +1535,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="1">
-        <v>0</v>
+        <v>1.3730000000000001E-3</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>8.5436999999999999E-2</v>
+        <v>6.5615999999999994E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>1.0252000000000001E-2</v>
+        <v>7.5180000000000004E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1601,7 +1601,7 @@
         <v>0</v>
       </c>
       <c r="T13" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="U13" s="1">
         <v>0</v>
@@ -1628,13 +1628,13 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>1.379E-3</v>
+        <v>2.068E-3</v>
       </c>
       <c r="AD13" s="1">
         <v>0</v>
       </c>
       <c r="AE13" s="1">
-        <v>2.0500000000000002E-3</v>
+        <v>2.7339999999999999E-3</v>
       </c>
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
@@ -1682,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="O14" s="1">
         <v>0</v>
@@ -1733,7 +1733,7 @@
         <v>0</v>
       </c>
       <c r="AE14" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="AF14" s="1"/>
       <c r="AG14" s="1"/>
@@ -1778,13 +1778,13 @@
         <v>0</v>
       </c>
       <c r="M15" s="1">
-        <v>0</v>
+        <v>2.392E-3</v>
       </c>
       <c r="N15" s="1">
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>0</v>
+        <v>1.709E-3</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1832,7 +1832,7 @@
         <v>0</v>
       </c>
       <c r="AE15" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1"/>
@@ -1841,35 +1841,35 @@
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
-        <v>8.9999999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="B16" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="C16" s="1">
-        <v>8.6805999999999994E-2</v>
+        <v>0.100443</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>8.8850000000000005E-3</v>
+        <v>5.4679999999999998E-3</v>
       </c>
       <c r="F16" s="1">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1">
+        <v>0</v>
+      </c>
+      <c r="H16" s="1">
+        <v>0</v>
+      </c>
+      <c r="I16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J16" s="1">
         <v>3.4200000000000002E-4</v>
       </c>
-      <c r="G16" s="1">
-        <v>0</v>
-      </c>
-      <c r="H16" s="1">
-        <v>0</v>
-      </c>
-      <c r="I16" s="1">
-        <v>0</v>
-      </c>
-      <c r="J16" s="1">
-        <v>0</v>
-      </c>
       <c r="K16" s="1">
         <v>0</v>
       </c>
@@ -1886,25 +1886,25 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.90179699999999996</v>
+        <v>0.71117699999999995</v>
       </c>
       <c r="Q16" s="1">
-        <v>2.9480000000000001E-3</v>
+        <v>3.2919999999999998E-3</v>
       </c>
       <c r="R16" s="1">
-        <v>0.47845399999999999</v>
+        <v>0.32514799999999999</v>
       </c>
       <c r="S16" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>1.034E-3</v>
       </c>
       <c r="T16" s="1">
-        <v>3.7919999999999998E-3</v>
+        <v>3.447E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
       </c>
       <c r="V16" s="1">
-        <v>2.4130000000000002E-3</v>
+        <v>1.7229999999999999E-3</v>
       </c>
       <c r="W16" s="1">
         <v>0</v>
@@ -1913,13 +1913,13 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>1.4477E-2</v>
+        <v>1.2753E-2</v>
       </c>
       <c r="Z16" s="1">
         <v>0</v>
       </c>
       <c r="AA16" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AB16" s="1">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>5.4696000000000002E-2</v>
+        <v>4.4310000000000002E-2</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1940,31 +1940,31 @@
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>1.7552000000000002E-2</v>
+        <v>1.1251000000000001E-2</v>
       </c>
       <c r="B17" s="1">
-        <v>2.1687999999999999E-2</v>
+        <v>1.2191E-2</v>
       </c>
       <c r="C17" s="1">
-        <v>1.2533000000000001E-2</v>
+        <v>1.1261E-2</v>
       </c>
       <c r="D17" s="1">
-        <v>6.5957000000000002E-2</v>
+        <v>6.2539999999999998E-2</v>
       </c>
       <c r="E17" s="1">
+        <v>1.709E-3</v>
+      </c>
+      <c r="F17" s="1">
+        <v>2.9389999999999999E-2</v>
+      </c>
+      <c r="G17" s="1">
         <v>1.0250000000000001E-3</v>
       </c>
-      <c r="F17" s="1">
-        <v>2.4948000000000001E-2</v>
-      </c>
-      <c r="G17" s="1">
-        <v>3.4200000000000002E-4</v>
-      </c>
       <c r="H17" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="I17" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="J17" s="1">
         <v>1.0250000000000001E-3</v>
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="L17" s="1">
-        <v>1.0250000000000001E-3</v>
+        <v>2.7339999999999999E-3</v>
       </c>
       <c r="M17" s="1">
         <v>3.4200000000000002E-4</v>
@@ -1982,31 +1982,31 @@
         <v>0</v>
       </c>
       <c r="O17" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="P17" s="1">
         <v>5.1310000000000001E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>5.158836</v>
+        <v>4.1856450000000001</v>
       </c>
       <c r="R17" s="1">
-        <v>6.8900000000000005E-4</v>
+        <v>4.3270000000000001E-3</v>
       </c>
       <c r="S17" s="1">
-        <v>0.78588199999999997</v>
+        <v>0.56149199999999999</v>
       </c>
       <c r="T17" s="1">
-        <v>3.3433999999999998E-2</v>
+        <v>1.7923999999999999E-2</v>
       </c>
       <c r="U17" s="1">
-        <v>8.2719999999999998E-3</v>
+        <v>5.1700000000000001E-3</v>
       </c>
       <c r="V17" s="1">
-        <v>9.9959999999999997E-3</v>
+        <v>4.1359999999999999E-3</v>
       </c>
       <c r="W17" s="1">
-        <v>4.4809999999999997E-3</v>
+        <v>2.7569999999999999E-3</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2015,22 +2015,22 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>4.3430000000000003E-2</v>
+        <v>4.0328000000000003E-2</v>
       </c>
       <c r="AA17" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="AB17" s="1">
-        <v>6.2040000000000003E-3</v>
+        <v>2.4130000000000002E-3</v>
       </c>
       <c r="AC17" s="1">
         <v>3.4499999999999998E-4</v>
       </c>
       <c r="AD17" s="1">
-        <v>1.379E-3</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AE17" s="1">
-        <v>5.4767000000000003E-2</v>
+        <v>5.0951999999999997E-2</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2042,31 +2042,31 @@
         <v>0</v>
       </c>
       <c r="B18" s="1">
+        <v>2.5829999999999998E-3</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2.1839000000000001E-2</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1.5037E-2</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0</v>
+      </c>
+      <c r="G18" s="1">
+        <v>0</v>
+      </c>
+      <c r="H18" s="1">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18" s="1">
         <v>3.4200000000000002E-4</v>
-      </c>
-      <c r="C18" s="1">
-        <v>1.121E-3</v>
-      </c>
-      <c r="D18" s="1">
-        <v>0</v>
-      </c>
-      <c r="E18" s="1">
-        <v>1.3669999999999999E-3</v>
-      </c>
-      <c r="F18" s="1">
-        <v>0</v>
-      </c>
-      <c r="G18" s="1">
-        <v>0</v>
-      </c>
-      <c r="H18" s="1">
-        <v>0</v>
-      </c>
-      <c r="I18" s="1">
-        <v>0</v>
-      </c>
-      <c r="J18" s="1">
-        <v>0</v>
       </c>
       <c r="K18" s="1">
         <v>3.4200000000000002E-4</v>
@@ -2084,44 +2084,44 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>0</v>
+        <v>3.2362000000000002E-2</v>
       </c>
       <c r="Q18" s="1">
-        <v>9.8299999999999993E-4</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="R18" s="1">
-        <v>7.9718999999999998E-2</v>
+        <v>0.42209200000000002</v>
       </c>
       <c r="S18" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="T18" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>2.7569999999999999E-3</v>
       </c>
       <c r="U18" s="1">
         <v>0</v>
       </c>
       <c r="V18" s="1">
+        <v>2.7569999999999999E-3</v>
+      </c>
+      <c r="W18" s="1">
+        <v>0</v>
+      </c>
+      <c r="X18" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="1">
+        <v>3.1022000000000001E-2</v>
+      </c>
+      <c r="Z18" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="1">
+        <v>3.4499999999999998E-4</v>
+      </c>
+      <c r="AB18" s="1">
         <v>6.8900000000000005E-4</v>
       </c>
-      <c r="W18" s="1">
-        <v>0</v>
-      </c>
-      <c r="X18" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="1">
-        <v>8.2719999999999998E-3</v>
-      </c>
-      <c r="Z18" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA18" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB18" s="1">
-        <v>0</v>
-      </c>
       <c r="AC18" s="1">
         <v>0</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>7.9249999999999998E-3</v>
+        <v>4.0667000000000002E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2141,70 +2141,70 @@
         <v>0</v>
       </c>
       <c r="B19" s="1">
+        <v>7.9000000000000008E-3</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1.804E-3</v>
+      </c>
+      <c r="D19" s="1">
+        <v>1.1278E-2</v>
+      </c>
+      <c r="E19" s="1">
+        <v>6.8300000000000001E-4</v>
+      </c>
+      <c r="F19" s="1">
+        <v>2.2214000000000001E-2</v>
+      </c>
+      <c r="G19" s="1">
+        <v>1.0250000000000001E-3</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>6.8300000000000001E-4</v>
+      </c>
+      <c r="J19" s="1">
         <v>1.3669999999999999E-3</v>
       </c>
-      <c r="C19" s="1">
-        <v>0</v>
-      </c>
-      <c r="D19" s="1">
-        <v>0</v>
-      </c>
-      <c r="E19" s="1">
+      <c r="K19" s="1">
+        <v>6.8300000000000001E-4</v>
+      </c>
+      <c r="L19" s="1">
+        <v>4.1009999999999996E-3</v>
+      </c>
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="N19" s="1">
         <v>3.4200000000000002E-4</v>
       </c>
-      <c r="F19" s="1">
-        <v>1.3669999999999999E-3</v>
-      </c>
-      <c r="G19" s="1">
-        <v>0</v>
-      </c>
-      <c r="H19" s="1">
-        <v>0</v>
-      </c>
-      <c r="I19" s="1">
-        <v>0</v>
-      </c>
-      <c r="J19" s="1">
-        <v>0</v>
-      </c>
-      <c r="K19" s="1">
-        <v>0</v>
-      </c>
-      <c r="L19" s="1">
-        <v>0</v>
-      </c>
-      <c r="M19" s="1">
-        <v>0</v>
-      </c>
-      <c r="N19" s="1">
-        <v>0</v>
-      </c>
       <c r="O19" s="1">
         <v>0</v>
       </c>
       <c r="P19" s="1">
-        <v>0</v>
+        <v>3.9500000000000001E-4</v>
       </c>
       <c r="Q19" s="1">
-        <v>1.3270000000000001E-3</v>
+        <v>0.179147</v>
       </c>
       <c r="R19" s="1">
-        <v>0</v>
+        <v>4.2750000000000002E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>2.3782999999999999E-2</v>
+        <v>0.45636300000000002</v>
       </c>
       <c r="T19" s="1">
-        <v>0</v>
+        <v>6.5490000000000001E-3</v>
       </c>
       <c r="U19" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="V19" s="1">
-        <v>0</v>
+        <v>4.8260000000000004E-3</v>
       </c>
       <c r="W19" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>3.1020000000000002E-3</v>
       </c>
       <c r="X19" s="1">
         <v>0</v>
@@ -2213,22 +2213,22 @@
         <v>0</v>
       </c>
       <c r="Z19" s="1">
-        <v>1.7229999999999999E-3</v>
+        <v>5.2736999999999999E-2</v>
       </c>
       <c r="AA19" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="AB19" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>1.034E-3</v>
       </c>
       <c r="AC19" s="1">
         <v>0</v>
       </c>
       <c r="AD19" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AE19" s="1">
-        <v>1.3760000000000001E-3</v>
+        <v>4.8558999999999998E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2243,25 +2243,25 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>3.2659999999999998E-3</v>
+        <v>2.9250000000000001E-3</v>
       </c>
       <c r="D20" s="1">
         <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>1.3669999999999999E-3</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>3.0760000000000002E-3</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
       </c>
       <c r="I20" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>1.709E-3</v>
       </c>
       <c r="J20" s="1">
         <v>0</v>
@@ -2285,28 +2285,28 @@
         <v>0</v>
       </c>
       <c r="Q20" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="R20" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="S20" s="1">
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>9.1686000000000004E-2</v>
+        <v>8.3757999999999999E-2</v>
       </c>
       <c r="U20" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="V20" s="1">
-        <v>4.2741000000000001E-2</v>
+        <v>2.8608999999999999E-2</v>
       </c>
       <c r="W20" s="1">
         <v>3.4499999999999998E-4</v>
       </c>
       <c r="X20" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="Y20" s="1">
         <v>0</v>
@@ -2315,19 +2315,19 @@
         <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>2.7569999999999999E-3</v>
+        <v>1.7229999999999999E-3</v>
       </c>
       <c r="AB20" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC20" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="AD20" s="1">
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>2.7569999999999999E-3</v>
+        <v>4.8260000000000004E-3</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2345,19 +2345,19 @@
         <v>0</v>
       </c>
       <c r="D21" s="1">
-        <v>6.8300000000000001E-4</v>
+        <v>1.3669999999999999E-3</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="G21" s="1">
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>1.3669999999999999E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="I21" s="1">
         <v>0</v>
@@ -2369,7 +2369,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>0</v>
       </c>
       <c r="M21" s="1">
         <v>0</v>
@@ -2384,13 +2384,13 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <v>0</v>
+        <v>9.8299999999999993E-4</v>
       </c>
       <c r="R21" s="1">
         <v>0</v>
       </c>
       <c r="S21" s="1">
-        <v>6.8900000000000005E-4</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="T21" s="1">
         <v>6.8900000000000005E-4</v>
@@ -2402,7 +2402,7 @@
         <v>3.4499999999999998E-4</v>
       </c>
       <c r="W21" s="1">
-        <v>1.9991999999999999E-2</v>
+        <v>1.4477E-2</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2411,7 +2411,7 @@
         <v>0</v>
       </c>
       <c r="Z21" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="AA21" s="1">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>5.5059999999999996E-3</v>
+        <v>8.9470000000000001E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2447,10 +2447,10 @@
         <v>0</v>
       </c>
       <c r="E22" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="F22" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G22" s="1">
         <v>0</v>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>0</v>
+        <v>1.4132E-2</v>
       </c>
       <c r="W22" s="1">
         <v>0</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="1">
-        <v>0</v>
+        <v>3.1020000000000002E-3</v>
       </c>
       <c r="AB22" s="1">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="1">
-        <v>0</v>
+        <v>1.3730000000000001E-3</v>
       </c>
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
@@ -2549,7 +2549,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="G23" s="1">
         <v>0</v>
@@ -2594,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="U23" s="1">
-        <v>0</v>
+        <v>1.034E-3</v>
       </c>
       <c r="V23" s="1">
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>0</v>
+        <v>3.447E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>0</v>
+        <v>1.3760000000000001E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2702,7 +2702,7 @@
         <v>0</v>
       </c>
       <c r="X24" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="Y24" s="1">
         <v>0</v>
@@ -2723,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="AE24" s="1">
-        <v>6.8900000000000005E-4</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AF24" s="1"/>
       <c r="AG24" s="1"/>
@@ -2735,16 +2735,16 @@
         <v>0</v>
       </c>
       <c r="B25" s="1">
-        <v>0</v>
+        <v>1.121E-3</v>
       </c>
       <c r="C25" s="1">
-        <v>0</v>
+        <v>1.462E-3</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>0</v>
+        <v>1.709E-3</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="L25" s="1">
         <v>0</v>
@@ -2777,13 +2777,13 @@
         <v>0</v>
       </c>
       <c r="P25" s="1">
-        <v>0</v>
+        <v>1.1839999999999999E-3</v>
       </c>
       <c r="Q25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>0</v>
+        <v>1.0911000000000001E-2</v>
       </c>
       <c r="S25" s="1">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="1">
-        <v>0</v>
+        <v>1.0340999999999999E-2</v>
       </c>
       <c r="Z25" s="1">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>0</v>
       </c>
       <c r="AB25" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC25" s="1">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>1.3779E-2</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2837,16 +2837,16 @@
         <v>0</v>
       </c>
       <c r="C26" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="D26" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="E26" s="1">
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>0</v>
+        <v>2.7339999999999999E-3</v>
       </c>
       <c r="G26" s="1">
         <v>0</v>
@@ -2858,13 +2858,13 @@
         <v>0</v>
       </c>
       <c r="J26" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="K26" s="1">
         <v>0</v>
       </c>
       <c r="L26" s="1">
-        <v>0</v>
+        <v>1.709E-3</v>
       </c>
       <c r="M26" s="1">
         <v>0</v>
@@ -2879,25 +2879,25 @@
         <v>0</v>
       </c>
       <c r="Q26" s="1">
-        <v>0</v>
+        <v>1.9650000000000002E-3</v>
       </c>
       <c r="R26" s="1">
         <v>0</v>
       </c>
       <c r="S26" s="1">
-        <v>0</v>
+        <v>9.306E-3</v>
       </c>
       <c r="T26" s="1">
-        <v>0</v>
+        <v>1.379E-3</v>
       </c>
       <c r="U26" s="1">
         <v>0</v>
       </c>
       <c r="V26" s="1">
-        <v>0</v>
+        <v>6.8900000000000005E-4</v>
       </c>
       <c r="W26" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="X26" s="1">
         <v>0</v>
@@ -2906,7 +2906,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="1">
-        <v>0</v>
+        <v>9.6509999999999999E-3</v>
       </c>
       <c r="AA26" s="1">
         <v>0</v>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>0</v>
+        <v>1.0673E-2</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -3020,7 +3020,7 @@
         <v>0</v>
       </c>
       <c r="AE27" s="1">
-        <v>0</v>
+        <v>1.0280000000000001E-3</v>
       </c>
       <c r="AF27" s="1"/>
       <c r="AG27" s="1"/>
@@ -3065,10 +3065,10 @@
         <v>0</v>
       </c>
       <c r="M28" s="1">
-        <v>0</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="N28" s="1">
-        <v>6.8300000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="O28" s="1">
         <v>0</v>
@@ -3110,16 +3110,16 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>8.9619999999999995E-3</v>
+        <v>5.8599999999999998E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
       </c>
       <c r="AD28" s="1">
-        <v>1.034E-3</v>
+        <v>2.4130000000000002E-3</v>
       </c>
       <c r="AE28" s="1">
-        <v>3.4200000000000002E-4</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AF28" s="1"/>
       <c r="AG28" s="1"/>
@@ -3212,13 +3212,13 @@
         <v>0</v>
       </c>
       <c r="AC29" s="1">
-        <v>2.7569999999999999E-3</v>
+        <v>1.034E-3</v>
       </c>
       <c r="AD29" s="1">
-        <v>3.4499999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="AE29" s="1">
-        <v>1.379E-3</v>
+        <v>1.034E-3</v>
       </c>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AB30" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AC30" s="1">
         <v>0</v>
       </c>
       <c r="AD30" s="1">
-        <v>0</v>
+        <v>3.4499999999999998E-4</v>
       </c>
       <c r="AE30" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
leptonID branch & fake lepton leaf
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2CCBE2-4293-4D73-A21F-FC76A20B681E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8649B3-1937-4C33-A27F-C4ADE1CFA2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,13 +356,13 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>9.0082249999999995</v>
+        <v>9.7890940000000004</v>
       </c>
       <c r="B1" s="1">
-        <v>1.9544919999999999</v>
+        <v>1.991169</v>
       </c>
       <c r="C1" s="1">
-        <v>0.115271</v>
+        <v>0.113939</v>
       </c>
       <c r="D1" s="1">
         <v>1.9633000000000001E-2</v>
@@ -371,7 +371,7 @@
         <v>4.5310000000000003E-3</v>
       </c>
       <c r="F1" s="1">
-        <v>7.5510000000000004E-3</v>
+        <v>7.1739999999999998E-3</v>
       </c>
       <c r="G1" s="1">
         <v>0</v>
@@ -380,10 +380,10 @@
         <v>0</v>
       </c>
       <c r="I1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>3.4736000000000003E-2</v>
+        <v>3.1337999999999998E-2</v>
       </c>
       <c r="K1" s="1">
         <v>3.7800000000000003E-4</v>
@@ -392,7 +392,7 @@
         <v>0</v>
       </c>
       <c r="M1" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="N1" s="1">
         <v>0</v>
@@ -401,16 +401,16 @@
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>0</v>
+        <v>1.2279999999999999E-3</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.29588900000000001</v>
+        <v>0.28952800000000001</v>
       </c>
       <c r="R1" s="1">
         <v>0</v>
       </c>
       <c r="S1" s="1">
-        <v>1.6257000000000001E-2</v>
+        <v>1.5500999999999999E-2</v>
       </c>
       <c r="T1" s="1">
         <v>7.5600000000000005E-4</v>
@@ -446,7 +446,7 @@
         <v>0</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.113709</v>
+        <v>0.10428999999999999</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -455,22 +455,22 @@
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>0.436699</v>
+        <v>0.43948599999999999</v>
       </c>
       <c r="B2" s="1">
-        <v>3.2951160000000002</v>
+        <v>3.248532</v>
       </c>
       <c r="C2" s="1">
-        <v>4.5511999999999997E-2</v>
+        <v>4.5532999999999997E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>8.3059999999999991E-3</v>
+        <v>6.0410000000000004E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>1.2082000000000001E-2</v>
+        <v>1.0949E-2</v>
       </c>
       <c r="F2" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>4.1529999999999996E-3</v>
       </c>
       <c r="G2" s="1">
         <v>3.7800000000000003E-4</v>
@@ -482,7 +482,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>0.16650499999999999</v>
+        <v>0.160464</v>
       </c>
       <c r="K2" s="1">
         <v>1.1329999999999999E-3</v>
@@ -491,25 +491,25 @@
         <v>7.5500000000000003E-4</v>
       </c>
       <c r="M2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="N2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="O2" s="1">
         <v>0</v>
       </c>
       <c r="P2" s="1">
-        <v>6.1300000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>6.0860999999999998E-2</v>
+        <v>5.2576999999999999E-2</v>
       </c>
       <c r="R2" s="1">
         <v>1.598E-3</v>
       </c>
       <c r="S2" s="1">
-        <v>4.3478000000000003E-2</v>
+        <v>3.9319E-2</v>
       </c>
       <c r="T2" s="1">
         <v>0</v>
@@ -518,7 +518,7 @@
         <v>0</v>
       </c>
       <c r="V2" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W2" s="1">
         <v>0</v>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="AA2" s="1">
         <v>0</v>
@@ -542,10 +542,10 @@
         <v>0</v>
       </c>
       <c r="AD2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>0.156134</v>
+        <v>0.13989799999999999</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -560,13 +560,13 @@
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>1.507655</v>
+        <v>1.6666529999999999</v>
       </c>
       <c r="D3" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>9.7410999999999998E-2</v>
+        <v>0.10609499999999999</v>
       </c>
       <c r="F3" s="1">
         <v>3.7800000000000003E-4</v>
@@ -578,13 +578,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="J3" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="K3" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>2.643E-3</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -599,25 +599,25 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>6.2040000000000003E-3</v>
+        <v>7.4609999999999998E-3</v>
       </c>
       <c r="Q3" s="1">
         <v>2.7330000000000002E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>3.5750000000000001E-3</v>
+        <v>2.3549999999999999E-3</v>
       </c>
       <c r="S3" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="T3" s="1">
-        <v>8.3180000000000007E-3</v>
+        <v>7.9399999999999991E-3</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
       </c>
       <c r="V3" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
@@ -656,40 +656,40 @@
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>1.3320000000000001E-3</v>
+        <v>3.0409999999999999E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>7.5919999999999998E-3</v>
+        <v>1.2343E-2</v>
       </c>
       <c r="D4" s="1">
-        <v>0.57389400000000002</v>
+        <v>0.61957899999999999</v>
       </c>
       <c r="E4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>0.128749</v>
+        <v>0.13969799999999999</v>
       </c>
       <c r="G4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="H4" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="I4" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
       <c r="J4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>5.6629999999999996E-3</v>
+        <v>6.4190000000000002E-3</v>
       </c>
       <c r="M4" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="N4" s="1">
         <v>3.7800000000000003E-4</v>
@@ -701,25 +701,25 @@
         <v>1.232E-3</v>
       </c>
       <c r="Q4" s="1">
-        <v>1.4041E-2</v>
+        <v>2.2120000000000001E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>2.647E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="T4" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="U4" s="1">
-        <v>6.0489999999999997E-3</v>
+        <v>5.6709999999999998E-3</v>
       </c>
       <c r="V4" s="1">
         <v>0</v>
       </c>
       <c r="W4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -728,13 +728,13 @@
         <v>0</v>
       </c>
       <c r="Z4" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AA4" s="1">
         <v>0</v>
       </c>
       <c r="AB4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="1">
         <v>0</v>
@@ -758,13 +758,13 @@
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>7.4213000000000001E-2</v>
+        <v>7.3457999999999996E-2</v>
       </c>
       <c r="D5" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="E5" s="1">
-        <v>0.14083100000000001</v>
+        <v>0.149892</v>
       </c>
       <c r="F5" s="1">
         <v>1.5100000000000001E-3</v>
@@ -782,7 +782,7 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="K5" s="1">
-        <v>1.2460000000000001E-2</v>
+        <v>1.1704000000000001E-2</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -803,7 +803,7 @@
         <v>0</v>
       </c>
       <c r="R5" s="1">
-        <v>0</v>
+        <v>1.2199999999999999E-3</v>
       </c>
       <c r="S5" s="1">
         <v>0</v>
@@ -815,7 +815,7 @@
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="W5" s="1">
         <v>3.7800000000000003E-4</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>5.2859999999999999E-3</v>
+        <v>6.0410000000000004E-3</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -860,13 +860,13 @@
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>2.1520999999999998E-2</v>
+        <v>2.3408999999999999E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>9.2880000000000004E-2</v>
+        <v>9.8166000000000003E-2</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>1.0194E-2</v>
+        <v>1.0572E-2</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -899,25 +899,25 @@
         <v>0</v>
       </c>
       <c r="Q6" s="1">
-        <v>2.441E-3</v>
+        <v>1.2199999999999999E-3</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="1">
-        <v>7.1739999999999998E-3</v>
+        <v>7.5519999999999997E-3</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -968,13 +968,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>8.6840000000000007E-3</v>
+        <v>9.4389999999999995E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
@@ -1007,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U7" s="1">
         <v>0</v>
@@ -1070,10 +1070,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="I8" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="J8" s="1">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="O8" s="1">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1205,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="T9" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U9" s="1">
         <v>0</v>
@@ -1247,22 +1247,22 @@
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
-        <v>7.4349999999999998E-3</v>
+        <v>8.77E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>0.101383</v>
+        <v>9.3612000000000001E-2</v>
       </c>
       <c r="C10" s="1">
-        <v>4.9290000000000002E-3</v>
+        <v>6.2610000000000001E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>2.643E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>4.1529999999999996E-3</v>
+        <v>3.398E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,13 +1274,13 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>7.2492000000000001E-2</v>
+        <v>7.1359000000000006E-2</v>
       </c>
       <c r="K10" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="L10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>1.977E-3</v>
+        <v>1.598E-3</v>
       </c>
       <c r="R10" s="1">
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>7.1830000000000001E-3</v>
+        <v>6.0489999999999997E-3</v>
       </c>
       <c r="T10" s="1">
         <v>0</v>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="1">
-        <v>3.4030000000000002E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="AA10" s="1">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="AE10" s="1">
-        <v>6.3432000000000002E-2</v>
+        <v>5.7014000000000002E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1358,7 +1358,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>2.643E-3</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>2.643E-3</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="AA11" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="1">
-        <v>1.511E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>4.7195000000000001E-2</v>
+        <v>5.4746000000000003E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
@@ -1784,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>2.643E-3</v>
+        <v>3.0200000000000001E-3</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1847,7 +1847,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="1">
-        <v>5.6426999999999998E-2</v>
+        <v>6.8014000000000005E-2</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
@@ -1886,19 +1886,19 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.84121599999999996</v>
+        <v>0.97987900000000006</v>
       </c>
       <c r="Q16" s="1">
-        <v>4.7949999999999998E-3</v>
+        <v>3.5750000000000001E-3</v>
       </c>
       <c r="R16" s="1">
-        <v>0.16694400000000001</v>
+        <v>0.194324</v>
       </c>
       <c r="S16" s="1">
         <v>0</v>
       </c>
       <c r="T16" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
@@ -1913,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>2.647E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="Z16" s="1">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>1.2563E-2</v>
+        <v>1.2184E-2</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1940,22 +1940,22 @@
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>1.0853E-2</v>
+        <v>1.2194999999999999E-2</v>
       </c>
       <c r="B17" s="1">
         <v>9.3019999999999995E-3</v>
       </c>
       <c r="C17" s="1">
+        <v>3.4190000000000002E-3</v>
+      </c>
+      <c r="D17" s="1">
+        <v>3.5112999999999998E-2</v>
+      </c>
+      <c r="E17" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
-      <c r="D17" s="1">
-        <v>3.3603000000000001E-2</v>
-      </c>
-      <c r="E17" s="1">
-        <v>0</v>
-      </c>
       <c r="F17" s="1">
-        <v>6.4190000000000002E-3</v>
+        <v>7.1739999999999998E-3</v>
       </c>
       <c r="G17" s="1">
         <v>0</v>
@@ -1979,34 +1979,34 @@
         <v>0</v>
       </c>
       <c r="N17" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>3.104E-3</v>
+        <v>5.5890000000000002E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>3.726648</v>
+        <v>4.110214</v>
       </c>
       <c r="R17" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="S17" s="1">
-        <v>0.31115300000000001</v>
+        <v>0.33534999999999998</v>
       </c>
       <c r="T17" s="1">
-        <v>1.0586E-2</v>
+        <v>1.0964E-2</v>
       </c>
       <c r="U17" s="1">
+        <v>1.89E-3</v>
+      </c>
+      <c r="V17" s="1">
+        <v>1.5120000000000001E-3</v>
+      </c>
+      <c r="W17" s="1">
         <v>7.5600000000000005E-4</v>
-      </c>
-      <c r="V17" s="1">
-        <v>1.134E-3</v>
-      </c>
-      <c r="W17" s="1">
-        <v>3.7800000000000003E-4</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="AE17" s="1">
-        <v>1.323E-2</v>
+        <v>1.3608E-2</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2045,13 +2045,13 @@
         <v>0</v>
       </c>
       <c r="C18" s="1">
-        <v>9.5010000000000008E-3</v>
+        <v>1.0255999999999999E-2</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>5.6629999999999996E-3</v>
+        <v>9.4389999999999995E-3</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -2084,13 +2084,13 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>5.8796000000000001E-2</v>
+        <v>5.5121000000000003E-2</v>
       </c>
       <c r="Q18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
-        <v>0.35392000000000001</v>
+        <v>0.38112699999999999</v>
       </c>
       <c r="S18" s="1">
         <v>1.5120000000000001E-3</v>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="1">
-        <v>1.134E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="W18" s="1">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>1.7013E-2</v>
+        <v>1.8526000000000001E-2</v>
       </c>
       <c r="Z18" s="1">
         <v>0</v>
@@ -2129,7 +2129,7 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="AE18" s="1">
-        <v>1.899E-2</v>
+        <v>2.0879999999999999E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2144,16 +2144,16 @@
         <v>2.464E-3</v>
       </c>
       <c r="C19" s="1">
-        <v>1.3320000000000001E-3</v>
+        <v>1.709E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>7.9290000000000003E-3</v>
+        <v>8.3059999999999991E-3</v>
       </c>
       <c r="E19" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="F19" s="1">
-        <v>9.4389999999999995E-3</v>
+        <v>1.0949E-2</v>
       </c>
       <c r="G19" s="1">
         <v>0</v>
@@ -2162,16 +2162,16 @@
         <v>0</v>
       </c>
       <c r="I19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="J19" s="1">
-        <v>0</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="M19" s="1">
         <v>3.7800000000000003E-4</v>
@@ -2186,25 +2186,25 @@
         <v>0</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.167355</v>
+        <v>0.17025999999999999</v>
       </c>
       <c r="R19" s="1">
         <v>4.0390000000000001E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>0.390926</v>
+        <v>0.41134199999999999</v>
       </c>
       <c r="T19" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="U19" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="V19" s="1">
         <v>7.5600000000000005E-4</v>
       </c>
       <c r="W19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="X19" s="1">
         <v>0</v>
@@ -2213,7 +2213,7 @@
         <v>0</v>
       </c>
       <c r="Z19" s="1">
-        <v>2.4197E-2</v>
+        <v>2.6842999999999999E-2</v>
       </c>
       <c r="AA19" s="1">
         <v>0</v>
@@ -2228,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>1.5499000000000001E-2</v>
+        <v>1.3609E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>2.0869999999999999E-3</v>
+        <v>3.4190000000000002E-3</v>
       </c>
       <c r="D20" s="1">
         <v>3.7800000000000003E-4</v>
@@ -2255,7 +2255,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -2294,13 +2294,13 @@
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>6.3894000000000006E-2</v>
+        <v>7.6370999999999994E-2</v>
       </c>
       <c r="U20" s="1">
         <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>1.4744999999999999E-2</v>
+        <v>1.7769E-2</v>
       </c>
       <c r="W20" s="1">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AB20" s="1">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>1.134E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2357,7 +2357,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="I21" s="1">
         <v>0</v>
@@ -2384,25 +2384,25 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <v>2.8189999999999999E-3</v>
+        <v>4.0390000000000001E-3</v>
       </c>
       <c r="R21" s="1">
         <v>0</v>
       </c>
       <c r="S21" s="1">
-        <v>1.134E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="T21" s="1">
         <v>0</v>
       </c>
       <c r="U21" s="1">
-        <v>1.172E-2</v>
+        <v>1.2475999999999999E-2</v>
       </c>
       <c r="V21" s="1">
         <v>0</v>
       </c>
       <c r="W21" s="1">
-        <v>1.0208E-2</v>
+        <v>1.1342E-2</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="AB21" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AC21" s="1">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>3.4020000000000001E-3</v>
+        <v>3.0240000000000002E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2498,7 +2498,7 @@
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>1.0586E-2</v>
+        <v>1.1342E-2</v>
       </c>
       <c r="W22" s="1">
         <v>3.7800000000000003E-4</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="1">
-        <v>1.89E-3</v>
+        <v>2.2680000000000001E-3</v>
       </c>
       <c r="AB22" s="1">
         <v>0</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>3.4030000000000002E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>2.6459999999999999E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="L25" s="1">
         <v>0</v>
@@ -2777,13 +2777,13 @@
         <v>0</v>
       </c>
       <c r="P25" s="1">
-        <v>1.2359999999999999E-3</v>
+        <v>2.4949999999999998E-3</v>
       </c>
       <c r="Q25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>1.4385999999999999E-2</v>
+        <v>1.3544E-2</v>
       </c>
       <c r="S25" s="1">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="1">
-        <v>9.8300000000000002E-3</v>
+        <v>1.0964E-2</v>
       </c>
       <c r="Z25" s="1">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="1">
-        <v>6.8050000000000003E-3</v>
+        <v>7.9399999999999991E-3</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2846,7 +2846,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="G26" s="1">
         <v>0</v>
@@ -2885,7 +2885,7 @@
         <v>0</v>
       </c>
       <c r="S26" s="1">
-        <v>9.8300000000000002E-3</v>
+        <v>1.0586E-2</v>
       </c>
       <c r="T26" s="1">
         <v>7.5600000000000005E-4</v>
@@ -2900,13 +2900,13 @@
         <v>0</v>
       </c>
       <c r="X26" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="Y26" s="1">
         <v>0</v>
       </c>
       <c r="Z26" s="1">
-        <v>8.3180000000000007E-3</v>
+        <v>9.0740000000000005E-3</v>
       </c>
       <c r="AA26" s="1">
         <v>0</v>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>4.9150000000000001E-3</v>
+        <v>4.5370000000000002E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -3110,13 +3110,13 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>7.561E-3</v>
+        <v>8.3180000000000007E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
       </c>
       <c r="AD28" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AE28" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
fit corr plot drawer
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8649B3-1937-4C33-A27F-C4ADE1CFA2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F32FB0-C0A0-4908-A0AA-C2FC59AD2D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,22 +356,22 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>9.7890940000000004</v>
+        <v>8.2884180000000001</v>
       </c>
       <c r="B1" s="1">
-        <v>1.991169</v>
+        <v>1.9901530000000001</v>
       </c>
       <c r="C1" s="1">
-        <v>0.113939</v>
+        <v>0.126083</v>
       </c>
       <c r="D1" s="1">
-        <v>1.9633000000000001E-2</v>
+        <v>1.8123E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>6.796E-3</v>
       </c>
       <c r="F1" s="1">
-        <v>7.1739999999999998E-3</v>
+        <v>1.0572E-2</v>
       </c>
       <c r="G1" s="1">
         <v>0</v>
@@ -383,16 +383,16 @@
         <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>3.1337999999999998E-2</v>
+        <v>3.6246E-2</v>
       </c>
       <c r="K1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="L1" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="M1" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="N1" s="1">
         <v>0</v>
@@ -401,16 +401,16 @@
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>1.2279999999999999E-3</v>
+        <v>6.1200000000000002E-4</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.28952800000000001</v>
+        <v>0.24680099999999999</v>
       </c>
       <c r="R1" s="1">
         <v>0</v>
       </c>
       <c r="S1" s="1">
-        <v>1.5500999999999999E-2</v>
+        <v>1.5122999999999999E-2</v>
       </c>
       <c r="T1" s="1">
         <v>7.5600000000000005E-4</v>
@@ -446,7 +446,7 @@
         <v>0</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.10428999999999999</v>
+        <v>0.126388</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -455,25 +455,25 @@
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
-        <v>0.43948599999999999</v>
+        <v>0.29477100000000001</v>
       </c>
       <c r="B2" s="1">
-        <v>3.248532</v>
+        <v>2.419508</v>
       </c>
       <c r="C2" s="1">
-        <v>4.5532999999999997E-2</v>
+        <v>3.0925000000000001E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>6.0410000000000004E-3</v>
+        <v>4.5310000000000003E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>1.0949E-2</v>
+        <v>7.1739999999999998E-3</v>
       </c>
       <c r="F2" s="1">
-        <v>4.1529999999999996E-3</v>
+        <v>3.398E-3</v>
       </c>
       <c r="G2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
@@ -482,10 +482,10 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>0.160464</v>
+        <v>0.107228</v>
       </c>
       <c r="K2" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="L2" s="1">
         <v>7.5500000000000003E-4</v>
@@ -503,13 +503,13 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>5.2576999999999999E-2</v>
+        <v>2.8514000000000001E-2</v>
       </c>
       <c r="R2" s="1">
-        <v>1.598E-3</v>
+        <v>1.2199999999999999E-3</v>
       </c>
       <c r="S2" s="1">
-        <v>3.9319E-2</v>
+        <v>2.3819E-2</v>
       </c>
       <c r="T2" s="1">
         <v>0</v>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>1.89E-3</v>
+        <v>2.2680000000000001E-3</v>
       </c>
       <c r="AA2" s="1">
         <v>0</v>
@@ -542,10 +542,10 @@
         <v>0</v>
       </c>
       <c r="AD2" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AE2" s="1">
-        <v>0.13989799999999999</v>
+        <v>9.3456999999999998E-2</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -560,13 +560,13 @@
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>1.6666529999999999</v>
+        <v>1.3433360000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>0.10609499999999999</v>
+        <v>7.7399999999999997E-2</v>
       </c>
       <c r="F3" s="1">
         <v>3.7800000000000003E-4</v>
@@ -581,10 +581,10 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="J3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="K3" s="1">
-        <v>2.643E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -599,19 +599,19 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>7.4609999999999998E-3</v>
+        <v>1.2359999999999999E-3</v>
       </c>
       <c r="Q3" s="1">
-        <v>2.7330000000000002E-3</v>
+        <v>1.977E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>2.3549999999999999E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="S3" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="T3" s="1">
-        <v>7.9399999999999991E-3</v>
+        <v>4.1590000000000004E-3</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>4.1539999999999997E-3</v>
+        <v>4.5319999999999996E-3</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -656,28 +656,28 @@
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>3.0409999999999999E-3</v>
+        <v>1.3320000000000001E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>1.2343E-2</v>
+        <v>6.8370000000000002E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>0.61957899999999999</v>
+        <v>0.47346199999999999</v>
       </c>
       <c r="E4" s="1">
+        <v>3.7800000000000003E-4</v>
+      </c>
+      <c r="F4" s="1">
+        <v>9.4768000000000005E-2</v>
+      </c>
+      <c r="G4" s="1">
+        <v>3.7800000000000003E-4</v>
+      </c>
+      <c r="H4" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
-      <c r="F4" s="1">
-        <v>0.13969799999999999</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1">
-        <v>1.5100000000000001E-3</v>
-      </c>
       <c r="I4" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J4" s="1">
         <v>0</v>
@@ -686,10 +686,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>6.4190000000000002E-3</v>
+        <v>4.1529999999999996E-3</v>
       </c>
       <c r="M4" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="N4" s="1">
         <v>3.7800000000000003E-4</v>
@@ -698,28 +698,28 @@
         <v>0</v>
       </c>
       <c r="P4" s="1">
-        <v>1.232E-3</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <v>2.2120000000000001E-2</v>
+        <v>1.0260999999999999E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
+        <v>2.2680000000000001E-3</v>
+      </c>
+      <c r="T4" s="1">
+        <v>0</v>
+      </c>
+      <c r="U4" s="1">
         <v>3.0249999999999999E-3</v>
       </c>
-      <c r="T4" s="1">
-        <v>3.7800000000000003E-4</v>
-      </c>
-      <c r="U4" s="1">
-        <v>5.6709999999999998E-3</v>
-      </c>
       <c r="V4" s="1">
         <v>0</v>
       </c>
       <c r="W4" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -728,13 +728,13 @@
         <v>0</v>
       </c>
       <c r="Z4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="1">
         <v>0</v>
       </c>
       <c r="AB4" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AC4" s="1">
         <v>0</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>1.5480000000000001E-2</v>
+        <v>9.4389999999999995E-3</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -758,16 +758,16 @@
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>7.3457999999999996E-2</v>
+        <v>6.2089999999999999E-2</v>
       </c>
       <c r="D5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="E5" s="1">
-        <v>0.149892</v>
+        <v>0.117044</v>
       </c>
       <c r="F5" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="G5" s="1">
         <v>0</v>
@@ -779,10 +779,10 @@
         <v>1.1329999999999999E-3</v>
       </c>
       <c r="J5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="K5" s="1">
-        <v>1.1704000000000001E-2</v>
+        <v>1.0194E-2</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -803,19 +803,19 @@
         <v>0</v>
       </c>
       <c r="R5" s="1">
-        <v>1.2199999999999999E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="S5" s="1">
         <v>0</v>
       </c>
       <c r="T5" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="U5" s="1">
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>2.647E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="W5" s="1">
         <v>3.7800000000000003E-4</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>6.0410000000000004E-3</v>
+        <v>4.5310000000000003E-3</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -860,13 +860,13 @@
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>2.3408999999999999E-2</v>
+        <v>1.3592E-2</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>9.8166000000000003E-2</v>
+        <v>7.2869000000000003E-2</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>1.0572E-2</v>
+        <v>8.3059999999999991E-3</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -905,19 +905,19 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>2.647E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="1">
-        <v>7.5519999999999997E-3</v>
+        <v>4.9090000000000002E-3</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -968,13 +968,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>9.4389999999999995E-3</v>
+        <v>8.6840000000000007E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
@@ -1007,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="T7" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="U7" s="1">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="AE7" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
@@ -1070,10 +1070,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J8" s="1">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="O8" s="1">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1172,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -1205,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="T9" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="U9" s="1">
         <v>0</v>
@@ -1247,22 +1247,22 @@
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
-        <v>8.77E-3</v>
+        <v>4.0619999999999996E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>9.3612000000000001E-2</v>
+        <v>7.2366E-2</v>
       </c>
       <c r="C10" s="1">
-        <v>6.2610000000000001E-3</v>
+        <v>7.5919999999999998E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="E10" s="1">
-        <v>2.643E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>3.398E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,13 +1274,13 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>7.1359000000000006E-2</v>
+        <v>5.0215999999999997E-2</v>
       </c>
       <c r="K10" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="L10" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>1.598E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="R10" s="1">
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>6.0489999999999997E-3</v>
+        <v>3.7810000000000001E-3</v>
       </c>
       <c r="T10" s="1">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="AE10" s="1">
-        <v>5.7014000000000002E-2</v>
+        <v>3.7002E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1358,7 +1358,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>2.643E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>2.643E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -1397,19 +1397,19 @@
         <v>0</v>
       </c>
       <c r="R11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="S11" s="1">
         <v>0</v>
       </c>
       <c r="T11" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U11" s="1">
         <v>0</v>
       </c>
       <c r="V11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1460,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
@@ -1535,7 +1535,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>5.4746000000000003E-2</v>
+        <v>3.7379000000000003E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>4.1529999999999996E-3</v>
+        <v>3.0200000000000001E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1628,7 +1628,7 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>1.134E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="AD13" s="1">
         <v>0</v>
@@ -1778,13 +1778,13 @@
         <v>0</v>
       </c>
       <c r="M15" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="N15" s="1">
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>3.0200000000000001E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1847,7 +1847,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="1">
-        <v>6.8014000000000005E-2</v>
+        <v>4.1798000000000002E-2</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
@@ -1886,19 +1886,19 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.97987900000000006</v>
+        <v>0.83131900000000003</v>
       </c>
       <c r="Q16" s="1">
-        <v>3.5750000000000001E-3</v>
+        <v>2.3549999999999999E-3</v>
       </c>
       <c r="R16" s="1">
-        <v>0.194324</v>
+        <v>0.151835</v>
       </c>
       <c r="S16" s="1">
         <v>0</v>
       </c>
       <c r="T16" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
@@ -1913,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="Z16" s="1">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>1.2184E-2</v>
+        <v>9.2460000000000007E-3</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1940,22 +1940,22 @@
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
-        <v>1.2194999999999999E-2</v>
+        <v>8.8389999999999996E-3</v>
       </c>
       <c r="B17" s="1">
-        <v>9.3019999999999995E-3</v>
+        <v>5.5050000000000003E-3</v>
       </c>
       <c r="C17" s="1">
-        <v>3.4190000000000002E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="D17" s="1">
-        <v>3.5112999999999998E-2</v>
+        <v>2.7562E-2</v>
       </c>
       <c r="E17" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="F17" s="1">
-        <v>7.1739999999999998E-3</v>
+        <v>4.5310000000000003E-3</v>
       </c>
       <c r="G17" s="1">
         <v>0</v>
@@ -1985,28 +1985,28 @@
         <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>5.5890000000000002E-3</v>
+        <v>4.3340000000000002E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>4.110214</v>
+        <v>3.3363689999999999</v>
       </c>
       <c r="R17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="S17" s="1">
-        <v>0.33534999999999998</v>
+        <v>0.25973499999999999</v>
       </c>
       <c r="T17" s="1">
-        <v>1.0964E-2</v>
+        <v>8.3180000000000007E-3</v>
       </c>
       <c r="U17" s="1">
-        <v>1.89E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="V17" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="W17" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2015,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>9.4520000000000003E-3</v>
+        <v>8.6960000000000006E-3</v>
       </c>
       <c r="AA17" s="1">
         <v>0</v>
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="AE17" s="1">
-        <v>1.3608E-2</v>
+        <v>7.9369999999999996E-3</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2045,13 +2045,13 @@
         <v>0</v>
       </c>
       <c r="C18" s="1">
-        <v>1.0255999999999999E-2</v>
+        <v>4.7499999999999999E-3</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>9.4389999999999995E-3</v>
+        <v>6.0410000000000004E-3</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -2084,25 +2084,25 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>5.5121000000000003E-2</v>
+        <v>4.7659E-2</v>
       </c>
       <c r="Q18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
-        <v>0.38112699999999999</v>
+        <v>0.33336500000000002</v>
       </c>
       <c r="S18" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="T18" s="1">
-        <v>1.134E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U18" s="1">
         <v>0</v>
       </c>
       <c r="V18" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="W18" s="1">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>1.8526000000000001E-2</v>
+        <v>1.5879000000000001E-2</v>
       </c>
       <c r="Z18" s="1">
         <v>0</v>
@@ -2126,10 +2126,10 @@
         <v>0</v>
       </c>
       <c r="AD18" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>2.0879999999999999E-2</v>
+        <v>1.8610999999999999E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2141,19 +2141,19 @@
         <v>0</v>
       </c>
       <c r="B19" s="1">
-        <v>2.464E-3</v>
+        <v>2.0869999999999999E-3</v>
       </c>
       <c r="C19" s="1">
         <v>1.709E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>8.3059999999999991E-3</v>
+        <v>4.5310000000000003E-3</v>
       </c>
       <c r="E19" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="F19" s="1">
-        <v>1.0949E-2</v>
+        <v>6.4190000000000002E-3</v>
       </c>
       <c r="G19" s="1">
         <v>0</v>
@@ -2162,19 +2162,19 @@
         <v>0</v>
       </c>
       <c r="I19" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J19" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="M19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="N19" s="1">
         <v>0</v>
@@ -2186,41 +2186,41 @@
         <v>0</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.17025999999999999</v>
+        <v>0.13564499999999999</v>
       </c>
       <c r="R19" s="1">
-        <v>4.0390000000000001E-3</v>
+        <v>1.2199999999999999E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>0.41134199999999999</v>
+        <v>0.31795899999999999</v>
       </c>
       <c r="T19" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>3.4030000000000002E-3</v>
       </c>
       <c r="U19" s="1">
         <v>0</v>
       </c>
       <c r="V19" s="1">
+        <v>1.134E-3</v>
+      </c>
+      <c r="W19" s="1">
+        <v>0</v>
+      </c>
+      <c r="X19" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="1">
+        <v>1.7769E-2</v>
+      </c>
+      <c r="AA19" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="1">
         <v>7.5600000000000005E-4</v>
       </c>
-      <c r="W19" s="1">
-        <v>0</v>
-      </c>
-      <c r="X19" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z19" s="1">
-        <v>2.6842999999999999E-2</v>
-      </c>
-      <c r="AA19" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="1">
-        <v>3.7800000000000003E-4</v>
-      </c>
       <c r="AC19" s="1">
         <v>0</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>1.3609E-2</v>
+        <v>8.3180000000000007E-3</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2243,19 +2243,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>3.4190000000000002E-3</v>
+        <v>1.3320000000000001E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -2294,13 +2294,13 @@
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>7.6370999999999994E-2</v>
+        <v>5.5577000000000001E-2</v>
       </c>
       <c r="U20" s="1">
         <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>1.7769E-2</v>
+        <v>1.2475999999999999E-2</v>
       </c>
       <c r="W20" s="1">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AB20" s="1">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2351,7 +2351,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="G21" s="1">
         <v>0</v>
@@ -2384,7 +2384,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <v>4.0390000000000001E-3</v>
+        <v>2.8189999999999999E-3</v>
       </c>
       <c r="R21" s="1">
         <v>0</v>
@@ -2396,13 +2396,13 @@
         <v>0</v>
       </c>
       <c r="U21" s="1">
-        <v>1.2475999999999999E-2</v>
+        <v>1.0586E-2</v>
       </c>
       <c r="V21" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W21" s="1">
-        <v>1.1342E-2</v>
+        <v>7.9399999999999991E-3</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="AB21" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="1">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>3.0240000000000002E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>2.647E-3</v>
+        <v>2.2680000000000001E-3</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>1.1342E-2</v>
+        <v>9.4520000000000003E-3</v>
       </c>
       <c r="W22" s="1">
         <v>3.7800000000000003E-4</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="AB22" s="1">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
@@ -2543,7 +2543,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>3.4030000000000002E-3</v>
+        <v>2.2680000000000001E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>1.89E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2744,7 +2744,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="L25" s="1">
         <v>0</v>
@@ -2777,13 +2777,13 @@
         <v>0</v>
       </c>
       <c r="P25" s="1">
-        <v>2.4949999999999998E-3</v>
+        <v>1.2359999999999999E-3</v>
       </c>
       <c r="Q25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>1.3544E-2</v>
+        <v>1.4008E-2</v>
       </c>
       <c r="S25" s="1">
         <v>0</v>
@@ -2795,7 +2795,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W25" s="1">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="1">
-        <v>1.0964E-2</v>
+        <v>8.6960000000000006E-3</v>
       </c>
       <c r="Z25" s="1">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="1">
-        <v>7.9399999999999991E-3</v>
+        <v>5.6709999999999998E-3</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2879,13 +2879,13 @@
         <v>0</v>
       </c>
       <c r="Q26" s="1">
-        <v>1.977E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="R26" s="1">
         <v>0</v>
       </c>
       <c r="S26" s="1">
-        <v>1.0586E-2</v>
+        <v>7.1830000000000001E-3</v>
       </c>
       <c r="T26" s="1">
         <v>7.5600000000000005E-4</v>
@@ -2894,19 +2894,19 @@
         <v>0</v>
       </c>
       <c r="V26" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W26" s="1">
         <v>0</v>
       </c>
       <c r="X26" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="Y26" s="1">
         <v>0</v>
       </c>
       <c r="Z26" s="1">
-        <v>9.0740000000000005E-3</v>
+        <v>6.4270000000000004E-3</v>
       </c>
       <c r="AA26" s="1">
         <v>0</v>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>4.5370000000000002E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -3110,7 +3110,7 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>8.3180000000000007E-3</v>
+        <v>6.8050000000000003E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
@@ -3218,7 +3218,7 @@
         <v>0</v>
       </c>
       <c r="AE29" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>

</xml_diff>

<commit_message>
add fit to data
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\purol\OneDrive\바탕 화면\github\Belle2_script\Belle2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F32FB0-C0A0-4908-A0AA-C2FC59AD2D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBDF2781-7FE3-45FE-8737-702512D499C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,19 +27,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Yu Gothic"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="6"/>
-      <name val="Yu Gothic"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -67,7 +67,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -349,29 +349,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI30"/>
-  <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="35" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="35" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:35">
       <c r="A1" s="1">
-        <v>8.2884180000000001</v>
+        <v>10.413365000000001</v>
       </c>
       <c r="B1" s="1">
-        <v>1.9901530000000001</v>
+        <v>2.224002</v>
       </c>
       <c r="C1" s="1">
-        <v>0.126083</v>
+        <v>0.124332</v>
       </c>
       <c r="D1" s="1">
-        <v>1.8123E-2</v>
+        <v>3.4736000000000003E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>6.796E-3</v>
+        <v>4.908E-3</v>
       </c>
       <c r="F1" s="1">
-        <v>1.0572E-2</v>
+        <v>1.2082000000000001E-2</v>
       </c>
       <c r="G1" s="1">
         <v>0</v>
@@ -380,19 +380,19 @@
         <v>0</v>
       </c>
       <c r="I1" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="J1" s="1">
-        <v>3.6246E-2</v>
+        <v>3.7755999999999998E-2</v>
       </c>
       <c r="K1" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
       <c r="L1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="M1" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="N1" s="1">
         <v>0</v>
@@ -401,25 +401,25 @@
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>6.1200000000000002E-4</v>
+        <v>1.2440000000000001E-3</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.24680099999999999</v>
+        <v>0.468696</v>
       </c>
       <c r="R1" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="S1" s="1">
-        <v>1.5122999999999999E-2</v>
+        <v>2.9489999999999999E-2</v>
       </c>
       <c r="T1" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.134E-3</v>
       </c>
       <c r="U1" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="V1" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W1" s="1">
         <v>0</v>
@@ -431,7 +431,7 @@
         <v>0</v>
       </c>
       <c r="Z1" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.134E-3</v>
       </c>
       <c r="AA1" s="1">
         <v>0</v>
@@ -446,34 +446,34 @@
         <v>0</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.126388</v>
+        <v>0.119036</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
       <c r="AH1" s="1"/>
       <c r="AI1" s="1"/>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:35">
       <c r="A2" s="1">
-        <v>0.29477100000000001</v>
+        <v>0.32779599999999998</v>
       </c>
       <c r="B2" s="1">
-        <v>2.419508</v>
+        <v>2.4604490000000001</v>
       </c>
       <c r="C2" s="1">
-        <v>3.0925000000000001E-2</v>
+        <v>2.6175E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>6.796E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>7.1739999999999998E-3</v>
+        <v>6.796E-3</v>
       </c>
       <c r="F2" s="1">
-        <v>3.398E-3</v>
+        <v>6.0410000000000004E-3</v>
       </c>
       <c r="G2" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
@@ -482,13 +482,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>0.107228</v>
+        <v>9.1747999999999996E-2</v>
       </c>
       <c r="K2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="L2" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -500,16 +500,16 @@
         <v>0</v>
       </c>
       <c r="P2" s="1">
-        <v>0</v>
+        <v>6.1799999999999995E-4</v>
       </c>
       <c r="Q2" s="1">
-        <v>2.8514000000000001E-2</v>
+        <v>4.4877E-2</v>
       </c>
       <c r="R2" s="1">
-        <v>1.2199999999999999E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="S2" s="1">
-        <v>2.3819E-2</v>
+        <v>4.0076000000000001E-2</v>
       </c>
       <c r="T2" s="1">
         <v>0</v>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="AA2" s="1">
         <v>0</v>
@@ -542,17 +542,17 @@
         <v>0</v>
       </c>
       <c r="AD2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>9.3456999999999998E-2</v>
+        <v>7.4957999999999997E-2</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
       <c r="AH2" s="1"/>
       <c r="AI2" s="1"/>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:35">
       <c r="A3" s="1">
         <v>0</v>
       </c>
@@ -560,16 +560,16 @@
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>1.3433360000000001</v>
+        <v>1.3919509999999999</v>
       </c>
       <c r="D3" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>7.7399999999999997E-2</v>
+        <v>7.2869000000000003E-2</v>
       </c>
       <c r="F3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="G3" s="1">
         <v>7.5500000000000003E-4</v>
@@ -584,7 +584,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>2.2650000000000001E-3</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -599,25 +599,25 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>1.2359999999999999E-3</v>
+        <v>6.842E-3</v>
       </c>
       <c r="Q3" s="1">
-        <v>1.977E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.5750000000000001E-3</v>
       </c>
       <c r="S3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="T3" s="1">
-        <v>4.1590000000000004E-3</v>
+        <v>1.172E-2</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
       </c>
       <c r="V3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.134E-3</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
@@ -644,82 +644,82 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>4.5319999999999996E-3</v>
+        <v>2.6440000000000001E-3</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
       <c r="AH3" s="1"/>
       <c r="AI3" s="1"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:35">
       <c r="A4" s="1">
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>1.3320000000000001E-3</v>
+        <v>2.663E-3</v>
       </c>
       <c r="C4" s="1">
         <v>6.8370000000000002E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>0.47346199999999999</v>
+        <v>0.48630000000000001</v>
       </c>
       <c r="E4" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>9.4768000000000005E-2</v>
+        <v>9.0236999999999998E-2</v>
       </c>
       <c r="G4" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="H4" s="1">
+        <v>1.1329999999999999E-3</v>
+      </c>
+      <c r="I4" s="1">
+        <v>3.7800000000000003E-4</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>2.2650000000000001E-3</v>
+      </c>
+      <c r="M4" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
-      <c r="I4" s="1">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1">
-        <v>0</v>
-      </c>
-      <c r="K4" s="1">
-        <v>0</v>
-      </c>
-      <c r="L4" s="1">
-        <v>4.1529999999999996E-3</v>
-      </c>
-      <c r="M4" s="1">
-        <v>3.7800000000000003E-4</v>
-      </c>
       <c r="N4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="O4" s="1">
         <v>0</v>
       </c>
       <c r="P4" s="1">
-        <v>0</v>
+        <v>1.232E-3</v>
       </c>
       <c r="Q4" s="1">
-        <v>1.0260999999999999E-2</v>
+        <v>1.7703E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>4.1590000000000004E-3</v>
       </c>
       <c r="T4" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U4" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>5.6709999999999998E-3</v>
       </c>
       <c r="V4" s="1">
         <v>0</v>
       </c>
       <c r="W4" s="1">
-        <v>0</v>
+        <v>1.134E-3</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -734,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="AB4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="1">
         <v>0</v>
@@ -743,14 +743,14 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>9.4389999999999995E-3</v>
+        <v>9.0609999999999996E-3</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="1"/>
       <c r="AI4" s="1"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:35">
       <c r="A5" s="1">
         <v>0</v>
       </c>
@@ -758,31 +758,31 @@
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>6.2089999999999999E-2</v>
+        <v>6.4732999999999999E-2</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1">
-        <v>0.117044</v>
+        <v>0.117799</v>
       </c>
       <c r="F5" s="1">
+        <v>1.1329999999999999E-3</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
-      <c r="G5" s="1">
-        <v>0</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1">
-        <v>1.1329999999999999E-3</v>
-      </c>
       <c r="J5" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="K5" s="1">
-        <v>1.0194E-2</v>
+        <v>9.8169999999999993E-3</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -803,19 +803,19 @@
         <v>0</v>
       </c>
       <c r="R5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.598E-3</v>
       </c>
       <c r="S5" s="1">
         <v>0</v>
       </c>
       <c r="T5" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="U5" s="1">
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>1.134E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="W5" s="1">
         <v>3.7800000000000003E-4</v>
@@ -824,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="Y5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="1">
         <v>0</v>
@@ -842,14 +842,14 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>2.2659999999999998E-3</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
       <c r="AH5" s="1"/>
       <c r="AI5" s="1"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:35">
       <c r="A6" s="1">
         <v>0</v>
       </c>
@@ -860,13 +860,13 @@
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>1.3592E-2</v>
+        <v>1.9255999999999999E-2</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>7.2869000000000003E-2</v>
+        <v>7.7778E-2</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
@@ -875,7 +875,7 @@
         <v>7.5500000000000003E-4</v>
       </c>
       <c r="I6" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>8.3059999999999991E-3</v>
+        <v>5.6629999999999996E-3</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -905,19 +905,19 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>1.134E-3</v>
+        <v>3.4030000000000002E-3</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>1.134E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
@@ -941,14 +941,14 @@
         <v>0</v>
       </c>
       <c r="AE6" s="1">
-        <v>4.9090000000000002E-3</v>
+        <v>4.5310000000000003E-3</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
       <c r="AH6" s="1"/>
       <c r="AI6" s="1"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:35">
       <c r="A7" s="1">
         <v>0</v>
       </c>
@@ -968,7 +968,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>8.6840000000000007E-3</v>
+        <v>7.5510000000000004E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
@@ -1040,14 +1040,14 @@
         <v>0</v>
       </c>
       <c r="AE7" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
       <c r="AH7" s="1"/>
       <c r="AI7" s="1"/>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:35">
       <c r="A8" s="1">
         <v>0</v>
       </c>
@@ -1070,7 +1070,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="I8" s="1">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="O8" s="1">
         <v>0</v>
@@ -1139,14 +1139,14 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
       <c r="AH8" s="1"/>
       <c r="AI8" s="1"/>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:35">
       <c r="A9" s="1">
         <v>0</v>
       </c>
@@ -1238,22 +1238,22 @@
         <v>0</v>
       </c>
       <c r="AE9" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="AF9" s="1"/>
       <c r="AG9" s="1"/>
       <c r="AH9" s="1"/>
       <c r="AI9" s="1"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:35">
       <c r="A10" s="1">
-        <v>4.0619999999999996E-3</v>
+        <v>6.7330000000000003E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>7.2366E-2</v>
+        <v>6.4555000000000001E-2</v>
       </c>
       <c r="C10" s="1">
-        <v>7.5919999999999998E-3</v>
+        <v>3.9750000000000002E-3</v>
       </c>
       <c r="D10" s="1">
         <v>7.5500000000000003E-4</v>
@@ -1262,7 +1262,7 @@
         <v>1.5100000000000001E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>4.1529999999999996E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>5.0215999999999997E-2</v>
+        <v>4.9083000000000002E-2</v>
       </c>
       <c r="K10" s="1">
         <v>3.7800000000000003E-4</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.2199999999999999E-3</v>
       </c>
       <c r="R10" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="S10" s="1">
-        <v>3.7810000000000001E-3</v>
+        <v>6.4270000000000004E-3</v>
       </c>
       <c r="T10" s="1">
         <v>0</v>
@@ -1337,14 +1337,14 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="AE10" s="1">
-        <v>3.7002E-2</v>
+        <v>3.3981999999999998E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
       <c r="AH10" s="1"/>
       <c r="AI10" s="1"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:35">
       <c r="A11" s="1">
         <v>0</v>
       </c>
@@ -1358,26 +1358,26 @@
         <v>0</v>
       </c>
       <c r="E11" s="1">
+        <v>1.5100000000000001E-3</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1">
         <v>1.1329999999999999E-3</v>
       </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0</v>
-      </c>
-      <c r="H11" s="1">
-        <v>0</v>
-      </c>
-      <c r="I11" s="1">
-        <v>0</v>
-      </c>
-      <c r="J11" s="1">
-        <v>0</v>
-      </c>
-      <c r="K11" s="1">
-        <v>1.8879999999999999E-3</v>
-      </c>
       <c r="L11" s="1">
         <v>0</v>
       </c>
@@ -1403,13 +1403,13 @@
         <v>0</v>
       </c>
       <c r="T11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="U11" s="1">
         <v>0</v>
       </c>
       <c r="V11" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="AA11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
@@ -1436,14 +1436,14 @@
         <v>0</v>
       </c>
       <c r="AE11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
       <c r="AH11" s="1"/>
       <c r="AI11" s="1"/>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:35">
       <c r="A12" s="1">
         <v>0</v>
       </c>
@@ -1460,89 +1460,89 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
+        <v>1.5100000000000001E-3</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3.7800000000000003E-4</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1">
+        <v>3.7800000000000003E-4</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="N12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
+        <v>0</v>
+      </c>
+      <c r="P12" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>0</v>
+      </c>
+      <c r="R12" s="1">
+        <v>0</v>
+      </c>
+      <c r="S12" s="1">
+        <v>0</v>
+      </c>
+      <c r="T12" s="1">
+        <v>0</v>
+      </c>
+      <c r="U12" s="1">
+        <v>0</v>
+      </c>
+      <c r="V12" s="1">
+        <v>0</v>
+      </c>
+      <c r="W12" s="1">
+        <v>1.134E-3</v>
+      </c>
+      <c r="X12" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="1">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="1">
         <v>7.5500000000000003E-4</v>
-      </c>
-      <c r="G12" s="1">
-        <v>0</v>
-      </c>
-      <c r="H12" s="1">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1">
-        <v>3.7800000000000003E-4</v>
-      </c>
-      <c r="J12" s="1">
-        <v>0</v>
-      </c>
-      <c r="K12" s="1">
-        <v>0</v>
-      </c>
-      <c r="L12" s="1">
-        <v>7.5500000000000003E-4</v>
-      </c>
-      <c r="M12" s="1">
-        <v>0</v>
-      </c>
-      <c r="N12" s="1">
-        <v>0</v>
-      </c>
-      <c r="O12" s="1">
-        <v>0</v>
-      </c>
-      <c r="P12" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="1">
-        <v>0</v>
-      </c>
-      <c r="R12" s="1">
-        <v>0</v>
-      </c>
-      <c r="S12" s="1">
-        <v>0</v>
-      </c>
-      <c r="T12" s="1">
-        <v>0</v>
-      </c>
-      <c r="U12" s="1">
-        <v>0</v>
-      </c>
-      <c r="V12" s="1">
-        <v>0</v>
-      </c>
-      <c r="W12" s="1">
-        <v>3.7800000000000003E-4</v>
-      </c>
-      <c r="X12" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="1">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="1">
-        <v>0</v>
-      </c>
-      <c r="AE12" s="1">
-        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
       <c r="AH12" s="1"/>
       <c r="AI12" s="1"/>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:35">
       <c r="A13" s="1">
         <v>0</v>
       </c>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>3.7379000000000003E-2</v>
+        <v>4.0777000000000001E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>3.0200000000000001E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1641,7 +1641,7 @@
       <c r="AH13" s="1"/>
       <c r="AI13" s="1"/>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:35">
       <c r="A14" s="1">
         <v>0</v>
       </c>
@@ -1740,7 +1740,7 @@
       <c r="AH14" s="1"/>
       <c r="AI14" s="1"/>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:35">
       <c r="A15" s="1">
         <v>0</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>2.2650000000000001E-3</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1839,7 +1839,7 @@
       <c r="AH15" s="1"/>
       <c r="AI15" s="1"/>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:35">
       <c r="A16" s="1">
         <v>0</v>
       </c>
@@ -1847,19 +1847,19 @@
         <v>0</v>
       </c>
       <c r="C16" s="1">
-        <v>4.1798000000000002E-2</v>
+        <v>8.4928000000000003E-2</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
       </c>
       <c r="G16" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="H16" s="1">
         <v>0</v>
@@ -1886,16 +1886,16 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.83131900000000003</v>
+        <v>0.86192800000000003</v>
       </c>
       <c r="Q16" s="1">
-        <v>2.3549999999999999E-3</v>
+        <v>1.977E-3</v>
       </c>
       <c r="R16" s="1">
-        <v>0.151835</v>
+        <v>0.135267</v>
       </c>
       <c r="S16" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="T16" s="1">
         <v>1.5120000000000001E-3</v>
@@ -1904,7 +1904,7 @@
         <v>0</v>
       </c>
       <c r="V16" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="W16" s="1">
         <v>0</v>
@@ -1913,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>1.89E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="Z16" s="1">
         <v>0</v>
@@ -1931,31 +1931,31 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>9.2460000000000007E-3</v>
+        <v>4.2449999999999996E-3</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
       <c r="AH16" s="1"/>
       <c r="AI16" s="1"/>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:35">
       <c r="A17" s="1">
-        <v>8.8389999999999996E-3</v>
+        <v>1.0812E-2</v>
       </c>
       <c r="B17" s="1">
-        <v>5.5050000000000003E-3</v>
+        <v>5.8830000000000002E-3</v>
       </c>
       <c r="C17" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7959999999999999E-3</v>
       </c>
       <c r="D17" s="1">
-        <v>2.7562E-2</v>
+        <v>4.342E-2</v>
       </c>
       <c r="E17" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="F17" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>6.0410000000000004E-3</v>
       </c>
       <c r="G17" s="1">
         <v>0</v>
@@ -1979,34 +1979,34 @@
         <v>0</v>
       </c>
       <c r="N17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="O17" s="1">
         <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>4.3340000000000002E-3</v>
+        <v>4.352E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>3.3363689999999999</v>
+        <v>3.31019</v>
       </c>
       <c r="R17" s="1">
         <v>0</v>
       </c>
       <c r="S17" s="1">
-        <v>0.25973499999999999</v>
+        <v>0.22117200000000001</v>
       </c>
       <c r="T17" s="1">
-        <v>8.3180000000000007E-3</v>
+        <v>6.8050000000000003E-3</v>
       </c>
       <c r="U17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.134E-3</v>
       </c>
       <c r="V17" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W17" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2015,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>8.6960000000000006E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="AA17" s="1">
         <v>0</v>
@@ -2030,14 +2030,14 @@
         <v>0</v>
       </c>
       <c r="AE17" s="1">
-        <v>7.9369999999999996E-3</v>
+        <v>4.1570000000000001E-3</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
       <c r="AH17" s="1"/>
       <c r="AI17" s="1"/>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:35">
       <c r="A18" s="1">
         <v>0</v>
       </c>
@@ -2045,13 +2045,13 @@
         <v>0</v>
       </c>
       <c r="C18" s="1">
-        <v>4.7499999999999999E-3</v>
+        <v>1.3098E-2</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>6.0410000000000004E-3</v>
+        <v>1.0194E-2</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>0</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -2084,19 +2084,19 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>4.7659E-2</v>
+        <v>4.7657999999999999E-2</v>
       </c>
       <c r="Q18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
-        <v>0.33336500000000002</v>
+        <v>0.31578200000000001</v>
       </c>
       <c r="S18" s="1">
+        <v>7.5600000000000005E-4</v>
+      </c>
+      <c r="T18" s="1">
         <v>1.134E-3</v>
-      </c>
-      <c r="T18" s="1">
-        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U18" s="1">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>1.5879000000000001E-2</v>
+        <v>1.172E-2</v>
       </c>
       <c r="Z18" s="1">
         <v>0</v>
@@ -2129,52 +2129,52 @@
         <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>1.8610999999999999E-2</v>
+        <v>9.5379999999999996E-3</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
       <c r="AH18" s="1"/>
       <c r="AI18" s="1"/>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:35">
       <c r="A19" s="1">
         <v>0</v>
       </c>
       <c r="B19" s="1">
-        <v>2.0869999999999999E-3</v>
+        <v>2.464E-3</v>
       </c>
       <c r="C19" s="1">
-        <v>1.709E-3</v>
+        <v>3.0409999999999999E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>7.5510000000000004E-3</v>
       </c>
       <c r="E19" s="1">
+        <v>1.5100000000000001E-3</v>
+      </c>
+      <c r="F19" s="1">
+        <v>1.3592E-2</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
+        <v>0</v>
+      </c>
+      <c r="I19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J19" s="1">
         <v>7.5500000000000003E-4</v>
       </c>
-      <c r="F19" s="1">
-        <v>6.4190000000000002E-3</v>
-      </c>
-      <c r="G19" s="1">
-        <v>0</v>
-      </c>
-      <c r="H19" s="1">
-        <v>0</v>
-      </c>
-      <c r="I19" s="1">
-        <v>0</v>
-      </c>
-      <c r="J19" s="1">
-        <v>3.7800000000000003E-4</v>
-      </c>
       <c r="K19" s="1">
         <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="M19" s="1">
-        <v>0</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="N19" s="1">
         <v>0</v>
@@ -2186,25 +2186,25 @@
         <v>0</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.13564499999999999</v>
+        <v>0.137793</v>
       </c>
       <c r="R19" s="1">
         <v>1.2199999999999999E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>0.31795899999999999</v>
+        <v>0.31115300000000001</v>
       </c>
       <c r="T19" s="1">
-        <v>3.4030000000000002E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="U19" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="V19" s="1">
         <v>1.134E-3</v>
       </c>
       <c r="W19" s="1">
-        <v>0</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="X19" s="1">
         <v>0</v>
@@ -2213,13 +2213,13 @@
         <v>0</v>
       </c>
       <c r="Z19" s="1">
-        <v>1.7769E-2</v>
+        <v>1.7391E-2</v>
       </c>
       <c r="AA19" s="1">
         <v>0</v>
       </c>
       <c r="AB19" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AC19" s="1">
         <v>0</v>
@@ -2228,14 +2228,14 @@
         <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>8.3180000000000007E-3</v>
+        <v>1.078E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
       <c r="AH19" s="1"/>
       <c r="AI19" s="1"/>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:35">
       <c r="A20" s="1">
         <v>0</v>
       </c>
@@ -2243,19 +2243,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>1.3320000000000001E-3</v>
+        <v>3.4190000000000002E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="E20" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -2294,13 +2294,13 @@
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>5.5577000000000001E-2</v>
+        <v>5.3308000000000001E-2</v>
       </c>
       <c r="U20" s="1">
         <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>1.2475999999999999E-2</v>
+        <v>1.172E-2</v>
       </c>
       <c r="W20" s="1">
         <v>0</v>
@@ -2327,14 +2327,14 @@
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
       <c r="AH20" s="1"/>
       <c r="AI20" s="1"/>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:35">
       <c r="A21" s="1">
         <v>0</v>
       </c>
@@ -2345,19 +2345,19 @@
         <v>0</v>
       </c>
       <c r="D21" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>0</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="G21" s="1">
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="I21" s="1">
         <v>0</v>
@@ -2384,7 +2384,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <v>2.8189999999999999E-3</v>
+        <v>4.4169999999999999E-3</v>
       </c>
       <c r="R21" s="1">
         <v>0</v>
@@ -2396,13 +2396,13 @@
         <v>0</v>
       </c>
       <c r="U21" s="1">
-        <v>1.0586E-2</v>
+        <v>9.4520000000000003E-3</v>
       </c>
       <c r="V21" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W21" s="1">
-        <v>7.9399999999999991E-3</v>
+        <v>6.4270000000000004E-3</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2426,14 +2426,14 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>1.134E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
       <c r="AH21" s="1"/>
       <c r="AI21" s="1"/>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:35">
       <c r="A22" s="1">
         <v>0</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="J22" s="1">
         <v>0</v>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>9.4520000000000003E-3</v>
+        <v>7.561E-3</v>
       </c>
       <c r="W22" s="1">
         <v>3.7800000000000003E-4</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="1">
-        <v>1.89E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="AB22" s="1">
         <v>0</v>
@@ -2532,7 +2532,7 @@
       <c r="AH22" s="1"/>
       <c r="AI22" s="1"/>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:35">
       <c r="A23" s="1">
         <v>0</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
@@ -2594,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="U23" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="V23" s="1">
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,14 +2624,14 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>1.134E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
       <c r="AH23" s="1"/>
       <c r="AI23" s="1"/>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:35">
       <c r="A24" s="1">
         <v>0</v>
       </c>
@@ -2730,7 +2730,7 @@
       <c r="AH24" s="1"/>
       <c r="AI24" s="1"/>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:35">
       <c r="A25" s="1">
         <v>0</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>0</v>
       </c>
       <c r="C25" s="1">
-        <v>0</v>
+        <v>1.3320000000000001E-3</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="L25" s="1">
         <v>0</v>
@@ -2783,7 +2783,7 @@
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>1.4008E-2</v>
+        <v>1.3166000000000001E-2</v>
       </c>
       <c r="S25" s="1">
         <v>0</v>
@@ -2795,7 +2795,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W25" s="1">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="1">
-        <v>8.6960000000000006E-3</v>
+        <v>7.561E-3</v>
       </c>
       <c r="Z25" s="1">
         <v>0</v>
@@ -2829,7 +2829,7 @@
       <c r="AH25" s="1"/>
       <c r="AI25" s="1"/>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:35">
       <c r="A26" s="1">
         <v>0</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="F26" s="1">
         <v>7.5500000000000003E-4</v>
@@ -2879,13 +2879,13 @@
         <v>0</v>
       </c>
       <c r="Q26" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.977E-3</v>
       </c>
       <c r="R26" s="1">
         <v>0</v>
       </c>
       <c r="S26" s="1">
-        <v>7.1830000000000001E-3</v>
+        <v>7.9399999999999991E-3</v>
       </c>
       <c r="T26" s="1">
         <v>7.5600000000000005E-4</v>
@@ -2921,14 +2921,14 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>3.7810000000000001E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
       <c r="AH26" s="1"/>
       <c r="AI26" s="1"/>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:35">
       <c r="A27" s="1">
         <v>0</v>
       </c>
@@ -3027,7 +3027,7 @@
       <c r="AH27" s="1"/>
       <c r="AI27" s="1"/>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:35">
       <c r="A28" s="1">
         <v>0</v>
       </c>
@@ -3110,7 +3110,7 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>6.8050000000000003E-3</v>
+        <v>6.4270000000000004E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
@@ -3126,7 +3126,7 @@
       <c r="AH28" s="1"/>
       <c r="AI28" s="1"/>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:35">
       <c r="A29" s="1">
         <v>0</v>
       </c>
@@ -3225,7 +3225,7 @@
       <c r="AH29" s="1"/>
       <c r="AI29" s="1"/>
     </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:35">
       <c r="A30" s="1">
         <v>0</v>
       </c>
@@ -3314,7 +3314,7 @@
         <v>0</v>
       </c>
       <c r="AD30" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AE30" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
correction Knn for generic instead of special
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBDF2781-7FE3-45FE-8737-702512D499C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0626C4ED-7DF4-4ACA-B28A-9538161EE145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,22 +356,22 @@
   <sheetData>
     <row r="1" spans="1:35">
       <c r="A1" s="1">
-        <v>10.413365000000001</v>
+        <v>10.218211999999999</v>
       </c>
       <c r="B1" s="1">
-        <v>2.224002</v>
+        <v>2.2635209999999999</v>
       </c>
       <c r="C1" s="1">
-        <v>0.124332</v>
+        <v>0.101796</v>
       </c>
       <c r="D1" s="1">
-        <v>3.4736000000000003E-2</v>
+        <v>3.1715E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>4.908E-3</v>
+        <v>4.5310000000000003E-3</v>
       </c>
       <c r="F1" s="1">
-        <v>1.2082000000000001E-2</v>
+        <v>1.397E-2</v>
       </c>
       <c r="G1" s="1">
         <v>0</v>
@@ -380,19 +380,19 @@
         <v>0</v>
       </c>
       <c r="I1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>3.7755999999999998E-2</v>
+        <v>4.0022000000000002E-2</v>
       </c>
       <c r="K1" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="L1" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="M1" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="N1" s="1">
         <v>0</v>
@@ -401,25 +401,25 @@
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>1.2440000000000001E-3</v>
+        <v>6.1700000000000004E-4</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.468696</v>
+        <v>0.470586</v>
       </c>
       <c r="R1" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="S1" s="1">
-        <v>2.9489999999999999E-2</v>
+        <v>2.9867999999999999E-2</v>
       </c>
       <c r="T1" s="1">
-        <v>1.134E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="U1" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="V1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W1" s="1">
         <v>0</v>
@@ -428,7 +428,7 @@
         <v>0</v>
       </c>
       <c r="Y1" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="Z1" s="1">
         <v>1.134E-3</v>
@@ -446,7 +446,7 @@
         <v>0</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.119036</v>
+        <v>0.13278599999999999</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -455,19 +455,19 @@
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="1">
-        <v>0.32779599999999998</v>
+        <v>0.32299299999999997</v>
       </c>
       <c r="B2" s="1">
-        <v>2.4604490000000001</v>
+        <v>2.3872719999999998</v>
       </c>
       <c r="C2" s="1">
-        <v>2.6175E-2</v>
+        <v>2.7129E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>6.796E-3</v>
+        <v>6.4190000000000002E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>6.796E-3</v>
+        <v>4.908E-3</v>
       </c>
       <c r="F2" s="1">
         <v>6.0410000000000004E-3</v>
@@ -482,13 +482,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>9.1747999999999996E-2</v>
+        <v>9.5522999999999997E-2</v>
       </c>
       <c r="K2" s="1">
         <v>0</v>
       </c>
       <c r="L2" s="1">
-        <v>0</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -503,22 +503,22 @@
         <v>6.1799999999999995E-4</v>
       </c>
       <c r="Q2" s="1">
-        <v>4.4877E-2</v>
+        <v>5.0049999999999997E-2</v>
       </c>
       <c r="R2" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="S2" s="1">
-        <v>4.0076000000000001E-2</v>
+        <v>3.4783000000000001E-2</v>
       </c>
       <c r="T2" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="U2" s="1">
         <v>0</v>
       </c>
       <c r="V2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="W2" s="1">
         <v>0</v>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>2.647E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="AA2" s="1">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>7.4957999999999997E-2</v>
+        <v>8.3067000000000002E-2</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -557,28 +557,28 @@
         <v>0</v>
       </c>
       <c r="B3" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="C3" s="1">
-        <v>1.3919509999999999</v>
+        <v>1.3043180000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>7.2869000000000003E-2</v>
+        <v>7.2492000000000001E-2</v>
       </c>
       <c r="F3" s="1">
         <v>0</v>
       </c>
       <c r="G3" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="J3" s="1">
         <v>0</v>
@@ -599,19 +599,19 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>6.842E-3</v>
+        <v>5.5859999999999998E-3</v>
       </c>
       <c r="Q3" s="1">
         <v>1.134E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>3.5750000000000001E-3</v>
+        <v>2.7330000000000002E-3</v>
       </c>
       <c r="S3" s="1">
         <v>0</v>
       </c>
       <c r="T3" s="1">
-        <v>1.172E-2</v>
+        <v>1.2097999999999999E-2</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>2.6440000000000001E-3</v>
+        <v>4.1539999999999997E-3</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -659,58 +659,58 @@
         <v>2.663E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>6.8370000000000002E-3</v>
+        <v>5.5050000000000003E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>0.48630000000000001</v>
+        <v>0.459115</v>
       </c>
       <c r="E4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>9.0236999999999998E-2</v>
+        <v>9.6278000000000002E-2</v>
       </c>
       <c r="G4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="H4" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="I4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J4" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>3.398E-3</v>
       </c>
       <c r="M4" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="N4" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="O4" s="1">
         <v>0</v>
       </c>
       <c r="P4" s="1">
-        <v>1.232E-3</v>
+        <v>6.1499999999999999E-4</v>
       </c>
       <c r="Q4" s="1">
-        <v>1.7703E-2</v>
+        <v>1.8459E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>4.1590000000000004E-3</v>
+        <v>3.4030000000000002E-3</v>
       </c>
       <c r="T4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="U4" s="1">
         <v>5.6709999999999998E-3</v>
@@ -719,7 +719,7 @@
         <v>0</v>
       </c>
       <c r="W4" s="1">
-        <v>1.134E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>9.0609999999999996E-3</v>
+        <v>9.4389999999999995E-3</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -758,31 +758,31 @@
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>6.4732999999999999E-2</v>
+        <v>6.2268999999999998E-2</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1">
-        <v>0.117799</v>
+        <v>0.117422</v>
       </c>
       <c r="F5" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="G5" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="J5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="K5" s="1">
-        <v>9.8169999999999993E-3</v>
+        <v>8.6840000000000007E-3</v>
       </c>
       <c r="L5" s="1">
         <v>0</v>
@@ -809,13 +809,13 @@
         <v>0</v>
       </c>
       <c r="T5" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="U5" s="1">
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>3.7810000000000001E-3</v>
       </c>
       <c r="W5" s="1">
         <v>3.7800000000000003E-4</v>
@@ -824,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="Y5" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="Z5" s="1">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>2.2659999999999998E-3</v>
+        <v>2.2650000000000001E-3</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -860,19 +860,19 @@
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>1.9255999999999999E-2</v>
+        <v>1.5858000000000001E-2</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>7.7778E-2</v>
+        <v>7.8909999999999994E-2</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="I6" s="1">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>5.6629999999999996E-3</v>
+        <v>7.5510000000000004E-3</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -905,19 +905,19 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>3.4030000000000002E-3</v>
+        <v>3.0249999999999999E-3</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>2.2680000000000001E-3</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
@@ -926,7 +926,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AA6" s="1">
         <v>0</v>
@@ -962,13 +962,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>7.5510000000000004E-3</v>
+        <v>6.796E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
@@ -1013,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="V7" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
@@ -1115,7 +1115,7 @@
         <v>0</v>
       </c>
       <c r="W8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="X8" s="1">
         <v>0</v>
@@ -1172,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -1247,22 +1247,22 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="1">
-        <v>6.7330000000000003E-3</v>
+        <v>6.7349999999999997E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>6.4555000000000001E-2</v>
+        <v>6.5310000000000007E-2</v>
       </c>
       <c r="C10" s="1">
-        <v>3.9750000000000002E-3</v>
+        <v>3.2200000000000002E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="E10" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>4.1529999999999996E-3</v>
+        <v>3.398E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,16 +1274,16 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>4.9083000000000002E-2</v>
+        <v>4.8704999999999998E-2</v>
       </c>
       <c r="K10" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="L10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="M10" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="N10" s="1">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>1.2199999999999999E-3</v>
+        <v>2.8189999999999999E-3</v>
       </c>
       <c r="R10" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="S10" s="1">
-        <v>6.4270000000000004E-3</v>
+        <v>7.1830000000000001E-3</v>
       </c>
       <c r="T10" s="1">
         <v>0</v>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>2.647E-3</v>
       </c>
       <c r="AA10" s="1">
         <v>0</v>
@@ -1334,10 +1334,10 @@
         <v>0</v>
       </c>
       <c r="AD10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AE10" s="1">
-        <v>3.3981999999999998E-2</v>
+        <v>3.3605999999999997E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -1460,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -1511,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="W12" s="1">
-        <v>1.134E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="X12" s="1">
         <v>0</v>
@@ -1535,7 +1535,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>4.0777000000000001E-2</v>
+        <v>3.7379000000000003E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>2.2650000000000001E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1628,13 +1628,13 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AD13" s="1">
         <v>0</v>
       </c>
       <c r="AE13" s="1">
-        <v>0</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
@@ -1784,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>1.8879999999999999E-3</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1847,7 +1847,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="1">
-        <v>8.4928000000000003E-2</v>
+        <v>8.4728999999999999E-2</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
@@ -1859,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="H16" s="1">
         <v>0</v>
@@ -1886,25 +1886,25 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.86192800000000003</v>
+        <v>0.81438900000000003</v>
       </c>
       <c r="Q16" s="1">
-        <v>1.977E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="R16" s="1">
-        <v>0.135267</v>
+        <v>0.14427400000000001</v>
       </c>
       <c r="S16" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="T16" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
       </c>
       <c r="V16" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="W16" s="1">
         <v>0</v>
@@ -1919,7 +1919,7 @@
         <v>0</v>
       </c>
       <c r="AA16" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AB16" s="1">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>4.2449999999999996E-3</v>
+        <v>7.7340000000000004E-3</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1940,22 +1940,22 @@
     </row>
     <row r="17" spans="1:35">
       <c r="A17" s="1">
-        <v>1.0812E-2</v>
+        <v>1.0111E-2</v>
       </c>
       <c r="B17" s="1">
-        <v>5.8830000000000002E-3</v>
+        <v>8.5459999999999998E-3</v>
       </c>
       <c r="C17" s="1">
-        <v>3.7959999999999999E-3</v>
+        <v>2.8419999999999999E-3</v>
       </c>
       <c r="D17" s="1">
-        <v>4.342E-2</v>
+        <v>4.4174999999999999E-2</v>
       </c>
       <c r="E17" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="F17" s="1">
-        <v>6.0410000000000004E-3</v>
+        <v>7.5510000000000004E-3</v>
       </c>
       <c r="G17" s="1">
         <v>0</v>
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="L17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="M17" s="1">
         <v>0</v>
@@ -1985,28 +1985,28 @@
         <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>4.352E-3</v>
+        <v>4.3470000000000002E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>3.31019</v>
+        <v>3.1307369999999999</v>
       </c>
       <c r="R17" s="1">
         <v>0</v>
       </c>
       <c r="S17" s="1">
-        <v>0.22117200000000001</v>
+        <v>0.214367</v>
       </c>
       <c r="T17" s="1">
-        <v>6.8050000000000003E-3</v>
+        <v>4.1590000000000004E-3</v>
       </c>
       <c r="U17" s="1">
         <v>1.134E-3</v>
       </c>
       <c r="V17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.134E-3</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2015,7 +2015,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>6.8050000000000003E-3</v>
       </c>
       <c r="AA17" s="1">
         <v>0</v>
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="AE17" s="1">
-        <v>4.1570000000000001E-3</v>
+        <v>7.5579999999999996E-3</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2045,13 +2045,13 @@
         <v>0</v>
       </c>
       <c r="C18" s="1">
-        <v>1.3098E-2</v>
+        <v>1.1011E-2</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>1.0194E-2</v>
+        <v>9.8169999999999993E-3</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2069,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -2084,16 +2084,16 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>4.7657999999999999E-2</v>
+        <v>4.5194999999999999E-2</v>
       </c>
       <c r="Q18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
-        <v>0.31578200000000001</v>
+        <v>0.30304700000000001</v>
       </c>
       <c r="S18" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.134E-3</v>
       </c>
       <c r="T18" s="1">
         <v>1.134E-3</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>1.172E-2</v>
+        <v>1.3233E-2</v>
       </c>
       <c r="Z18" s="1">
         <v>0</v>
@@ -2129,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>9.5379999999999996E-3</v>
+        <v>1.0293E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2141,7 +2141,7 @@
         <v>0</v>
       </c>
       <c r="B19" s="1">
-        <v>2.464E-3</v>
+        <v>2.0869999999999999E-3</v>
       </c>
       <c r="C19" s="1">
         <v>3.0409999999999999E-3</v>
@@ -2150,10 +2150,10 @@
         <v>7.5510000000000004E-3</v>
       </c>
       <c r="E19" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.1329999999999999E-3</v>
       </c>
       <c r="F19" s="1">
-        <v>1.3592E-2</v>
+        <v>1.2836999999999999E-2</v>
       </c>
       <c r="G19" s="1">
         <v>0</v>
@@ -2165,7 +2165,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
@@ -2174,7 +2174,7 @@
         <v>1.5100000000000001E-3</v>
       </c>
       <c r="M19" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="N19" s="1">
         <v>0</v>
@@ -2186,25 +2186,25 @@
         <v>0</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.137793</v>
+        <v>0.13683200000000001</v>
       </c>
       <c r="R19" s="1">
-        <v>1.2199999999999999E-3</v>
+        <v>1.598E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>0.31115300000000001</v>
+        <v>0.299433</v>
       </c>
       <c r="T19" s="1">
-        <v>2.647E-3</v>
+        <v>1.89E-3</v>
       </c>
       <c r="U19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="V19" s="1">
-        <v>1.134E-3</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W19" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="X19" s="1">
         <v>0</v>
@@ -2213,7 +2213,7 @@
         <v>0</v>
       </c>
       <c r="Z19" s="1">
-        <v>1.7391E-2</v>
+        <v>1.6257000000000001E-2</v>
       </c>
       <c r="AA19" s="1">
         <v>0</v>
@@ -2228,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>1.078E-2</v>
+        <v>9.4490000000000008E-3</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2243,19 +2243,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>3.4190000000000002E-3</v>
+        <v>2.0869999999999999E-3</v>
       </c>
       <c r="D20" s="1">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="E20" s="1">
-        <v>0</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -2294,13 +2294,13 @@
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>5.3308000000000001E-2</v>
+        <v>4.7636999999999999E-2</v>
       </c>
       <c r="U20" s="1">
         <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>1.172E-2</v>
+        <v>1.3611E-2</v>
       </c>
       <c r="W20" s="1">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>0</v>
+        <v>7.5600000000000005E-4</v>
       </c>
       <c r="AB20" s="1">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2357,7 +2357,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>7.5500000000000003E-4</v>
       </c>
       <c r="I21" s="1">
         <v>0</v>
@@ -2384,25 +2384,25 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <v>4.4169999999999999E-3</v>
+        <v>2.441E-3</v>
       </c>
       <c r="R21" s="1">
         <v>0</v>
       </c>
       <c r="S21" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="T21" s="1">
         <v>0</v>
       </c>
       <c r="U21" s="1">
-        <v>9.4520000000000003E-3</v>
+        <v>7.9399999999999991E-3</v>
       </c>
       <c r="V21" s="1">
         <v>0</v>
       </c>
       <c r="W21" s="1">
-        <v>6.4270000000000004E-3</v>
+        <v>4.9150000000000001E-3</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>3.0240000000000002E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>2.647E-3</v>
+        <v>1.5120000000000001E-3</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>7.561E-3</v>
+        <v>7.1830000000000001E-3</v>
       </c>
       <c r="W22" s="1">
         <v>3.7800000000000003E-4</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
@@ -2594,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="U23" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="V23" s="1">
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>2.647E-3</v>
+        <v>2.2680000000000001E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.134E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2744,7 +2744,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2777,7 +2777,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="1">
-        <v>1.2359999999999999E-3</v>
+        <v>6.1600000000000001E-4</v>
       </c>
       <c r="Q25" s="1">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="1">
-        <v>5.6709999999999998E-3</v>
+        <v>4.9150000000000001E-3</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2885,7 +2885,7 @@
         <v>0</v>
       </c>
       <c r="S26" s="1">
-        <v>7.9399999999999991E-3</v>
+        <v>7.561E-3</v>
       </c>
       <c r="T26" s="1">
         <v>7.5600000000000005E-4</v>
@@ -2894,7 +2894,7 @@
         <v>0</v>
       </c>
       <c r="V26" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="W26" s="1">
         <v>0</v>
@@ -2906,7 +2906,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="1">
-        <v>6.4270000000000004E-3</v>
+        <v>4.9150000000000001E-3</v>
       </c>
       <c r="AA26" s="1">
         <v>0</v>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>3.7810000000000001E-3</v>
+        <v>3.4030000000000002E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -3212,13 +3212,13 @@
         <v>0</v>
       </c>
       <c r="AC29" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AD29" s="1">
         <v>0</v>
       </c>
       <c r="AE29" s="1">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>

</xml_diff>

<commit_message>
set labet box poisition for Linearity test
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0626C4ED-7DF4-4ACA-B28A-9538161EE145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{132C67F4-B31D-4808-9377-494EDA46E597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,22 +356,22 @@
   <sheetData>
     <row r="1" spans="1:35">
       <c r="A1" s="1">
-        <v>10.218211999999999</v>
+        <v>9.921913</v>
       </c>
       <c r="B1" s="1">
-        <v>2.2635209999999999</v>
+        <v>1.993042</v>
       </c>
       <c r="C1" s="1">
-        <v>0.101796</v>
+        <v>8.0480999999999997E-2</v>
       </c>
       <c r="D1" s="1">
-        <v>3.1715E-2</v>
+        <v>3.3762E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>1.0442E-2</v>
       </c>
       <c r="F1" s="1">
-        <v>1.397E-2</v>
+        <v>1.8780999999999999E-2</v>
       </c>
       <c r="G1" s="1">
         <v>0</v>
@@ -383,43 +383,43 @@
         <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>4.0022000000000002E-2</v>
+        <v>4.8607999999999998E-2</v>
       </c>
       <c r="K1" s="1">
-        <v>0</v>
+        <v>1.1820000000000001E-3</v>
       </c>
       <c r="L1" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.621E-3</v>
       </c>
       <c r="M1" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.1969999999999999E-3</v>
       </c>
       <c r="N1" s="1">
-        <v>0</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="O1" s="1">
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>6.1700000000000004E-4</v>
+        <v>8.7900000000000001E-4</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.470586</v>
+        <v>0.358987</v>
       </c>
       <c r="R1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="S1" s="1">
-        <v>2.9867999999999999E-2</v>
+        <v>4.0078000000000003E-2</v>
       </c>
       <c r="T1" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>3.7199999999999999E-4</v>
       </c>
       <c r="U1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>9.3800000000000003E-4</v>
       </c>
       <c r="V1" s="1">
-        <v>0</v>
+        <v>4.4000000000000002E-4</v>
       </c>
       <c r="W1" s="1">
         <v>0</v>
@@ -428,10 +428,10 @@
         <v>0</v>
       </c>
       <c r="Y1" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="Z1" s="1">
-        <v>1.134E-3</v>
+        <v>6.9399999999999996E-4</v>
       </c>
       <c r="AA1" s="1">
         <v>0</v>
@@ -446,7 +446,7 @@
         <v>0</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.13278599999999999</v>
+        <v>0.15743799999999999</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -455,25 +455,25 @@
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="1">
-        <v>0.32299299999999997</v>
+        <v>0.23813999999999999</v>
       </c>
       <c r="B2" s="1">
-        <v>2.3872719999999998</v>
+        <v>1.713425</v>
       </c>
       <c r="C2" s="1">
-        <v>2.7129E-2</v>
+        <v>1.4224000000000001E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>6.4190000000000002E-3</v>
+        <v>2.8939999999999999E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>4.908E-3</v>
+        <v>9.7179999999999992E-3</v>
       </c>
       <c r="F2" s="1">
-        <v>6.0410000000000004E-3</v>
+        <v>1.1943E-2</v>
       </c>
       <c r="G2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="H2" s="1">
         <v>0</v>
@@ -482,13 +482,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>9.5522999999999997E-2</v>
+        <v>0.108473</v>
       </c>
       <c r="K2" s="1">
-        <v>0</v>
+        <v>5.4199999999999995E-4</v>
       </c>
       <c r="L2" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -500,25 +500,25 @@
         <v>0</v>
       </c>
       <c r="P2" s="1">
-        <v>6.1799999999999995E-4</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>5.0049999999999997E-2</v>
+        <v>3.1519999999999999E-2</v>
       </c>
       <c r="R2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="S2" s="1">
-        <v>3.4783000000000001E-2</v>
+        <v>6.2542E-2</v>
       </c>
       <c r="T2" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>8.5099999999999998E-4</v>
       </c>
       <c r="U2" s="1">
         <v>0</v>
       </c>
       <c r="V2" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="W2" s="1">
         <v>0</v>
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>1.89E-3</v>
+        <v>2.5920000000000001E-3</v>
       </c>
       <c r="AA2" s="1">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>8.3067000000000002E-2</v>
+        <v>6.9095000000000004E-2</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -554,37 +554,37 @@
     </row>
     <row r="3" spans="1:35">
       <c r="A3" s="1">
-        <v>0</v>
+        <v>1E-3</v>
       </c>
       <c r="B3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>1.3043180000000001</v>
+        <v>0.92485399999999995</v>
       </c>
       <c r="D3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>9.9200000000000004E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>7.2492000000000001E-2</v>
+        <v>9.0979000000000004E-2</v>
       </c>
       <c r="F3" s="1">
-        <v>0</v>
+        <v>6.8300000000000001E-4</v>
       </c>
       <c r="G3" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>2.1940000000000002E-3</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>3.59E-4</v>
       </c>
       <c r="J3" s="1">
         <v>0</v>
       </c>
       <c r="K3" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>5.2449999999999997E-3</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -599,25 +599,25 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>5.5859999999999998E-3</v>
+        <v>3.5639999999999999E-3</v>
       </c>
       <c r="Q3" s="1">
-        <v>1.134E-3</v>
+        <v>1.106E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>2.7330000000000002E-3</v>
+        <v>1.76E-4</v>
       </c>
       <c r="S3" s="1">
         <v>0</v>
       </c>
       <c r="T3" s="1">
-        <v>1.2097999999999999E-2</v>
+        <v>1.1568E-2</v>
       </c>
       <c r="U3" s="1">
         <v>0</v>
       </c>
       <c r="V3" s="1">
-        <v>1.134E-3</v>
+        <v>1.8309999999999999E-3</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>4.1539999999999997E-3</v>
+        <v>2.4819999999999998E-3</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -656,40 +656,40 @@
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>2.663E-3</v>
+        <v>1.168E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>5.5050000000000003E-3</v>
+        <v>2.41E-4</v>
       </c>
       <c r="D4" s="1">
-        <v>0.459115</v>
+        <v>0.53972600000000004</v>
       </c>
       <c r="E4" s="1">
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>9.6278000000000002E-2</v>
+        <v>0.169936</v>
       </c>
       <c r="G4" s="1">
-        <v>0</v>
+        <v>1.0059999999999999E-3</v>
       </c>
       <c r="H4" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>5.8200000000000005E-4</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
       </c>
       <c r="J4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>3.398E-3</v>
+        <v>1.2200000000000001E-2</v>
       </c>
       <c r="M4" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="N4" s="1">
         <v>0</v>
@@ -698,28 +698,28 @@
         <v>0</v>
       </c>
       <c r="P4" s="1">
-        <v>6.1499999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <v>1.8459E-2</v>
+        <v>1.4555999999999999E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>3.4030000000000002E-3</v>
+        <v>5.3429999999999997E-3</v>
       </c>
       <c r="T4" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>7.4299999999999995E-4</v>
       </c>
       <c r="U4" s="1">
-        <v>5.6709999999999998E-3</v>
+        <v>9.0950000000000007E-3</v>
       </c>
       <c r="V4" s="1">
         <v>0</v>
       </c>
       <c r="W4" s="1">
-        <v>1.89E-3</v>
+        <v>2.124E-3</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -728,7 +728,7 @@
         <v>0</v>
       </c>
       <c r="Z4" s="1">
-        <v>0</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AA4" s="1">
         <v>0</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>9.4389999999999995E-3</v>
+        <v>1.2005999999999999E-2</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -758,34 +758,34 @@
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>6.2268999999999998E-2</v>
+        <v>3.5987999999999999E-2</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1">
-        <v>0.117422</v>
+        <v>0.144652</v>
       </c>
       <c r="F5" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>4.3199999999999998E-4</v>
       </c>
       <c r="G5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.0380000000000001E-3</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>3.59E-4</v>
       </c>
       <c r="J5" s="1">
         <v>0</v>
       </c>
       <c r="K5" s="1">
-        <v>8.6840000000000007E-3</v>
+        <v>1.0409E-2</v>
       </c>
       <c r="L5" s="1">
-        <v>0</v>
+        <v>6.4000000000000005E-4</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
@@ -797,40 +797,40 @@
         <v>0</v>
       </c>
       <c r="P5" s="1">
-        <v>6.1300000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="1">
-        <v>0</v>
+        <v>9.2800000000000001E-4</v>
       </c>
       <c r="R5" s="1">
-        <v>1.598E-3</v>
+        <v>2.1050000000000001E-3</v>
       </c>
       <c r="S5" s="1">
         <v>0</v>
       </c>
       <c r="T5" s="1">
-        <v>1.89E-3</v>
+        <v>2.529E-3</v>
       </c>
       <c r="U5" s="1">
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>3.7810000000000001E-3</v>
+        <v>3.6619999999999999E-3</v>
       </c>
       <c r="W5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="X5" s="1">
         <v>0</v>
       </c>
       <c r="Y5" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="1">
         <v>0</v>
       </c>
       <c r="AA5" s="1">
-        <v>0</v>
+        <v>3.4699999999999998E-4</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>2.8219999999999999E-3</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -854,25 +854,25 @@
         <v>0</v>
       </c>
       <c r="B6" s="1">
-        <v>0</v>
+        <v>1.34E-4</v>
       </c>
       <c r="C6" s="1">
-        <v>0</v>
+        <v>1.21E-4</v>
       </c>
       <c r="D6" s="1">
-        <v>1.5858000000000001E-2</v>
+        <v>1.5311E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>0</v>
+        <v>1.5020000000000001E-3</v>
       </c>
       <c r="F6" s="1">
-        <v>7.8909999999999994E-2</v>
+        <v>9.6351000000000006E-2</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="I6" s="1">
         <v>0</v>
@@ -884,10 +884,10 @@
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>7.5510000000000004E-3</v>
+        <v>1.0189999999999999E-2</v>
       </c>
       <c r="M6" s="1">
-        <v>0</v>
+        <v>3.7500000000000001E-4</v>
       </c>
       <c r="N6" s="1">
         <v>0</v>
@@ -899,25 +899,25 @@
         <v>0</v>
       </c>
       <c r="Q6" s="1">
-        <v>1.2199999999999999E-3</v>
+        <v>1.2300000000000001E-4</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>3.0249999999999999E-3</v>
+        <v>2.2950000000000002E-3</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.0579999999999999E-3</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>9.5799999999999998E-4</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
@@ -926,10 +926,10 @@
         <v>0</v>
       </c>
       <c r="Z6" s="1">
-        <v>0</v>
+        <v>1.204E-3</v>
       </c>
       <c r="AA6" s="1">
-        <v>0</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AB6" s="1">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="1">
-        <v>4.5310000000000003E-3</v>
+        <v>6.7149999999999996E-3</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -956,25 +956,25 @@
         <v>0</v>
       </c>
       <c r="C7" s="1">
-        <v>0</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
       </c>
       <c r="E7" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>6.796E-3</v>
+        <v>2.3119999999999998E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.4350000000000001E-3</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
@@ -1013,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="V7" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="AE7" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>3.59E-4</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
@@ -1070,7 +1070,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>7.18E-4</v>
       </c>
       <c r="I8" s="1">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="O8" s="1">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1172,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>3.59E-4</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -1247,22 +1247,22 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="1">
-        <v>6.7349999999999997E-3</v>
+        <v>4.0299999999999997E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>6.5310000000000007E-2</v>
+        <v>4.5633E-2</v>
       </c>
       <c r="C10" s="1">
-        <v>3.2200000000000002E-3</v>
+        <v>5.9400000000000002E-4</v>
       </c>
       <c r="D10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>4.7100000000000001E-4</v>
       </c>
       <c r="E10" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>4.0679999999999996E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>3.398E-3</v>
+        <v>1.3649999999999999E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,16 +1274,16 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>4.8704999999999998E-2</v>
+        <v>5.7117000000000001E-2</v>
       </c>
       <c r="K10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>6.4000000000000005E-4</v>
       </c>
       <c r="L10" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>5.4199999999999995E-4</v>
       </c>
       <c r="M10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="N10" s="1">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>2.8189999999999999E-3</v>
+        <v>1.745E-3</v>
       </c>
       <c r="R10" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>7.1830000000000001E-3</v>
+        <v>4.9550000000000002E-3</v>
       </c>
       <c r="T10" s="1">
         <v>0</v>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="1">
-        <v>2.647E-3</v>
+        <v>3.4699999999999998E-4</v>
       </c>
       <c r="AA10" s="1">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="1">
-        <v>3.3605999999999997E-2</v>
+        <v>2.9277999999999998E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1352,13 +1352,13 @@
         <v>0</v>
       </c>
       <c r="C11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.116E-3</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.872E-3</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.2800000000000001E-3</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
@@ -1421,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="Z11" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="1">
         <v>0</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>7.0500000000000001E-4</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1460,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.797E-3</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -1469,7 +1469,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J12" s="1">
         <v>0</v>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>6.4000000000000005E-4</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
@@ -1511,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="W12" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="X12" s="1">
         <v>0</v>
@@ -1535,7 +1535,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.4109999999999999E-3</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
@@ -1547,19 +1547,19 @@
         <v>0</v>
       </c>
       <c r="B13" s="1">
-        <v>0</v>
+        <v>1.34E-4</v>
       </c>
       <c r="C13" s="1">
         <v>0</v>
       </c>
       <c r="D13" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.3060000000000001E-3</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>3.7379000000000003E-2</v>
+        <v>2.8874E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>2.2650000000000001E-3</v>
+        <v>2.7669999999999999E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1628,13 +1628,13 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AD13" s="1">
         <v>0</v>
       </c>
       <c r="AE13" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
@@ -1682,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="O14" s="1">
         <v>0</v>
@@ -1778,13 +1778,13 @@
         <v>0</v>
       </c>
       <c r="M15" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>4.6900000000000002E-4</v>
       </c>
       <c r="N15" s="1">
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>1.8879999999999999E-3</v>
+        <v>7.0399999999999998E-4</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1826,13 +1826,13 @@
         <v>0</v>
       </c>
       <c r="AC15" s="1">
-        <v>0</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AD15" s="1">
         <v>0</v>
       </c>
       <c r="AE15" s="1">
-        <v>0</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1"/>
@@ -1844,16 +1844,16 @@
         <v>0</v>
       </c>
       <c r="B16" s="1">
-        <v>0</v>
+        <v>9.9500000000000001E-4</v>
       </c>
       <c r="C16" s="1">
-        <v>8.4728999999999999E-2</v>
+        <v>6.9081000000000004E-2</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>6.6969999999999998E-3</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -1865,7 +1865,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="1">
-        <v>0</v>
+        <v>2.9100000000000003E-4</v>
       </c>
       <c r="J16" s="1">
         <v>0</v>
@@ -1886,25 +1886,25 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.81438900000000003</v>
+        <v>0.87813799999999997</v>
       </c>
       <c r="Q16" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.119E-3</v>
       </c>
       <c r="R16" s="1">
-        <v>0.14427400000000001</v>
+        <v>0.105959</v>
       </c>
       <c r="S16" s="1">
         <v>0</v>
       </c>
       <c r="T16" s="1">
-        <v>1.134E-3</v>
+        <v>3.7520000000000001E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
       </c>
       <c r="V16" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.8309999999999999E-3</v>
       </c>
       <c r="W16" s="1">
         <v>0</v>
@@ -1913,13 +1913,13 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>1.134E-3</v>
+        <v>1.346E-3</v>
       </c>
       <c r="Z16" s="1">
         <v>0</v>
       </c>
       <c r="AA16" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AB16" s="1">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>7.7340000000000004E-3</v>
+        <v>5.3889999999999997E-3</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1940,25 +1940,25 @@
     </row>
     <row r="17" spans="1:35">
       <c r="A17" s="1">
-        <v>1.0111E-2</v>
+        <v>1.1169E-2</v>
       </c>
       <c r="B17" s="1">
-        <v>8.5459999999999998E-3</v>
+        <v>8.3859999999999994E-3</v>
       </c>
       <c r="C17" s="1">
-        <v>2.8419999999999999E-3</v>
+        <v>3.6879999999999999E-3</v>
       </c>
       <c r="D17" s="1">
-        <v>4.4174999999999999E-2</v>
+        <v>5.6411000000000003E-2</v>
       </c>
       <c r="E17" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>7.5510000000000004E-3</v>
+        <v>1.721E-2</v>
       </c>
       <c r="G17" s="1">
-        <v>0</v>
+        <v>1.0059999999999999E-3</v>
       </c>
       <c r="H17" s="1">
         <v>0</v>
@@ -1973,10 +1973,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>6.4000000000000005E-4</v>
       </c>
       <c r="M17" s="1">
-        <v>0</v>
+        <v>2.3499999999999999E-4</v>
       </c>
       <c r="N17" s="1">
         <v>0</v>
@@ -1985,28 +1985,28 @@
         <v>0</v>
       </c>
       <c r="P17" s="1">
-        <v>4.3470000000000002E-3</v>
+        <v>3.5230000000000001E-3</v>
       </c>
       <c r="Q17" s="1">
-        <v>3.1307369999999999</v>
+        <v>2.3540679999999998</v>
       </c>
       <c r="R17" s="1">
-        <v>0</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="S17" s="1">
-        <v>0.214367</v>
+        <v>0.33002900000000002</v>
       </c>
       <c r="T17" s="1">
-        <v>4.1590000000000004E-3</v>
+        <v>7.9120000000000006E-3</v>
       </c>
       <c r="U17" s="1">
-        <v>1.134E-3</v>
+        <v>2.9880000000000002E-3</v>
       </c>
       <c r="V17" s="1">
-        <v>0</v>
+        <v>6.02E-4</v>
       </c>
       <c r="W17" s="1">
-        <v>1.134E-3</v>
+        <v>3.59E-4</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2015,22 +2015,22 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>6.8050000000000003E-3</v>
+        <v>7.9559999999999995E-3</v>
       </c>
       <c r="AA17" s="1">
         <v>0</v>
       </c>
       <c r="AB17" s="1">
-        <v>0</v>
+        <v>7.4100000000000001E-4</v>
       </c>
       <c r="AC17" s="1">
         <v>0</v>
       </c>
       <c r="AD17" s="1">
-        <v>0</v>
+        <v>3.8200000000000002E-4</v>
       </c>
       <c r="AE17" s="1">
-        <v>7.5579999999999996E-3</v>
+        <v>7.5319999999999996E-3</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2042,16 +2042,16 @@
         <v>0</v>
       </c>
       <c r="B18" s="1">
-        <v>0</v>
+        <v>1.129E-3</v>
       </c>
       <c r="C18" s="1">
-        <v>1.1011E-2</v>
+        <v>9.0720000000000002E-3</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>9.8169999999999993E-3</v>
+        <v>2.1701000000000002E-2</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2063,13 +2063,13 @@
         <v>0</v>
       </c>
       <c r="I18" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="J18" s="1">
         <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -2084,25 +2084,25 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>4.5194999999999999E-2</v>
+        <v>3.3656999999999999E-2</v>
       </c>
       <c r="Q18" s="1">
         <v>0</v>
       </c>
       <c r="R18" s="1">
-        <v>0.30304700000000001</v>
+        <v>0.19733999999999999</v>
       </c>
       <c r="S18" s="1">
-        <v>1.134E-3</v>
+        <v>1.5299999999999999E-3</v>
       </c>
       <c r="T18" s="1">
-        <v>1.134E-3</v>
+        <v>8.5099999999999998E-4</v>
       </c>
       <c r="U18" s="1">
         <v>0</v>
       </c>
       <c r="V18" s="1">
-        <v>1.89E-3</v>
+        <v>1.1360000000000001E-3</v>
       </c>
       <c r="W18" s="1">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>1.3233E-2</v>
+        <v>1.6022000000000002E-2</v>
       </c>
       <c r="Z18" s="1">
         <v>0</v>
@@ -2129,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>1.0293E-2</v>
+        <v>7.5449999999999996E-3</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2141,40 +2141,40 @@
         <v>0</v>
       </c>
       <c r="B19" s="1">
-        <v>2.0869999999999999E-3</v>
+        <v>5.2830000000000004E-3</v>
       </c>
       <c r="C19" s="1">
-        <v>3.0409999999999999E-3</v>
+        <v>1.116E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>7.5510000000000004E-3</v>
+        <v>1.2772E-2</v>
       </c>
       <c r="E19" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>1.8599999999999999E-4</v>
       </c>
       <c r="F19" s="1">
-        <v>1.2836999999999999E-2</v>
+        <v>2.7526999999999999E-2</v>
       </c>
       <c r="G19" s="1">
-        <v>0</v>
+        <v>2.7629999999999998E-3</v>
       </c>
       <c r="H19" s="1">
-        <v>0</v>
+        <v>3.59E-4</v>
       </c>
       <c r="I19" s="1">
         <v>0</v>
       </c>
       <c r="J19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>3.4099999999999999E-4</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>5.4199999999999995E-4</v>
       </c>
       <c r="M19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>3.7500000000000001E-4</v>
       </c>
       <c r="N19" s="1">
         <v>0</v>
@@ -2183,28 +2183,28 @@
         <v>0</v>
       </c>
       <c r="P19" s="1">
-        <v>0</v>
+        <v>8.8800000000000001E-4</v>
       </c>
       <c r="Q19" s="1">
-        <v>0.13683200000000001</v>
+        <v>9.3853000000000006E-2</v>
       </c>
       <c r="R19" s="1">
-        <v>1.598E-3</v>
+        <v>1.882E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>0.299433</v>
+        <v>0.451289</v>
       </c>
       <c r="T19" s="1">
-        <v>1.89E-3</v>
+        <v>2.5569999999999998E-3</v>
       </c>
       <c r="U19" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>1.0579999999999999E-3</v>
       </c>
       <c r="V19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>3.222E-3</v>
       </c>
       <c r="W19" s="1">
-        <v>0</v>
+        <v>3.1510000000000002E-3</v>
       </c>
       <c r="X19" s="1">
         <v>0</v>
@@ -2213,13 +2213,13 @@
         <v>0</v>
       </c>
       <c r="Z19" s="1">
-        <v>1.6257000000000001E-2</v>
+        <v>3.6332000000000003E-2</v>
       </c>
       <c r="AA19" s="1">
-        <v>0</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AB19" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AC19" s="1">
         <v>0</v>
@@ -2228,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>9.4490000000000008E-3</v>
+        <v>1.1811E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2243,19 +2243,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>2.0869999999999999E-3</v>
+        <v>2.3530000000000001E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="E20" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.6999999999999999E-4</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>3.7690000000000002E-3</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
@@ -2267,7 +2267,7 @@
         <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>0</v>
+        <v>6.4000000000000005E-4</v>
       </c>
       <c r="L20" s="1">
         <v>0</v>
@@ -2282,25 +2282,25 @@
         <v>0</v>
       </c>
       <c r="P20" s="1">
-        <v>0</v>
+        <v>8.9899999999999995E-4</v>
       </c>
       <c r="Q20" s="1">
         <v>0</v>
       </c>
       <c r="R20" s="1">
-        <v>0</v>
+        <v>4.0000000000000003E-5</v>
       </c>
       <c r="S20" s="1">
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>4.7636999999999999E-2</v>
+        <v>6.1135000000000002E-2</v>
       </c>
       <c r="U20" s="1">
         <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>1.3611E-2</v>
+        <v>1.2663000000000001E-2</v>
       </c>
       <c r="W20" s="1">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AB20" s="1">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>0</v>
+        <v>1.078E-3</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2339,25 +2339,25 @@
         <v>0</v>
       </c>
       <c r="B21" s="1">
-        <v>0</v>
+        <v>3.8999999999999999E-5</v>
       </c>
       <c r="C21" s="1">
         <v>0</v>
       </c>
       <c r="D21" s="1">
-        <v>0</v>
+        <v>3.6499999999999998E-4</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>1.1329999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="G21" s="1">
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="I21" s="1">
         <v>0</v>
@@ -2384,7 +2384,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="1">
-        <v>2.441E-3</v>
+        <v>0</v>
       </c>
       <c r="R21" s="1">
         <v>0</v>
@@ -2393,16 +2393,16 @@
         <v>0</v>
       </c>
       <c r="T21" s="1">
-        <v>0</v>
+        <v>1.702E-3</v>
       </c>
       <c r="U21" s="1">
-        <v>7.9399999999999991E-3</v>
+        <v>1.95E-2</v>
       </c>
       <c r="V21" s="1">
-        <v>0</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W21" s="1">
-        <v>4.9150000000000001E-3</v>
+        <v>5.9589999999999999E-3</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="AB21" s="1">
-        <v>0</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AC21" s="1">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>3.0240000000000002E-3</v>
+        <v>2.1489999999999999E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2444,10 +2444,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="E22" s="1">
-        <v>0</v>
+        <v>1.8599999999999999E-4</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
@@ -2459,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>1.3669999999999999E-3</v>
       </c>
       <c r="J22" s="1">
         <v>0</v>
@@ -2492,16 +2492,16 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>1.954E-3</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>7.1830000000000001E-3</v>
+        <v>1.1110999999999999E-2</v>
       </c>
       <c r="W22" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="X22" s="1">
         <v>0</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="1">
-        <v>1.5120000000000001E-3</v>
+        <v>9.990000000000001E-4</v>
       </c>
       <c r="AB22" s="1">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="1">
-        <v>0</v>
+        <v>7.1900000000000002E-4</v>
       </c>
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
@@ -2588,19 +2588,19 @@
         <v>0</v>
       </c>
       <c r="S23" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="T23" s="1">
         <v>0</v>
       </c>
       <c r="U23" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="V23" s="1">
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>2.2680000000000001E-3</v>
+        <v>1.8270000000000001E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>1.134E-3</v>
+        <v>1.7769999999999999E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2738,13 +2738,13 @@
         <v>0</v>
       </c>
       <c r="C25" s="1">
-        <v>1.3320000000000001E-3</v>
+        <v>5.3999999999999998E-5</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>1.5100000000000001E-3</v>
+        <v>1.872E-3</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>3.4099999999999999E-4</v>
       </c>
       <c r="L25" s="1">
         <v>0</v>
@@ -2777,13 +2777,13 @@
         <v>0</v>
       </c>
       <c r="P25" s="1">
-        <v>6.1600000000000001E-4</v>
+        <v>4.3800000000000002E-4</v>
       </c>
       <c r="Q25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>1.3166000000000001E-2</v>
+        <v>5.764E-3</v>
       </c>
       <c r="S25" s="1">
         <v>0</v>
@@ -2795,7 +2795,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="1">
-        <v>0</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W25" s="1">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="1">
-        <v>7.561E-3</v>
+        <v>9.0460000000000002E-3</v>
       </c>
       <c r="Z25" s="1">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="1">
-        <v>4.9150000000000001E-3</v>
+        <v>4.6709999999999998E-3</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2837,16 +2837,16 @@
         <v>0</v>
       </c>
       <c r="C26" s="1">
-        <v>0</v>
+        <v>9.9500000000000001E-4</v>
       </c>
       <c r="D26" s="1">
         <v>0</v>
       </c>
       <c r="E26" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>7.5500000000000003E-4</v>
+        <v>1.547E-3</v>
       </c>
       <c r="G26" s="1">
         <v>0</v>
@@ -2858,19 +2858,19 @@
         <v>0</v>
       </c>
       <c r="J26" s="1">
-        <v>0</v>
+        <v>3.4099999999999999E-4</v>
       </c>
       <c r="K26" s="1">
         <v>0</v>
       </c>
       <c r="L26" s="1">
-        <v>0</v>
+        <v>1.1820000000000001E-3</v>
       </c>
       <c r="M26" s="1">
         <v>0</v>
       </c>
       <c r="N26" s="1">
-        <v>0</v>
+        <v>2.3499999999999999E-4</v>
       </c>
       <c r="O26" s="1">
         <v>0</v>
@@ -2879,22 +2879,22 @@
         <v>0</v>
       </c>
       <c r="Q26" s="1">
-        <v>1.977E-3</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="R26" s="1">
-        <v>0</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="S26" s="1">
-        <v>7.561E-3</v>
+        <v>9.0930000000000004E-3</v>
       </c>
       <c r="T26" s="1">
-        <v>7.5600000000000005E-4</v>
+        <v>0</v>
       </c>
       <c r="U26" s="1">
         <v>0</v>
       </c>
       <c r="V26" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="W26" s="1">
         <v>0</v>
@@ -2906,7 +2906,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="1">
-        <v>4.9150000000000001E-3</v>
+        <v>7.5189999999999996E-3</v>
       </c>
       <c r="AA26" s="1">
         <v>0</v>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>3.4030000000000002E-3</v>
+        <v>3.2269999999999998E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -3008,7 +3008,7 @@
         <v>0</v>
       </c>
       <c r="AA27" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AB27" s="1">
         <v>0</v>
@@ -3092,7 +3092,7 @@
         <v>0</v>
       </c>
       <c r="V28" s="1">
-        <v>0</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W28" s="1">
         <v>0</v>
@@ -3110,16 +3110,16 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>6.4270000000000004E-3</v>
+        <v>3.3470000000000001E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
       </c>
       <c r="AD28" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AE28" s="1">
-        <v>0</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="AF28" s="1"/>
       <c r="AG28" s="1"/>
@@ -3212,13 +3212,13 @@
         <v>0</v>
       </c>
       <c r="AC29" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AD29" s="1">
         <v>0</v>
       </c>
       <c r="AE29" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>3.5300000000000002E-4</v>
       </c>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="AB30" s="1">
-        <v>3.7800000000000003E-4</v>
+        <v>0</v>
       </c>
       <c r="AC30" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
add non-physical PID checker/drawer
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{132C67F4-B31D-4808-9377-494EDA46E597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2930D254-8559-4ACD-BD02-CC42AA91FB94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,25 +356,25 @@
   <sheetData>
     <row r="1" spans="1:35">
       <c r="A1" s="1">
-        <v>9.921913</v>
+        <v>11.632858000000001</v>
       </c>
       <c r="B1" s="1">
-        <v>1.993042</v>
+        <v>3.0487649999999999</v>
       </c>
       <c r="C1" s="1">
-        <v>8.0480999999999997E-2</v>
+        <v>0.152229</v>
       </c>
       <c r="D1" s="1">
-        <v>3.3762E-2</v>
+        <v>6.0838000000000003E-2</v>
       </c>
       <c r="E1" s="1">
-        <v>1.0442E-2</v>
+        <v>2.2849999999999999E-2</v>
       </c>
       <c r="F1" s="1">
-        <v>1.8780999999999999E-2</v>
+        <v>4.1363999999999998E-2</v>
       </c>
       <c r="G1" s="1">
-        <v>0</v>
+        <v>1.18E-4</v>
       </c>
       <c r="H1" s="1">
         <v>0</v>
@@ -383,46 +383,46 @@
         <v>0</v>
       </c>
       <c r="J1" s="1">
-        <v>4.8607999999999998E-2</v>
+        <v>9.9738999999999994E-2</v>
       </c>
       <c r="K1" s="1">
-        <v>1.1820000000000001E-3</v>
+        <v>1.186E-3</v>
       </c>
       <c r="L1" s="1">
-        <v>1.621E-3</v>
+        <v>3.797E-3</v>
       </c>
       <c r="M1" s="1">
-        <v>1.1969999999999999E-3</v>
+        <v>2.166E-3</v>
       </c>
       <c r="N1" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="O1" s="1">
         <v>0</v>
       </c>
       <c r="P1" s="1">
-        <v>8.7900000000000001E-4</v>
+        <v>1.3129999999999999E-3</v>
       </c>
       <c r="Q1" s="1">
-        <v>0.358987</v>
+        <v>0.55441200000000002</v>
       </c>
       <c r="R1" s="1">
-        <v>8.7299999999999997E-4</v>
+        <v>2.0969999999999999E-3</v>
       </c>
       <c r="S1" s="1">
-        <v>4.0078000000000003E-2</v>
+        <v>8.3446999999999993E-2</v>
       </c>
       <c r="T1" s="1">
-        <v>3.7199999999999999E-4</v>
+        <v>2.2820000000000002E-3</v>
       </c>
       <c r="U1" s="1">
-        <v>9.3800000000000003E-4</v>
+        <v>3.7390000000000001E-3</v>
       </c>
       <c r="V1" s="1">
-        <v>4.4000000000000002E-4</v>
+        <v>1.8240000000000001E-3</v>
       </c>
       <c r="W1" s="1">
-        <v>0</v>
+        <v>3.6400000000000001E-4</v>
       </c>
       <c r="X1" s="1">
         <v>0</v>
@@ -431,22 +431,22 @@
         <v>0</v>
       </c>
       <c r="Z1" s="1">
-        <v>6.9399999999999996E-4</v>
+        <v>5.1240000000000001E-3</v>
       </c>
       <c r="AA1" s="1">
         <v>0</v>
       </c>
       <c r="AB1" s="1">
-        <v>0</v>
+        <v>8.3500000000000002E-4</v>
       </c>
       <c r="AC1" s="1">
         <v>0</v>
       </c>
       <c r="AD1" s="1">
-        <v>0</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AE1" s="1">
-        <v>0.15743799999999999</v>
+        <v>0.32191700000000001</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -455,22 +455,22 @@
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="1">
-        <v>0.23813999999999999</v>
+        <v>0.34477999999999998</v>
       </c>
       <c r="B2" s="1">
-        <v>1.713425</v>
+        <v>2.651691</v>
       </c>
       <c r="C2" s="1">
-        <v>1.4224000000000001E-2</v>
+        <v>3.6687999999999998E-2</v>
       </c>
       <c r="D2" s="1">
-        <v>2.8939999999999999E-3</v>
+        <v>1.0817999999999999E-2</v>
       </c>
       <c r="E2" s="1">
-        <v>9.7179999999999992E-3</v>
+        <v>2.6793000000000001E-2</v>
       </c>
       <c r="F2" s="1">
-        <v>1.1943E-2</v>
+        <v>3.7034999999999998E-2</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
@@ -482,19 +482,19 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>0.108473</v>
+        <v>0.22554299999999999</v>
       </c>
       <c r="K2" s="1">
-        <v>5.4199999999999995E-4</v>
+        <v>5.44E-4</v>
       </c>
       <c r="L2" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>3.8210000000000002E-3</v>
       </c>
       <c r="M2" s="1">
-        <v>0</v>
+        <v>7.5199999999999996E-4</v>
       </c>
       <c r="N2" s="1">
-        <v>0</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="O2" s="1">
         <v>0</v>
@@ -503,25 +503,25 @@
         <v>0</v>
       </c>
       <c r="Q2" s="1">
-        <v>3.1519999999999999E-2</v>
+        <v>6.0588000000000003E-2</v>
       </c>
       <c r="R2" s="1">
         <v>0</v>
       </c>
       <c r="S2" s="1">
-        <v>6.2542E-2</v>
+        <v>0.106918</v>
       </c>
       <c r="T2" s="1">
-        <v>8.5099999999999998E-4</v>
+        <v>4.7800000000000002E-4</v>
       </c>
       <c r="U2" s="1">
         <v>0</v>
       </c>
       <c r="V2" s="1">
-        <v>0</v>
+        <v>5.9900000000000003E-4</v>
       </c>
       <c r="W2" s="1">
-        <v>0</v>
+        <v>2.9500000000000001E-4</v>
       </c>
       <c r="X2" s="1">
         <v>0</v>
@@ -530,13 +530,13 @@
         <v>0</v>
       </c>
       <c r="Z2" s="1">
-        <v>2.5920000000000001E-3</v>
+        <v>8.2760000000000004E-3</v>
       </c>
       <c r="AA2" s="1">
-        <v>0</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="AB2" s="1">
-        <v>0</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AC2" s="1">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="1">
-        <v>6.9095000000000004E-2</v>
+        <v>0.161357</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -554,37 +554,37 @@
     </row>
     <row r="3" spans="1:35">
       <c r="A3" s="1">
-        <v>1E-3</v>
+        <v>1.505E-3</v>
       </c>
       <c r="B3" s="1">
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>0.92485399999999995</v>
+        <v>1.4794830000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>9.9200000000000004E-4</v>
+        <v>1.8220000000000001E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>9.0979000000000004E-2</v>
+        <v>0.216921</v>
       </c>
       <c r="F3" s="1">
-        <v>6.8300000000000001E-4</v>
+        <v>1.3699999999999999E-3</v>
       </c>
       <c r="G3" s="1">
-        <v>2.1940000000000002E-3</v>
+        <v>4.3709999999999999E-3</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>3.59E-4</v>
+        <v>7.2000000000000005E-4</v>
       </c>
       <c r="J3" s="1">
         <v>0</v>
       </c>
       <c r="K3" s="1">
-        <v>5.2449999999999997E-3</v>
+        <v>1.2172000000000001E-2</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -599,25 +599,25 @@
         <v>0</v>
       </c>
       <c r="P3" s="1">
-        <v>3.5639999999999999E-3</v>
+        <v>7.5269999999999998E-3</v>
       </c>
       <c r="Q3" s="1">
-        <v>1.106E-3</v>
+        <v>3.0179999999999998E-3</v>
       </c>
       <c r="R3" s="1">
-        <v>1.76E-4</v>
+        <v>3.0279999999999999E-3</v>
       </c>
       <c r="S3" s="1">
         <v>0</v>
       </c>
       <c r="T3" s="1">
-        <v>1.1568E-2</v>
+        <v>2.5527999999999999E-2</v>
       </c>
       <c r="U3" s="1">
-        <v>0</v>
+        <v>1.021E-3</v>
       </c>
       <c r="V3" s="1">
-        <v>1.8309999999999999E-3</v>
+        <v>5.7270000000000003E-3</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
@@ -632,10 +632,10 @@
         <v>0</v>
       </c>
       <c r="AA3" s="1">
-        <v>0</v>
+        <v>1.645E-3</v>
       </c>
       <c r="AB3" s="1">
-        <v>0</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AC3" s="1">
         <v>0</v>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="1">
-        <v>2.4819999999999998E-3</v>
+        <v>1.0984000000000001E-2</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -653,28 +653,28 @@
     </row>
     <row r="4" spans="1:35">
       <c r="A4" s="1">
-        <v>0</v>
+        <v>5.0100000000000003E-4</v>
       </c>
       <c r="B4" s="1">
-        <v>1.168E-3</v>
+        <v>2.6589999999999999E-3</v>
       </c>
       <c r="C4" s="1">
-        <v>2.41E-4</v>
+        <v>2.0790000000000001E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>0.53972600000000004</v>
+        <v>0.81034200000000001</v>
       </c>
       <c r="E4" s="1">
-        <v>0</v>
+        <v>3.7199999999999999E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>0.169936</v>
+        <v>0.32391799999999998</v>
       </c>
       <c r="G4" s="1">
-        <v>1.0059999999999999E-3</v>
+        <v>2.9429999999999999E-3</v>
       </c>
       <c r="H4" s="1">
-        <v>5.8200000000000005E-4</v>
+        <v>1.122E-3</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
@@ -686,7 +686,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="1">
-        <v>1.2200000000000001E-2</v>
+        <v>1.7492000000000001E-2</v>
       </c>
       <c r="M4" s="1">
         <v>0</v>
@@ -701,25 +701,25 @@
         <v>0</v>
       </c>
       <c r="Q4" s="1">
-        <v>1.4555999999999999E-2</v>
+        <v>2.8833999999999999E-2</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>5.3429999999999997E-3</v>
+        <v>9.8639999999999995E-3</v>
       </c>
       <c r="T4" s="1">
-        <v>7.4299999999999995E-4</v>
+        <v>1.2179999999999999E-3</v>
       </c>
       <c r="U4" s="1">
-        <v>9.0950000000000007E-3</v>
+        <v>2.2223E-2</v>
       </c>
       <c r="V4" s="1">
-        <v>0</v>
+        <v>6.9300000000000004E-4</v>
       </c>
       <c r="W4" s="1">
-        <v>2.124E-3</v>
+        <v>6.0489999999999997E-3</v>
       </c>
       <c r="X4" s="1">
         <v>0</v>
@@ -728,13 +728,13 @@
         <v>0</v>
       </c>
       <c r="Z4" s="1">
-        <v>6.5200000000000002E-4</v>
+        <v>6.4999999999999997E-4</v>
       </c>
       <c r="AA4" s="1">
         <v>0</v>
       </c>
       <c r="AB4" s="1">
-        <v>0</v>
+        <v>3.8000000000000002E-4</v>
       </c>
       <c r="AC4" s="1">
         <v>0</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="1">
-        <v>1.2005999999999999E-2</v>
+        <v>2.5862E-2</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -758,34 +758,34 @@
         <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>3.5987999999999999E-2</v>
+        <v>6.0587000000000002E-2</v>
       </c>
       <c r="D5" s="1">
-        <v>0</v>
+        <v>3.6600000000000001E-4</v>
       </c>
       <c r="E5" s="1">
-        <v>0.144652</v>
+        <v>0.26051800000000003</v>
       </c>
       <c r="F5" s="1">
-        <v>4.3199999999999998E-4</v>
+        <v>4.3399999999999998E-4</v>
       </c>
       <c r="G5" s="1">
-        <v>1.0380000000000001E-3</v>
+        <v>1.9659999999999999E-3</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>3.59E-4</v>
+        <v>1.4400000000000001E-3</v>
       </c>
       <c r="J5" s="1">
         <v>0</v>
       </c>
       <c r="K5" s="1">
-        <v>1.0409E-2</v>
+        <v>1.9961E-2</v>
       </c>
       <c r="L5" s="1">
-        <v>6.4000000000000005E-4</v>
+        <v>6.4199999999999999E-4</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
@@ -800,22 +800,22 @@
         <v>0</v>
       </c>
       <c r="Q5" s="1">
-        <v>9.2800000000000001E-4</v>
+        <v>9.2400000000000002E-4</v>
       </c>
       <c r="R5" s="1">
-        <v>2.1050000000000001E-3</v>
+        <v>3.3249999999999998E-3</v>
       </c>
       <c r="S5" s="1">
-        <v>0</v>
+        <v>3.7500000000000001E-4</v>
       </c>
       <c r="T5" s="1">
-        <v>2.529E-3</v>
+        <v>3.4749999999999998E-3</v>
       </c>
       <c r="U5" s="1">
         <v>0</v>
       </c>
       <c r="V5" s="1">
-        <v>3.6619999999999999E-3</v>
+        <v>9.3729999999999994E-3</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
@@ -824,13 +824,13 @@
         <v>0</v>
       </c>
       <c r="Y5" s="1">
-        <v>0</v>
+        <v>6.9200000000000002E-4</v>
       </c>
       <c r="Z5" s="1">
         <v>0</v>
       </c>
       <c r="AA5" s="1">
-        <v>3.4699999999999998E-4</v>
+        <v>1.5460000000000001E-3</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
@@ -842,7 +842,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="1">
-        <v>2.8219999999999999E-3</v>
+        <v>8.5070000000000007E-3</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -860,13 +860,13 @@
         <v>1.21E-4</v>
       </c>
       <c r="D6" s="1">
-        <v>1.5311E-2</v>
+        <v>2.4680000000000001E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>1.5020000000000001E-3</v>
+        <v>1.5070000000000001E-3</v>
       </c>
       <c r="F6" s="1">
-        <v>9.6351000000000006E-2</v>
+        <v>0.15723000000000001</v>
       </c>
       <c r="G6" s="1">
         <v>0</v>
@@ -875,7 +875,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>0</v>
+        <v>3.6000000000000002E-4</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
@@ -884,10 +884,10 @@
         <v>0</v>
       </c>
       <c r="L6" s="1">
-        <v>1.0189999999999999E-2</v>
+        <v>2.8459000000000002E-2</v>
       </c>
       <c r="M6" s="1">
-        <v>3.7500000000000001E-4</v>
+        <v>3.7599999999999998E-4</v>
       </c>
       <c r="N6" s="1">
         <v>0</v>
@@ -905,19 +905,19 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>2.2950000000000002E-3</v>
+        <v>3.6129999999999999E-3</v>
       </c>
       <c r="T6" s="1">
         <v>0</v>
       </c>
       <c r="U6" s="1">
-        <v>1.0579999999999999E-3</v>
+        <v>1.173E-3</v>
       </c>
       <c r="V6" s="1">
         <v>0</v>
       </c>
       <c r="W6" s="1">
-        <v>9.5799999999999998E-4</v>
+        <v>1.614E-3</v>
       </c>
       <c r="X6" s="1">
         <v>0</v>
@@ -926,10 +926,10 @@
         <v>0</v>
       </c>
       <c r="Z6" s="1">
-        <v>1.204E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="AA6" s="1">
-        <v>6.5200000000000002E-4</v>
+        <v>6.4999999999999997E-4</v>
       </c>
       <c r="AB6" s="1">
         <v>0</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="1">
-        <v>6.7149999999999996E-3</v>
+        <v>1.3469999999999999E-2</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -956,7 +956,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
@@ -968,13 +968,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <v>2.3119999999999998E-3</v>
+        <v>7.058E-3</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>1.4350000000000001E-3</v>
+        <v>2.4060000000000002E-3</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
@@ -1013,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="V7" s="1">
-        <v>0</v>
+        <v>1.8240000000000001E-3</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v>0</v>
       </c>
       <c r="AE7" s="1">
-        <v>3.59E-4</v>
+        <v>1.42E-3</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
@@ -1070,7 +1070,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <v>7.18E-4</v>
+        <v>1.4400000000000001E-3</v>
       </c>
       <c r="I8" s="1">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="1">
-        <v>0</v>
+        <v>7.1199999999999996E-4</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1172,7 +1172,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>3.59E-4</v>
+        <v>1.08E-3</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
@@ -1238,7 +1238,7 @@
         <v>0</v>
       </c>
       <c r="AE9" s="1">
-        <v>0</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="AF9" s="1"/>
       <c r="AG9" s="1"/>
@@ -1247,22 +1247,22 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="1">
-        <v>4.0299999999999997E-3</v>
+        <v>7.6270000000000001E-3</v>
       </c>
       <c r="B10" s="1">
-        <v>4.5633E-2</v>
+        <v>7.9524999999999998E-2</v>
       </c>
       <c r="C10" s="1">
-        <v>5.9400000000000002E-4</v>
+        <v>2.7690000000000002E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>4.7100000000000001E-4</v>
+        <v>1.0889999999999999E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>4.0679999999999996E-3</v>
+        <v>1.0656000000000001E-2</v>
       </c>
       <c r="F10" s="1">
-        <v>1.3649999999999999E-3</v>
+        <v>5.8209999999999998E-3</v>
       </c>
       <c r="G10" s="1">
         <v>0</v>
@@ -1274,19 +1274,19 @@
         <v>0</v>
       </c>
       <c r="J10" s="1">
-        <v>5.7117000000000001E-2</v>
+        <v>8.8736999999999996E-2</v>
       </c>
       <c r="K10" s="1">
-        <v>6.4000000000000005E-4</v>
+        <v>1.186E-3</v>
       </c>
       <c r="L10" s="1">
-        <v>5.4199999999999995E-4</v>
+        <v>2.4710000000000001E-3</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>0</v>
+        <v>2.3599999999999999E-4</v>
       </c>
       <c r="O10" s="1">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="1">
-        <v>1.745E-3</v>
+        <v>4.4580000000000002E-3</v>
       </c>
       <c r="R10" s="1">
-        <v>0</v>
+        <v>3.9800000000000002E-4</v>
       </c>
       <c r="S10" s="1">
-        <v>4.9550000000000002E-3</v>
+        <v>7.9170000000000004E-3</v>
       </c>
       <c r="T10" s="1">
         <v>0</v>
@@ -1313,7 +1313,7 @@
         <v>0</v>
       </c>
       <c r="W10" s="1">
-        <v>0</v>
+        <v>2.4899999999999998E-4</v>
       </c>
       <c r="X10" s="1">
         <v>0</v>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="1">
-        <v>3.4699999999999998E-4</v>
+        <v>1.645E-3</v>
       </c>
       <c r="AA10" s="1">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="1">
-        <v>2.9277999999999998E-2</v>
+        <v>7.0454000000000003E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1352,16 +1352,16 @@
         <v>0</v>
       </c>
       <c r="C11" s="1">
-        <v>1.116E-3</v>
+        <v>1.1199999999999999E-3</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>1.872E-3</v>
+        <v>7.1419999999999999E-3</v>
       </c>
       <c r="F11" s="1">
-        <v>0</v>
+        <v>6.8499999999999995E-4</v>
       </c>
       <c r="G11" s="1">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <v>1.2800000000000001E-3</v>
+        <v>5.1380000000000002E-3</v>
       </c>
       <c r="L11" s="1">
         <v>0</v>
@@ -1391,7 +1391,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="1">
-        <v>0</v>
+        <v>4.4999999999999999E-4</v>
       </c>
       <c r="Q11" s="1">
         <v>0</v>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="1">
-        <v>6.9499999999999998E-4</v>
+        <v>6.9300000000000004E-4</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="1">
-        <v>0</v>
+        <v>5.5000000000000003E-4</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
@@ -1436,7 +1436,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="1">
-        <v>7.0500000000000001E-4</v>
+        <v>1.7700000000000001E-3</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1460,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>1.797E-3</v>
+        <v>4.7260000000000002E-3</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
@@ -1478,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="1">
-        <v>6.4000000000000005E-4</v>
+        <v>1.2849999999999999E-3</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
@@ -1505,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="U12" s="1">
-        <v>0</v>
+        <v>1.1900000000000001E-4</v>
       </c>
       <c r="V12" s="1">
         <v>0</v>
@@ -1535,7 +1535,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="1">
-        <v>1.4109999999999999E-3</v>
+        <v>2.1280000000000001E-3</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
@@ -1553,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="1">
-        <v>1.3060000000000001E-3</v>
+        <v>1.3110000000000001E-3</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="1">
-        <v>2.8874E-2</v>
+        <v>4.5222999999999999E-2</v>
       </c>
       <c r="N13" s="1">
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>2.7669999999999999E-3</v>
+        <v>5.8110000000000002E-3</v>
       </c>
       <c r="P13" s="1">
         <v>0</v>
@@ -1628,13 +1628,13 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>2.3900000000000001E-4</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AD13" s="1">
         <v>0</v>
       </c>
       <c r="AE13" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
@@ -1682,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>0</v>
+        <v>9.4200000000000002E-4</v>
       </c>
       <c r="O14" s="1">
         <v>0</v>
@@ -1778,13 +1778,13 @@
         <v>0</v>
       </c>
       <c r="M15" s="1">
-        <v>4.6900000000000002E-4</v>
+        <v>9.4200000000000002E-4</v>
       </c>
       <c r="N15" s="1">
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>7.0399999999999998E-4</v>
+        <v>7.0699999999999995E-4</v>
       </c>
       <c r="P15" s="1">
         <v>0</v>
@@ -1826,13 +1826,13 @@
         <v>0</v>
       </c>
       <c r="AC15" s="1">
-        <v>2.3900000000000001E-4</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AD15" s="1">
         <v>0</v>
       </c>
       <c r="AE15" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>7.1199999999999996E-4</v>
       </c>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1"/>
@@ -1844,16 +1844,16 @@
         <v>0</v>
       </c>
       <c r="B16" s="1">
-        <v>9.9500000000000001E-4</v>
+        <v>9.990000000000001E-4</v>
       </c>
       <c r="C16" s="1">
-        <v>6.9081000000000004E-2</v>
+        <v>0.12876099999999999</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" s="1">
-        <v>6.6969999999999998E-3</v>
+        <v>1.268E-2</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -1865,13 +1865,13 @@
         <v>0</v>
       </c>
       <c r="I16" s="1">
-        <v>2.9100000000000003E-4</v>
+        <v>2.92E-4</v>
       </c>
       <c r="J16" s="1">
         <v>0</v>
       </c>
       <c r="K16" s="1">
-        <v>0</v>
+        <v>8.8599999999999996E-4</v>
       </c>
       <c r="L16" s="1">
         <v>0</v>
@@ -1886,25 +1886,25 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>0.87813799999999997</v>
+        <v>1.163289</v>
       </c>
       <c r="Q16" s="1">
-        <v>1.119E-3</v>
+        <v>3.1540000000000001E-3</v>
       </c>
       <c r="R16" s="1">
-        <v>0.105959</v>
+        <v>0.21071100000000001</v>
       </c>
       <c r="S16" s="1">
-        <v>0</v>
+        <v>3.5799999999999997E-4</v>
       </c>
       <c r="T16" s="1">
-        <v>3.7520000000000001E-3</v>
+        <v>7.241E-3</v>
       </c>
       <c r="U16" s="1">
         <v>0</v>
       </c>
       <c r="V16" s="1">
-        <v>1.8309999999999999E-3</v>
+        <v>3.117E-3</v>
       </c>
       <c r="W16" s="1">
         <v>0</v>
@@ -1913,10 +1913,10 @@
         <v>0</v>
       </c>
       <c r="Y16" s="1">
-        <v>1.346E-3</v>
+        <v>5.3899999999999998E-3</v>
       </c>
       <c r="Z16" s="1">
-        <v>0</v>
+        <v>6.4999999999999997E-4</v>
       </c>
       <c r="AA16" s="1">
         <v>0</v>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="1">
-        <v>5.3889999999999997E-3</v>
+        <v>2.1118999999999999E-2</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1940,73 +1940,73 @@
     </row>
     <row r="17" spans="1:35">
       <c r="A17" s="1">
-        <v>1.1169E-2</v>
+        <v>1.5751000000000001E-2</v>
       </c>
       <c r="B17" s="1">
-        <v>8.3859999999999994E-3</v>
+        <v>1.5212E-2</v>
       </c>
       <c r="C17" s="1">
-        <v>3.6879999999999999E-3</v>
+        <v>7.1580000000000003E-3</v>
       </c>
       <c r="D17" s="1">
-        <v>5.6411000000000003E-2</v>
+        <v>9.6978999999999996E-2</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
+        <v>3.7100000000000002E-4</v>
       </c>
       <c r="F17" s="1">
-        <v>1.721E-2</v>
+        <v>4.3985999999999997E-2</v>
       </c>
       <c r="G17" s="1">
+        <v>1.934E-3</v>
+      </c>
+      <c r="H17" s="1">
+        <v>0</v>
+      </c>
+      <c r="I17" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1">
+        <v>6.4199999999999999E-4</v>
+      </c>
+      <c r="K17" s="1">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1">
+        <v>2.31E-3</v>
+      </c>
+      <c r="M17" s="1">
+        <v>4.7100000000000001E-4</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
+        <v>0</v>
+      </c>
+      <c r="P17" s="1">
+        <v>7.0340000000000003E-3</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>3.3522599999999998</v>
+      </c>
+      <c r="R17" s="1">
         <v>1.0059999999999999E-3</v>
       </c>
-      <c r="H17" s="1">
-        <v>0</v>
-      </c>
-      <c r="I17" s="1">
-        <v>0</v>
-      </c>
-      <c r="J17" s="1">
-        <v>0</v>
-      </c>
-      <c r="K17" s="1">
-        <v>0</v>
-      </c>
-      <c r="L17" s="1">
-        <v>6.4000000000000005E-4</v>
-      </c>
-      <c r="M17" s="1">
-        <v>2.3499999999999999E-4</v>
-      </c>
-      <c r="N17" s="1">
-        <v>0</v>
-      </c>
-      <c r="O17" s="1">
-        <v>0</v>
-      </c>
-      <c r="P17" s="1">
-        <v>3.5230000000000001E-3</v>
-      </c>
-      <c r="Q17" s="1">
-        <v>2.3540679999999998</v>
-      </c>
-      <c r="R17" s="1">
-        <v>8.7299999999999997E-4</v>
-      </c>
       <c r="S17" s="1">
-        <v>0.33002900000000002</v>
+        <v>0.59404599999999996</v>
       </c>
       <c r="T17" s="1">
-        <v>7.9120000000000006E-3</v>
+        <v>1.8009000000000001E-2</v>
       </c>
       <c r="U17" s="1">
-        <v>2.9880000000000002E-3</v>
+        <v>7.9959999999999996E-3</v>
       </c>
       <c r="V17" s="1">
-        <v>6.02E-4</v>
+        <v>2.6779999999999998E-3</v>
       </c>
       <c r="W17" s="1">
-        <v>3.59E-4</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2015,22 +2015,22 @@
         <v>0</v>
       </c>
       <c r="Z17" s="1">
-        <v>7.9559999999999995E-3</v>
+        <v>2.3429999999999999E-2</v>
       </c>
       <c r="AA17" s="1">
         <v>0</v>
       </c>
       <c r="AB17" s="1">
-        <v>7.4100000000000001E-4</v>
+        <v>1.5950000000000001E-3</v>
       </c>
       <c r="AC17" s="1">
-        <v>0</v>
+        <v>3.8000000000000002E-4</v>
       </c>
       <c r="AD17" s="1">
-        <v>3.8200000000000002E-4</v>
+        <v>3.8000000000000002E-4</v>
       </c>
       <c r="AE17" s="1">
-        <v>7.5319999999999996E-3</v>
+        <v>2.3595999999999999E-2</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2042,16 +2042,16 @@
         <v>0</v>
       </c>
       <c r="B18" s="1">
-        <v>1.129E-3</v>
+        <v>1.1720000000000001E-3</v>
       </c>
       <c r="C18" s="1">
-        <v>9.0720000000000002E-3</v>
+        <v>1.6025000000000001E-2</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
       </c>
       <c r="E18" s="1">
-        <v>2.1701000000000002E-2</v>
+        <v>4.0693E-2</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2066,10 +2066,10 @@
         <v>0</v>
       </c>
       <c r="J18" s="1">
-        <v>0</v>
+        <v>6.4199999999999999E-4</v>
       </c>
       <c r="K18" s="1">
-        <v>0</v>
+        <v>1.6260000000000001E-3</v>
       </c>
       <c r="L18" s="1">
         <v>0</v>
@@ -2084,25 +2084,25 @@
         <v>0</v>
       </c>
       <c r="P18" s="1">
-        <v>3.3656999999999999E-2</v>
+        <v>5.4786000000000001E-2</v>
       </c>
       <c r="Q18" s="1">
-        <v>0</v>
+        <v>5.5000000000000002E-5</v>
       </c>
       <c r="R18" s="1">
-        <v>0.19733999999999999</v>
+        <v>0.31938499999999997</v>
       </c>
       <c r="S18" s="1">
-        <v>1.5299999999999999E-3</v>
+        <v>3.0490000000000001E-3</v>
       </c>
       <c r="T18" s="1">
-        <v>8.5099999999999998E-4</v>
+        <v>1.2179999999999999E-3</v>
       </c>
       <c r="U18" s="1">
         <v>0</v>
       </c>
       <c r="V18" s="1">
-        <v>1.1360000000000001E-3</v>
+        <v>2.5170000000000001E-3</v>
       </c>
       <c r="W18" s="1">
         <v>0</v>
@@ -2111,7 +2111,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="1">
-        <v>1.6022000000000002E-2</v>
+        <v>3.1233E-2</v>
       </c>
       <c r="Z18" s="1">
         <v>0</v>
@@ -2129,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="1">
-        <v>7.5449999999999996E-3</v>
+        <v>2.1114000000000001E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2138,43 +2138,43 @@
     </row>
     <row r="19" spans="1:35">
       <c r="A19" s="1">
-        <v>0</v>
+        <v>5.0699999999999996E-4</v>
       </c>
       <c r="B19" s="1">
-        <v>5.2830000000000004E-3</v>
+        <v>7.6449999999999999E-3</v>
       </c>
       <c r="C19" s="1">
-        <v>1.116E-3</v>
+        <v>1.1199999999999999E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>1.2772E-2</v>
+        <v>2.2617000000000002E-2</v>
       </c>
       <c r="E19" s="1">
-        <v>1.8599999999999999E-4</v>
+        <v>9.2800000000000001E-4</v>
       </c>
       <c r="F19" s="1">
-        <v>2.7526999999999999E-2</v>
+        <v>4.5710000000000001E-2</v>
       </c>
       <c r="G19" s="1">
-        <v>2.7629999999999998E-3</v>
+        <v>2.7720000000000002E-3</v>
       </c>
       <c r="H19" s="1">
-        <v>3.59E-4</v>
+        <v>3.6000000000000002E-4</v>
       </c>
       <c r="I19" s="1">
-        <v>0</v>
+        <v>3.6000000000000002E-4</v>
       </c>
       <c r="J19" s="1">
-        <v>3.4099999999999999E-4</v>
+        <v>6.8400000000000004E-4</v>
       </c>
       <c r="K19" s="1">
         <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>5.4199999999999995E-4</v>
+        <v>4.653E-3</v>
       </c>
       <c r="M19" s="1">
-        <v>3.7500000000000001E-4</v>
+        <v>3.7599999999999998E-4</v>
       </c>
       <c r="N19" s="1">
         <v>0</v>
@@ -2183,28 +2183,28 @@
         <v>0</v>
       </c>
       <c r="P19" s="1">
-        <v>8.8800000000000001E-4</v>
+        <v>8.8500000000000004E-4</v>
       </c>
       <c r="Q19" s="1">
-        <v>9.3853000000000006E-2</v>
+        <v>0.133967</v>
       </c>
       <c r="R19" s="1">
-        <v>1.882E-3</v>
+        <v>3.0170000000000002E-3</v>
       </c>
       <c r="S19" s="1">
-        <v>0.451289</v>
+        <v>0.65218100000000001</v>
       </c>
       <c r="T19" s="1">
-        <v>2.5569999999999998E-3</v>
+        <v>5.4619999999999998E-3</v>
       </c>
       <c r="U19" s="1">
-        <v>1.0579999999999999E-3</v>
+        <v>4.0309999999999999E-3</v>
       </c>
       <c r="V19" s="1">
-        <v>3.222E-3</v>
+        <v>5.6340000000000001E-3</v>
       </c>
       <c r="W19" s="1">
-        <v>3.1510000000000002E-3</v>
+        <v>5.2370000000000003E-3</v>
       </c>
       <c r="X19" s="1">
         <v>0</v>
@@ -2213,22 +2213,22 @@
         <v>0</v>
       </c>
       <c r="Z19" s="1">
-        <v>3.6332000000000003E-2</v>
+        <v>5.9267E-2</v>
       </c>
       <c r="AA19" s="1">
-        <v>6.5200000000000002E-4</v>
+        <v>6.4999999999999997E-4</v>
       </c>
       <c r="AB19" s="1">
-        <v>0</v>
+        <v>4.7600000000000002E-4</v>
       </c>
       <c r="AC19" s="1">
-        <v>0</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AD19" s="1">
         <v>0</v>
       </c>
       <c r="AE19" s="1">
-        <v>1.1811E-2</v>
+        <v>2.6093999999999999E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2243,31 +2243,31 @@
         <v>0</v>
       </c>
       <c r="C20" s="1">
-        <v>2.3530000000000001E-3</v>
+        <v>5.4780000000000002E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>0</v>
+        <v>4.7199999999999998E-4</v>
       </c>
       <c r="E20" s="1">
-        <v>3.6999999999999999E-4</v>
+        <v>3.7100000000000002E-4</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1">
-        <v>3.7690000000000002E-3</v>
+        <v>9.6159999999999995E-3</v>
       </c>
       <c r="H20" s="1">
         <v>0</v>
       </c>
       <c r="I20" s="1">
-        <v>0</v>
+        <v>1.258E-3</v>
       </c>
       <c r="J20" s="1">
         <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>6.4000000000000005E-4</v>
+        <v>6.4199999999999999E-4</v>
       </c>
       <c r="L20" s="1">
         <v>0</v>
@@ -2282,28 +2282,28 @@
         <v>0</v>
       </c>
       <c r="P20" s="1">
-        <v>8.9899999999999995E-4</v>
+        <v>8.9599999999999999E-4</v>
       </c>
       <c r="Q20" s="1">
-        <v>0</v>
+        <v>8.7000000000000001E-4</v>
       </c>
       <c r="R20" s="1">
         <v>4.0000000000000003E-5</v>
       </c>
       <c r="S20" s="1">
-        <v>0</v>
+        <v>7.6199999999999998E-4</v>
       </c>
       <c r="T20" s="1">
-        <v>6.1135000000000002E-2</v>
+        <v>0.10109600000000001</v>
       </c>
       <c r="U20" s="1">
         <v>0</v>
       </c>
       <c r="V20" s="1">
-        <v>1.2663000000000001E-2</v>
+        <v>3.3466999999999997E-2</v>
       </c>
       <c r="W20" s="1">
-        <v>0</v>
+        <v>3.6400000000000001E-4</v>
       </c>
       <c r="X20" s="1">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="1">
-        <v>6.5200000000000002E-4</v>
+        <v>1.5460000000000001E-3</v>
       </c>
       <c r="AB20" s="1">
         <v>0</v>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="1">
-        <v>1.078E-3</v>
+        <v>2.5019999999999999E-3</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2345,19 +2345,19 @@
         <v>0</v>
       </c>
       <c r="D21" s="1">
-        <v>3.6499999999999998E-4</v>
+        <v>7.3200000000000001E-4</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>0</v>
+        <v>1.039E-3</v>
       </c>
       <c r="G21" s="1">
         <v>0</v>
       </c>
       <c r="H21" s="1">
-        <v>0</v>
+        <v>5.8399999999999999E-4</v>
       </c>
       <c r="I21" s="1">
         <v>0</v>
@@ -2390,19 +2390,19 @@
         <v>0</v>
       </c>
       <c r="S21" s="1">
-        <v>0</v>
+        <v>7.6199999999999998E-4</v>
       </c>
       <c r="T21" s="1">
-        <v>1.702E-3</v>
+        <v>2.5439999999999998E-3</v>
       </c>
       <c r="U21" s="1">
-        <v>1.95E-2</v>
+        <v>3.4374000000000002E-2</v>
       </c>
       <c r="V21" s="1">
-        <v>6.9499999999999998E-4</v>
+        <v>1.0510000000000001E-3</v>
       </c>
       <c r="W21" s="1">
-        <v>5.9589999999999999E-3</v>
+        <v>1.4074E-2</v>
       </c>
       <c r="X21" s="1">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="AB21" s="1">
-        <v>2.3900000000000001E-4</v>
+        <v>2.3800000000000001E-4</v>
       </c>
       <c r="AC21" s="1">
         <v>0</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="1">
-        <v>2.1489999999999999E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2453,13 +2453,13 @@
         <v>0</v>
       </c>
       <c r="G22" s="1">
-        <v>0</v>
+        <v>9.2400000000000002E-4</v>
       </c>
       <c r="H22" s="1">
         <v>0</v>
       </c>
       <c r="I22" s="1">
-        <v>1.3669999999999999E-3</v>
+        <v>2.0240000000000002E-3</v>
       </c>
       <c r="J22" s="1">
         <v>0</v>
@@ -2492,13 +2492,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>1.954E-3</v>
+        <v>2.7950000000000002E-3</v>
       </c>
       <c r="U22" s="1">
         <v>0</v>
       </c>
       <c r="V22" s="1">
-        <v>1.1110999999999999E-2</v>
+        <v>1.9140999999999998E-2</v>
       </c>
       <c r="W22" s="1">
         <v>0</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="1">
-        <v>9.990000000000001E-4</v>
+        <v>2.1949999999999999E-3</v>
       </c>
       <c r="AB22" s="1">
         <v>0</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="1">
-        <v>7.1900000000000002E-4</v>
+        <v>1.4319999999999999E-3</v>
       </c>
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
@@ -2543,7 +2543,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="1">
-        <v>0</v>
+        <v>4.7199999999999998E-4</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
@@ -2594,13 +2594,13 @@
         <v>0</v>
       </c>
       <c r="U23" s="1">
-        <v>0</v>
+        <v>1.1900000000000001E-4</v>
       </c>
       <c r="V23" s="1">
         <v>0</v>
       </c>
       <c r="W23" s="1">
-        <v>1.8270000000000001E-3</v>
+        <v>2.48E-3</v>
       </c>
       <c r="X23" s="1">
         <v>0</v>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="1">
-        <v>1.7769999999999999E-3</v>
+        <v>2.8479999999999998E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2738,13 +2738,13 @@
         <v>0</v>
       </c>
       <c r="C25" s="1">
-        <v>5.3999999999999998E-5</v>
+        <v>1.0529999999999999E-3</v>
       </c>
       <c r="D25" s="1">
         <v>0</v>
       </c>
       <c r="E25" s="1">
-        <v>1.872E-3</v>
+        <v>4.4990000000000004E-3</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>3.4099999999999999E-4</v>
+        <v>3.4200000000000002E-4</v>
       </c>
       <c r="L25" s="1">
         <v>0</v>
@@ -2777,13 +2777,13 @@
         <v>0</v>
       </c>
       <c r="P25" s="1">
-        <v>4.3800000000000002E-4</v>
+        <v>4.37E-4</v>
       </c>
       <c r="Q25" s="1">
         <v>0</v>
       </c>
       <c r="R25" s="1">
-        <v>5.764E-3</v>
+        <v>1.1273E-2</v>
       </c>
       <c r="S25" s="1">
         <v>0</v>
@@ -2795,7 +2795,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="1">
-        <v>6.9499999999999998E-4</v>
+        <v>2.4369999999999999E-3</v>
       </c>
       <c r="W25" s="1">
         <v>0</v>
@@ -2804,13 +2804,13 @@
         <v>0</v>
       </c>
       <c r="Y25" s="1">
-        <v>9.0460000000000002E-3</v>
+        <v>1.2662E-2</v>
       </c>
       <c r="Z25" s="1">
-        <v>0</v>
+        <v>3.5799999999999997E-4</v>
       </c>
       <c r="AA25" s="1">
-        <v>0</v>
+        <v>3.5799999999999997E-4</v>
       </c>
       <c r="AB25" s="1">
         <v>0</v>
@@ -2822,7 +2822,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="1">
-        <v>4.6709999999999998E-3</v>
+        <v>7.1520000000000004E-3</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2837,16 +2837,16 @@
         <v>0</v>
       </c>
       <c r="C26" s="1">
-        <v>9.9500000000000001E-4</v>
+        <v>9.990000000000001E-4</v>
       </c>
       <c r="D26" s="1">
-        <v>0</v>
+        <v>8.3799999999999999E-4</v>
       </c>
       <c r="E26" s="1">
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>1.547E-3</v>
+        <v>2.1450000000000002E-3</v>
       </c>
       <c r="G26" s="1">
         <v>0</v>
@@ -2858,19 +2858,19 @@
         <v>0</v>
       </c>
       <c r="J26" s="1">
-        <v>3.4099999999999999E-4</v>
+        <v>9.8400000000000007E-4</v>
       </c>
       <c r="K26" s="1">
         <v>0</v>
       </c>
       <c r="L26" s="1">
-        <v>1.1820000000000001E-3</v>
+        <v>1.186E-3</v>
       </c>
       <c r="M26" s="1">
         <v>0</v>
       </c>
       <c r="N26" s="1">
-        <v>2.3499999999999999E-4</v>
+        <v>2.3599999999999999E-4</v>
       </c>
       <c r="O26" s="1">
         <v>0</v>
@@ -2879,13 +2879,13 @@
         <v>0</v>
       </c>
       <c r="Q26" s="1">
-        <v>8.7299999999999997E-4</v>
+        <v>8.7000000000000001E-4</v>
       </c>
       <c r="R26" s="1">
-        <v>8.7299999999999997E-4</v>
+        <v>8.7000000000000001E-4</v>
       </c>
       <c r="S26" s="1">
-        <v>9.0930000000000004E-3</v>
+        <v>1.5879999999999998E-2</v>
       </c>
       <c r="T26" s="1">
         <v>0</v>
@@ -2894,10 +2894,10 @@
         <v>0</v>
       </c>
       <c r="V26" s="1">
-        <v>0</v>
+        <v>4.3899999999999999E-4</v>
       </c>
       <c r="W26" s="1">
-        <v>0</v>
+        <v>1.0920000000000001E-3</v>
       </c>
       <c r="X26" s="1">
         <v>0</v>
@@ -2906,7 +2906,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="1">
-        <v>7.5189999999999996E-3</v>
+        <v>1.1291000000000001E-2</v>
       </c>
       <c r="AA26" s="1">
         <v>0</v>
@@ -2921,7 +2921,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="1">
-        <v>3.2269999999999998E-3</v>
+        <v>6.0819999999999997E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -3008,7 +3008,7 @@
         <v>0</v>
       </c>
       <c r="AA27" s="1">
-        <v>6.5200000000000002E-4</v>
+        <v>6.4999999999999997E-4</v>
       </c>
       <c r="AB27" s="1">
         <v>0</v>
@@ -3068,7 +3068,7 @@
         <v>0</v>
       </c>
       <c r="N28" s="1">
-        <v>0</v>
+        <v>3.7599999999999998E-4</v>
       </c>
       <c r="O28" s="1">
         <v>0</v>
@@ -3086,13 +3086,13 @@
         <v>0</v>
       </c>
       <c r="T28" s="1">
-        <v>0</v>
+        <v>4.7800000000000002E-4</v>
       </c>
       <c r="U28" s="1">
         <v>0</v>
       </c>
       <c r="V28" s="1">
-        <v>6.9499999999999998E-4</v>
+        <v>6.9300000000000004E-4</v>
       </c>
       <c r="W28" s="1">
         <v>0</v>
@@ -3110,16 +3110,16 @@
         <v>0</v>
       </c>
       <c r="AB28" s="1">
-        <v>3.3470000000000001E-3</v>
+        <v>5.0029999999999996E-3</v>
       </c>
       <c r="AC28" s="1">
         <v>0</v>
       </c>
       <c r="AD28" s="1">
-        <v>0</v>
+        <v>3.8000000000000002E-4</v>
       </c>
       <c r="AE28" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>7.0799999999999997E-4</v>
       </c>
       <c r="AF28" s="1"/>
       <c r="AG28" s="1"/>
@@ -3164,7 +3164,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="1">
-        <v>0</v>
+        <v>2.3599999999999999E-4</v>
       </c>
       <c r="N29" s="1">
         <v>0</v>
@@ -3212,13 +3212,13 @@
         <v>0</v>
       </c>
       <c r="AC29" s="1">
-        <v>2.3900000000000001E-4</v>
+        <v>4.7600000000000002E-4</v>
       </c>
       <c r="AD29" s="1">
         <v>0</v>
       </c>
       <c r="AE29" s="1">
-        <v>3.5300000000000002E-4</v>
+        <v>3.5399999999999999E-4</v>
       </c>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>

</xml_diff>

<commit_message>
add FBDTTrain for RC check
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7834B1AA-7022-4E71-BB68-0FE5F9642E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB053617-7DF4-4122-BE4C-F7E78F574CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7810" yWindow="340" windowWidth="17790" windowHeight="14000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -358,25 +358,25 @@
   <sheetData>
     <row r="1" spans="1:35">
       <c r="A1" s="2">
-        <v>12.040509999999999</v>
+        <v>12.026999</v>
       </c>
       <c r="B1" s="2">
-        <v>3.4387840000000001</v>
+        <v>3.4237449999999998</v>
       </c>
       <c r="C1" s="2">
-        <v>0.179115</v>
+        <v>0.18410099999999999</v>
       </c>
       <c r="D1" s="2">
-        <v>7.2114999999999999E-2</v>
+        <v>7.1387000000000006E-2</v>
       </c>
       <c r="E1" s="2">
-        <v>3.3653000000000002E-2</v>
+        <v>3.1815000000000003E-2</v>
       </c>
       <c r="F1" s="2">
-        <v>5.5481000000000003E-2</v>
+        <v>5.5015000000000001E-2</v>
       </c>
       <c r="G1" s="2">
-        <v>1.036E-3</v>
+        <v>1.17E-4</v>
       </c>
       <c r="H1" s="2">
         <v>0</v>
@@ -385,7 +385,7 @@
         <v>0</v>
       </c>
       <c r="J1" s="2">
-        <v>0.119711</v>
+        <v>0.11765299999999999</v>
       </c>
       <c r="K1" s="2">
         <v>1.1789999999999999E-3</v>
@@ -397,31 +397,31 @@
         <v>2.3869999999999998E-3</v>
       </c>
       <c r="N1" s="2">
-        <v>3.5199999999999999E-4</v>
+        <v>7.2499999999999995E-4</v>
       </c>
       <c r="O1" s="2">
         <v>0</v>
       </c>
       <c r="P1" s="2">
-        <v>1.776E-3</v>
+        <v>1.3209999999999999E-3</v>
       </c>
       <c r="Q1" s="2">
-        <v>0.63344999999999996</v>
+        <v>0.63055600000000001</v>
       </c>
       <c r="R1" s="2">
         <v>3.4359999999999998E-3</v>
       </c>
       <c r="S1" s="2">
-        <v>0.112136</v>
+        <v>0.108932</v>
       </c>
       <c r="T1" s="2">
-        <v>3.4020000000000001E-3</v>
+        <v>3.0409999999999999E-3</v>
       </c>
       <c r="U1" s="2">
         <v>4.1229999999999999E-3</v>
       </c>
       <c r="V1" s="2">
-        <v>1.836E-3</v>
+        <v>2.2769999999999999E-3</v>
       </c>
       <c r="W1" s="2">
         <v>3.6600000000000001E-4</v>
@@ -448,7 +448,7 @@
         <v>2.4000000000000001E-4</v>
       </c>
       <c r="AE1" s="2">
-        <v>0.407943</v>
+        <v>0.41075800000000001</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -457,22 +457,22 @@
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="2">
-        <v>0.38566299999999998</v>
+        <v>0.38770500000000002</v>
       </c>
       <c r="B2" s="2">
-        <v>2.9663110000000001</v>
+        <v>2.9267210000000001</v>
       </c>
       <c r="C2" s="2">
-        <v>4.5406000000000002E-2</v>
+        <v>4.7163999999999998E-2</v>
       </c>
       <c r="D2" s="2">
-        <v>1.6469999999999999E-2</v>
+        <v>1.5519E-2</v>
       </c>
       <c r="E2" s="2">
-        <v>3.3313000000000002E-2</v>
+        <v>3.2028000000000001E-2</v>
       </c>
       <c r="F2" s="2">
-        <v>4.5323000000000002E-2</v>
+        <v>4.3905E-2</v>
       </c>
       <c r="G2" s="2">
         <v>0</v>
@@ -484,16 +484,16 @@
         <v>2.9E-4</v>
       </c>
       <c r="J2" s="2">
-        <v>0.26583899999999999</v>
+        <v>0.26112200000000002</v>
       </c>
       <c r="K2" s="2">
-        <v>1.232E-3</v>
+        <v>1.8710000000000001E-3</v>
       </c>
       <c r="L2" s="2">
-        <v>5.5180000000000003E-3</v>
+        <v>4.8789999999999997E-3</v>
       </c>
       <c r="M2" s="2">
-        <v>9.810000000000001E-4</v>
+        <v>1.121E-3</v>
       </c>
       <c r="N2" s="2">
         <v>3.5199999999999999E-4</v>
@@ -511,7 +511,7 @@
         <v>8.7500000000000002E-4</v>
       </c>
       <c r="S2" s="2">
-        <v>0.13201499999999999</v>
+        <v>0.13042300000000001</v>
       </c>
       <c r="T2" s="2">
         <v>1.815E-3</v>
@@ -520,7 +520,7 @@
         <v>0</v>
       </c>
       <c r="V2" s="2">
-        <v>6.0300000000000002E-4</v>
+        <v>1.0449999999999999E-3</v>
       </c>
       <c r="W2" s="2">
         <v>2.9700000000000001E-4</v>
@@ -532,13 +532,13 @@
         <v>0</v>
       </c>
       <c r="Z2" s="2">
-        <v>9.6360000000000005E-3</v>
+        <v>8.9829999999999997E-3</v>
       </c>
       <c r="AA2" s="2">
         <v>1.5679999999999999E-3</v>
       </c>
       <c r="AB2" s="2">
-        <v>4.8000000000000001E-4</v>
+        <v>7.1900000000000002E-4</v>
       </c>
       <c r="AC2" s="2">
         <v>0</v>
@@ -547,7 +547,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="2">
-        <v>0.21810299999999999</v>
+        <v>0.21177000000000001</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -562,13 +562,13 @@
         <v>0</v>
       </c>
       <c r="C3" s="2">
-        <v>1.6726510000000001</v>
+        <v>1.664979</v>
       </c>
       <c r="D3" s="2">
-        <v>2.542E-3</v>
+        <v>2.2799999999999999E-3</v>
       </c>
       <c r="E3" s="2">
-        <v>0.26965299999999998</v>
+        <v>0.26414700000000002</v>
       </c>
       <c r="F3" s="2">
         <v>1.951E-3</v>
@@ -580,13 +580,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="2">
-        <v>1.2509999999999999E-3</v>
+        <v>1.2960000000000001E-3</v>
       </c>
       <c r="J3" s="2">
         <v>0</v>
       </c>
       <c r="K3" s="2">
-        <v>1.6374E-2</v>
+        <v>1.6913999999999998E-2</v>
       </c>
       <c r="L3" s="2">
         <v>0</v>
@@ -601,25 +601,25 @@
         <v>0</v>
       </c>
       <c r="P3" s="2">
-        <v>7.5750000000000001E-3</v>
+        <v>8.4749999999999999E-3</v>
       </c>
       <c r="Q3" s="2">
         <v>5.326E-3</v>
       </c>
       <c r="R3" s="2">
-        <v>3.9230000000000003E-3</v>
+        <v>3.9519999999999998E-3</v>
       </c>
       <c r="S3" s="2">
         <v>0</v>
       </c>
       <c r="T3" s="2">
-        <v>3.3384999999999998E-2</v>
+        <v>3.2745000000000003E-2</v>
       </c>
       <c r="U3" s="2">
         <v>1.0280000000000001E-3</v>
       </c>
       <c r="V3" s="2">
-        <v>1.0038E-2</v>
+        <v>8.6440000000000006E-3</v>
       </c>
       <c r="W3" s="2">
         <v>0</v>
@@ -646,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="2">
-        <v>1.3403E-2</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -661,22 +661,22 @@
         <v>2.6819999999999999E-3</v>
       </c>
       <c r="C4" s="2">
-        <v>6.0910000000000001E-3</v>
+        <v>7.0299999999999998E-3</v>
       </c>
       <c r="D4" s="2">
-        <v>0.89956100000000006</v>
+        <v>0.90019499999999997</v>
       </c>
       <c r="E4" s="2">
         <v>3.6999999999999999E-4</v>
       </c>
       <c r="F4" s="2">
-        <v>0.38763199999999998</v>
+        <v>0.39141599999999999</v>
       </c>
       <c r="G4" s="2">
         <v>4.2810000000000001E-3</v>
       </c>
       <c r="H4" s="2">
-        <v>1.4729999999999999E-3</v>
+        <v>1.7639999999999999E-3</v>
       </c>
       <c r="I4" s="2">
         <v>2.4499999999999999E-4</v>
@@ -688,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="2">
-        <v>2.6352E-2</v>
+        <v>2.5107999999999998E-2</v>
       </c>
       <c r="M4" s="2">
         <v>0</v>
@@ -703,25 +703,25 @@
         <v>0</v>
       </c>
       <c r="Q4" s="2">
-        <v>3.4702999999999998E-2</v>
+        <v>3.4218999999999999E-2</v>
       </c>
       <c r="R4" s="2">
         <v>0</v>
       </c>
       <c r="S4" s="2">
-        <v>1.2995E-2</v>
+        <v>1.3762E-2</v>
       </c>
       <c r="T4" s="2">
-        <v>1.5989999999999999E-3</v>
+        <v>2.0799999999999998E-3</v>
       </c>
       <c r="U4" s="2">
-        <v>2.5392000000000001E-2</v>
+        <v>2.7274E-2</v>
       </c>
       <c r="V4" s="2">
         <v>1.3940000000000001E-3</v>
       </c>
       <c r="W4" s="2">
-        <v>7.4840000000000002E-3</v>
+        <v>7.4780000000000003E-3</v>
       </c>
       <c r="X4" s="2">
         <v>0</v>
@@ -745,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="2">
-        <v>3.6339999999999997E-2</v>
+        <v>3.5987999999999999E-2</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -760,13 +760,13 @@
         <v>0</v>
       </c>
       <c r="C5" s="2">
-        <v>6.9336999999999996E-2</v>
+        <v>6.9403999999999993E-2</v>
       </c>
       <c r="D5" s="2">
         <v>8.3299999999999997E-4</v>
       </c>
       <c r="E5" s="2">
-        <v>0.30460599999999999</v>
+        <v>0.29631299999999999</v>
       </c>
       <c r="F5" s="2">
         <v>8.6200000000000003E-4</v>
@@ -778,13 +778,13 @@
         <v>0</v>
       </c>
       <c r="I5" s="2">
-        <v>1.431E-3</v>
+        <v>2.1410000000000001E-3</v>
       </c>
       <c r="J5" s="2">
         <v>0</v>
       </c>
       <c r="K5" s="2">
-        <v>2.4698000000000001E-2</v>
+        <v>2.3719E-2</v>
       </c>
       <c r="L5" s="2">
         <v>6.38E-4</v>
@@ -805,19 +805,19 @@
         <v>9.3000000000000005E-4</v>
       </c>
       <c r="R5" s="2">
-        <v>3.346E-3</v>
+        <v>3.483E-3</v>
       </c>
       <c r="S5" s="2">
         <v>3.7800000000000003E-4</v>
       </c>
       <c r="T5" s="2">
-        <v>5.6610000000000002E-3</v>
+        <v>5.3E-3</v>
       </c>
       <c r="U5" s="2">
         <v>0</v>
       </c>
       <c r="V5" s="2">
-        <v>1.2768E-2</v>
+        <v>1.2848999999999999E-2</v>
       </c>
       <c r="W5" s="2">
         <v>0</v>
@@ -844,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="2">
-        <v>1.1636000000000001E-2</v>
+        <v>1.0580000000000001E-2</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -862,13 +862,13 @@
         <v>1.2E-4</v>
       </c>
       <c r="D6" s="2">
-        <v>2.8441999999999999E-2</v>
+        <v>2.7503E-2</v>
       </c>
       <c r="E6" s="2">
         <v>1.498E-3</v>
       </c>
       <c r="F6" s="2">
-        <v>0.17683099999999999</v>
+        <v>0.172067</v>
       </c>
       <c r="G6" s="2">
         <v>0</v>
@@ -880,13 +880,13 @@
         <v>6.0300000000000002E-4</v>
       </c>
       <c r="J6" s="2">
-        <v>0</v>
+        <v>3.4000000000000002E-4</v>
       </c>
       <c r="K6" s="2">
         <v>0</v>
       </c>
       <c r="L6" s="2">
-        <v>3.2368000000000001E-2</v>
+        <v>3.1287000000000002E-2</v>
       </c>
       <c r="M6" s="2">
         <v>3.7399999999999998E-4</v>
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
       <c r="Q6" s="2">
-        <v>9.9799999999999997E-4</v>
+        <v>1.2300000000000001E-4</v>
       </c>
       <c r="R6" s="2">
         <v>0</v>
@@ -913,13 +913,13 @@
         <v>0</v>
       </c>
       <c r="U6" s="2">
-        <v>1.181E-3</v>
+        <v>2.1210000000000001E-3</v>
       </c>
       <c r="V6" s="2">
         <v>0</v>
       </c>
       <c r="W6" s="2">
-        <v>2.9510000000000001E-3</v>
+        <v>2.2190000000000001E-3</v>
       </c>
       <c r="X6" s="2">
         <v>0</v>
@@ -943,7 +943,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="2">
-        <v>1.6930000000000001E-2</v>
+        <v>1.7634E-2</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -970,13 +970,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="2">
-        <v>1.0808E-2</v>
+        <v>1.2645E-2</v>
       </c>
       <c r="H7" s="2">
         <v>0</v>
       </c>
       <c r="I7" s="2">
-        <v>3.398E-3</v>
+        <v>3.6879999999999999E-3</v>
       </c>
       <c r="J7" s="2">
         <v>0</v>
@@ -1141,7 +1141,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="2">
-        <v>2.1280000000000001E-3</v>
+        <v>1.776E-3</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1204,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="S9" s="2">
-        <v>0</v>
+        <v>3.7800000000000003E-4</v>
       </c>
       <c r="T9" s="2">
         <v>0</v>
@@ -1249,22 +1249,22 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="2">
-        <v>7.5820000000000002E-3</v>
+        <v>9.0860000000000003E-3</v>
       </c>
       <c r="B10" s="2">
-        <v>8.5429000000000005E-2</v>
+        <v>0.10488699999999999</v>
       </c>
       <c r="C10" s="2">
-        <v>5.2100000000000002E-3</v>
+        <v>5.4510000000000001E-3</v>
       </c>
       <c r="D10" s="2">
-        <v>1.083E-3</v>
+        <v>1.916E-3</v>
       </c>
       <c r="E10" s="2">
-        <v>1.1342E-2</v>
+        <v>1.2840000000000001E-2</v>
       </c>
       <c r="F10" s="2">
-        <v>8.1679999999999999E-3</v>
+        <v>8.5990000000000007E-3</v>
       </c>
       <c r="G10" s="2">
         <v>0</v>
@@ -1276,13 +1276,13 @@
         <v>0</v>
       </c>
       <c r="J10" s="2">
-        <v>0.101885</v>
+        <v>0.108443</v>
       </c>
       <c r="K10" s="2">
         <v>1.1789999999999999E-3</v>
       </c>
       <c r="L10" s="2">
-        <v>3.7330000000000002E-3</v>
+        <v>5.0099999999999997E-3</v>
       </c>
       <c r="M10" s="2">
         <v>0</v>
@@ -1297,13 +1297,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="2">
-        <v>4.6090000000000002E-3</v>
+        <v>5.6080000000000001E-3</v>
       </c>
       <c r="R10" s="2">
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="S10" s="2">
-        <v>1.021E-2</v>
+        <v>1.2872E-2</v>
       </c>
       <c r="T10" s="2">
         <v>0</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="2">
-        <v>4.1710000000000002E-3</v>
+        <v>4.8240000000000002E-3</v>
       </c>
       <c r="AA10" s="2">
         <v>0</v>
@@ -1339,7 +1339,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="2">
-        <v>8.5537000000000002E-2</v>
+        <v>9.9618999999999999E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1360,7 +1360,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="2">
-        <v>7.0990000000000003E-3</v>
+        <v>8.5970000000000005E-3</v>
       </c>
       <c r="F11" s="2">
         <v>6.8099999999999996E-4</v>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="2">
-        <v>2.4710000000000001E-3</v>
+        <v>2.4629999999999999E-3</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1456,13 +1456,13 @@
         <v>0</v>
       </c>
       <c r="D12" s="2">
-        <v>0</v>
+        <v>4.6999999999999999E-4</v>
       </c>
       <c r="E12" s="2">
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>4.6979999999999999E-3</v>
+        <v>5.3790000000000001E-3</v>
       </c>
       <c r="G12" s="2">
         <v>0</v>
@@ -1480,7 +1480,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="2">
-        <v>1.915E-3</v>
+        <v>2.5539999999999998E-3</v>
       </c>
       <c r="M12" s="2">
         <v>0</v>
@@ -1513,7 +1513,7 @@
         <v>0</v>
       </c>
       <c r="W12" s="2">
-        <v>0</v>
+        <v>3.6600000000000001E-4</v>
       </c>
       <c r="X12" s="2">
         <v>0</v>
@@ -1582,7 +1582,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2">
-        <v>5.2586000000000001E-2</v>
+        <v>5.2352000000000003E-2</v>
       </c>
       <c r="N13" s="2">
         <v>0</v>
@@ -1636,7 +1636,7 @@
         <v>0</v>
       </c>
       <c r="AE13" s="2">
-        <v>1.776E-3</v>
+        <v>1.768E-3</v>
       </c>
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
@@ -1684,7 +1684,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="2">
-        <v>1.639E-3</v>
+        <v>1.405E-3</v>
       </c>
       <c r="O14" s="2">
         <v>0</v>
@@ -1849,13 +1849,13 @@
         <v>9.9299999999999996E-4</v>
       </c>
       <c r="C16" s="2">
-        <v>0.14453299999999999</v>
+        <v>0.14616899999999999</v>
       </c>
       <c r="D16" s="2">
         <v>8.3299999999999997E-4</v>
       </c>
       <c r="E16" s="2">
-        <v>1.5924000000000001E-2</v>
+        <v>1.5174999999999999E-2</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
@@ -1888,19 +1888,19 @@
         <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>1.262826</v>
+        <v>1.2677020000000001</v>
       </c>
       <c r="Q16" s="2">
-        <v>3.1740000000000002E-3</v>
+        <v>4.0489999999999996E-3</v>
       </c>
       <c r="R16" s="2">
-        <v>0.26345000000000002</v>
+        <v>0.26593099999999997</v>
       </c>
       <c r="S16" s="2">
         <v>3.6000000000000002E-4</v>
       </c>
       <c r="T16" s="2">
-        <v>8.6730000000000002E-3</v>
+        <v>9.0329999999999994E-3</v>
       </c>
       <c r="U16" s="2">
         <v>0</v>
@@ -1915,7 +1915,7 @@
         <v>0</v>
       </c>
       <c r="Y16" s="2">
-        <v>8.7139999999999995E-3</v>
+        <v>9.0620000000000006E-3</v>
       </c>
       <c r="Z16" s="2">
         <v>6.5399999999999996E-4</v>
@@ -1924,7 +1924,7 @@
         <v>0</v>
       </c>
       <c r="AB16" s="2">
-        <v>0</v>
+        <v>2.4000000000000001E-4</v>
       </c>
       <c r="AC16" s="2">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="2">
-        <v>3.1327000000000001E-2</v>
+        <v>3.1688000000000001E-2</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1942,25 +1942,25 @@
     </row>
     <row r="17" spans="1:35">
       <c r="A17" s="2">
-        <v>1.5657000000000001E-2</v>
+        <v>1.6160000000000001E-2</v>
       </c>
       <c r="B17" s="2">
-        <v>1.7413000000000001E-2</v>
+        <v>1.8540000000000001E-2</v>
       </c>
       <c r="C17" s="2">
-        <v>9.1009999999999997E-3</v>
+        <v>8.0549999999999997E-3</v>
       </c>
       <c r="D17" s="2">
-        <v>0.11409</v>
+        <v>0.113506</v>
       </c>
       <c r="E17" s="2">
         <v>1.867E-3</v>
       </c>
       <c r="F17" s="2">
-        <v>5.7473000000000003E-2</v>
+        <v>5.8821999999999999E-2</v>
       </c>
       <c r="G17" s="2">
-        <v>3.8440000000000002E-3</v>
+        <v>2.8410000000000002E-3</v>
       </c>
       <c r="H17" s="2">
         <v>0</v>
@@ -1975,10 +1975,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="2">
-        <v>2.2959999999999999E-3</v>
+        <v>2.9350000000000001E-3</v>
       </c>
       <c r="M17" s="2">
-        <v>7.0200000000000004E-4</v>
+        <v>4.6799999999999999E-4</v>
       </c>
       <c r="N17" s="2">
         <v>0</v>
@@ -1987,28 +1987,28 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>8.4010000000000005E-3</v>
+        <v>8.3999999999999995E-3</v>
       </c>
       <c r="Q17" s="2">
-        <v>3.7281140000000001</v>
+        <v>3.7176960000000001</v>
       </c>
       <c r="R17" s="2">
         <v>1.0120000000000001E-3</v>
       </c>
       <c r="S17" s="2">
-        <v>0.72091000000000005</v>
+        <v>0.72534699999999996</v>
       </c>
       <c r="T17" s="2">
-        <v>1.9724999999999999E-2</v>
+        <v>2.1432E-2</v>
       </c>
       <c r="U17" s="2">
-        <v>1.0494E-2</v>
+        <v>9.554E-3</v>
       </c>
       <c r="V17" s="2">
-        <v>3.392E-3</v>
+        <v>4.7869999999999996E-3</v>
       </c>
       <c r="W17" s="2">
-        <v>1.7099999999999999E-3</v>
+        <v>2.4369999999999999E-3</v>
       </c>
       <c r="X17" s="2">
         <v>0</v>
@@ -2017,13 +2017,13 @@
         <v>0</v>
       </c>
       <c r="Z17" s="2">
-        <v>3.5478999999999997E-2</v>
+        <v>3.5784999999999997E-2</v>
       </c>
       <c r="AA17" s="2">
-        <v>6.5399999999999996E-4</v>
+        <v>0</v>
       </c>
       <c r="AB17" s="2">
-        <v>2.0839999999999999E-3</v>
+        <v>1.8450000000000001E-3</v>
       </c>
       <c r="AC17" s="2">
         <v>7.6499999999999995E-4</v>
@@ -2032,7 +2032,7 @@
         <v>3.8299999999999999E-4</v>
       </c>
       <c r="AE17" s="2">
-        <v>3.4812000000000003E-2</v>
+        <v>3.3009999999999998E-2</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2047,16 +2047,16 @@
         <v>2.1580000000000002E-3</v>
       </c>
       <c r="C18" s="2">
-        <v>2.0249E-2</v>
+        <v>2.0181999999999999E-2</v>
       </c>
       <c r="D18" s="2">
         <v>0</v>
       </c>
       <c r="E18" s="2">
-        <v>4.8835999999999997E-2</v>
+        <v>4.7701E-2</v>
       </c>
       <c r="F18" s="2">
-        <v>6.8099999999999996E-4</v>
+        <v>1.1119999999999999E-3</v>
       </c>
       <c r="G18" s="2">
         <v>0</v>
@@ -2068,10 +2068,10 @@
         <v>0</v>
       </c>
       <c r="J18" s="2">
-        <v>6.38E-4</v>
+        <v>0</v>
       </c>
       <c r="K18" s="2">
-        <v>1.9689999999999998E-3</v>
+        <v>1.6169999999999999E-3</v>
       </c>
       <c r="L18" s="2">
         <v>0</v>
@@ -2086,25 +2086,25 @@
         <v>0</v>
       </c>
       <c r="P18" s="2">
-        <v>6.0453E-2</v>
+        <v>6.0437999999999999E-2</v>
       </c>
       <c r="Q18" s="2">
         <v>5.5000000000000002E-5</v>
       </c>
       <c r="R18" s="2">
-        <v>0.36832500000000001</v>
+        <v>0.36191499999999999</v>
       </c>
       <c r="S18" s="2">
         <v>3.8349999999999999E-3</v>
       </c>
       <c r="T18" s="2">
-        <v>2.4520000000000002E-3</v>
+        <v>2.5600000000000002E-3</v>
       </c>
       <c r="U18" s="2">
         <v>0</v>
       </c>
       <c r="V18" s="2">
-        <v>3.4160000000000002E-3</v>
+        <v>2.0920000000000001E-3</v>
       </c>
       <c r="W18" s="2">
         <v>0</v>
@@ -2113,10 +2113,10 @@
         <v>0</v>
       </c>
       <c r="Y18" s="2">
-        <v>4.0406999999999998E-2</v>
+        <v>4.0016999999999997E-2</v>
       </c>
       <c r="Z18" s="2">
-        <v>3.48E-4</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="2">
         <v>0</v>
@@ -2131,7 +2131,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="2">
-        <v>3.2759999999999997E-2</v>
+        <v>3.2399999999999998E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2149,16 +2149,16 @@
         <v>1.1130000000000001E-3</v>
       </c>
       <c r="D19" s="2">
-        <v>2.5922000000000001E-2</v>
+        <v>2.6391999999999999E-2</v>
       </c>
       <c r="E19" s="2">
         <v>9.2299999999999999E-4</v>
       </c>
       <c r="F19" s="2">
-        <v>5.2527999999999998E-2</v>
+        <v>5.4149999999999997E-2</v>
       </c>
       <c r="G19" s="2">
-        <v>3.6749999999999999E-3</v>
+        <v>3.7919999999999998E-3</v>
       </c>
       <c r="H19" s="2">
         <v>6.4800000000000003E-4</v>
@@ -2167,13 +2167,13 @@
         <v>7.1599999999999995E-4</v>
       </c>
       <c r="J19" s="2">
-        <v>6.8000000000000005E-4</v>
+        <v>3.4000000000000002E-4</v>
       </c>
       <c r="K19" s="2">
         <v>0</v>
       </c>
       <c r="L19" s="2">
-        <v>5.8050000000000003E-3</v>
+        <v>6.4429999999999999E-3</v>
       </c>
       <c r="M19" s="2">
         <v>3.7399999999999998E-4</v>
@@ -2188,22 +2188,22 @@
         <v>8.9099999999999997E-4</v>
       </c>
       <c r="Q19" s="2">
-        <v>0.14893999999999999</v>
+        <v>0.15104699999999999</v>
       </c>
       <c r="R19" s="2">
-        <v>4.0480000000000004E-3</v>
+        <v>3.0360000000000001E-3</v>
       </c>
       <c r="S19" s="2">
-        <v>0.71958800000000001</v>
+        <v>0.71881600000000001</v>
       </c>
       <c r="T19" s="2">
-        <v>7.0959999999999999E-3</v>
+        <v>6.1339999999999997E-3</v>
       </c>
       <c r="U19" s="2">
         <v>4.9969999999999997E-3</v>
       </c>
       <c r="V19" s="2">
-        <v>7.156E-3</v>
+        <v>6.7140000000000003E-3</v>
       </c>
       <c r="W19" s="2">
         <v>6.3E-3</v>
@@ -2215,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="Z19" s="2">
-        <v>7.2568999999999995E-2</v>
+        <v>7.0707999999999993E-2</v>
       </c>
       <c r="AA19" s="2">
-        <v>1.761E-3</v>
+        <v>1.207E-3</v>
       </c>
       <c r="AB19" s="2">
         <v>4.8000000000000001E-4</v>
@@ -2230,7 +2230,7 @@
         <v>3.8299999999999999E-4</v>
       </c>
       <c r="AE19" s="2">
-        <v>3.3765000000000003E-2</v>
+        <v>3.4117000000000001E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2">
-        <v>1.0562E-2</v>
+        <v>9.5580000000000005E-3</v>
       </c>
       <c r="H20" s="2">
         <v>0</v>
@@ -2296,13 +2296,13 @@
         <v>7.67E-4</v>
       </c>
       <c r="T20" s="2">
-        <v>0.110968</v>
+        <v>0.11144900000000001</v>
       </c>
       <c r="U20" s="2">
-        <v>9.41E-4</v>
+        <v>0</v>
       </c>
       <c r="V20" s="2">
-        <v>4.1648999999999999E-2</v>
+        <v>4.2251999999999998E-2</v>
       </c>
       <c r="W20" s="2">
         <v>3.6600000000000001E-4</v>
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="2">
-        <v>2.7629999999999998E-3</v>
+        <v>2.209E-3</v>
       </c>
       <c r="AB20" s="2">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="2">
-        <v>2.8739999999999998E-3</v>
+        <v>3.2260000000000001E-3</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2353,10 +2353,10 @@
         <v>0</v>
       </c>
       <c r="F21" s="2">
-        <v>1.714E-3</v>
+        <v>1.0330000000000001E-3</v>
       </c>
       <c r="G21" s="2">
-        <v>0</v>
+        <v>9.19E-4</v>
       </c>
       <c r="H21" s="2">
         <v>5.8E-4</v>
@@ -2398,13 +2398,13 @@
         <v>2.5600000000000002E-3</v>
       </c>
       <c r="U21" s="2">
-        <v>4.1175999999999997E-2</v>
+        <v>4.0236000000000001E-2</v>
       </c>
       <c r="V21" s="2">
         <v>1.057E-3</v>
       </c>
       <c r="W21" s="2">
-        <v>1.5443999999999999E-2</v>
+        <v>1.6404999999999999E-2</v>
       </c>
       <c r="X21" s="2">
         <v>0</v>
@@ -2428,7 +2428,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="2">
-        <v>5.7390000000000002E-3</v>
+        <v>6.0990000000000003E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2461,7 +2461,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="2">
-        <v>2.66E-3</v>
+        <v>2.3700000000000001E-3</v>
       </c>
       <c r="J22" s="2">
         <v>0</v>
@@ -2494,13 +2494,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="2">
-        <v>2.8119999999999998E-3</v>
+        <v>2.4399999999999999E-3</v>
       </c>
       <c r="U22" s="2">
         <v>0</v>
       </c>
       <c r="V22" s="2">
-        <v>2.0506E-2</v>
+        <v>2.0145E-2</v>
       </c>
       <c r="W22" s="2">
         <v>0</v>
@@ -2515,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="2">
-        <v>2.5569999999999998E-3</v>
+        <v>3.1110000000000001E-3</v>
       </c>
       <c r="AB22" s="2">
         <v>0</v>
@@ -2593,7 +2593,7 @@
         <v>0</v>
       </c>
       <c r="T23" s="2">
-        <v>0</v>
+        <v>3.7300000000000001E-4</v>
       </c>
       <c r="U23" s="2">
         <v>1.2E-4</v>
@@ -2746,7 +2746,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="2">
-        <v>5.5900000000000004E-3</v>
+        <v>8.5749999999999993E-3</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -2785,19 +2785,19 @@
         <v>0</v>
       </c>
       <c r="R25" s="2">
-        <v>1.1873999999999999E-2</v>
+        <v>1.5552E-2</v>
       </c>
       <c r="S25" s="2">
-        <v>0</v>
+        <v>7.67E-4</v>
       </c>
       <c r="T25" s="2">
-        <v>4.8099999999999998E-4</v>
+        <v>0</v>
       </c>
       <c r="U25" s="2">
         <v>0</v>
       </c>
       <c r="V25" s="2">
-        <v>2.4520000000000002E-3</v>
+        <v>2.8930000000000002E-3</v>
       </c>
       <c r="W25" s="2">
         <v>0</v>
@@ -2806,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="Y25" s="2">
-        <v>1.4657999999999999E-2</v>
+        <v>1.5006E-2</v>
       </c>
       <c r="Z25" s="2">
         <v>3.6000000000000002E-4</v>
@@ -2824,7 +2824,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="2">
-        <v>8.6300000000000005E-3</v>
+        <v>1.0054E-2</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2857,10 +2857,10 @@
         <v>0</v>
       </c>
       <c r="I26" s="2">
-        <v>3.5799999999999997E-4</v>
+        <v>0</v>
       </c>
       <c r="J26" s="2">
-        <v>9.7799999999999992E-4</v>
+        <v>1.3179999999999999E-3</v>
       </c>
       <c r="K26" s="2">
         <v>0</v>
@@ -2887,19 +2887,19 @@
         <v>8.7500000000000002E-4</v>
       </c>
       <c r="S26" s="2">
-        <v>1.6358000000000001E-2</v>
+        <v>1.8658999999999999E-2</v>
       </c>
       <c r="T26" s="2">
-        <v>4.8099999999999998E-4</v>
+        <v>9.6199999999999996E-4</v>
       </c>
       <c r="U26" s="2">
         <v>0</v>
       </c>
       <c r="V26" s="2">
-        <v>4.4099999999999999E-4</v>
+        <v>8.83E-4</v>
       </c>
       <c r="W26" s="2">
-        <v>1.0989999999999999E-3</v>
+        <v>1.4660000000000001E-3</v>
       </c>
       <c r="X26" s="2">
         <v>0</v>
@@ -2923,7 +2923,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="2">
-        <v>7.8919999999999997E-3</v>
+        <v>8.9560000000000004E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -2956,7 +2956,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="2">
-        <v>0</v>
+        <v>2.9E-4</v>
       </c>
       <c r="J27" s="2">
         <v>0</v>
@@ -2995,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="V27" s="2">
-        <v>0</v>
+        <v>6.9700000000000003E-4</v>
       </c>
       <c r="W27" s="2">
         <v>0</v>

</xml_diff>

<commit_message>
update initial num Nevt why?
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB053617-7DF4-4122-BE4C-F7E78F574CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7ADD60-1D84-46E7-B56E-940017F5F899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -358,22 +358,22 @@
   <sheetData>
     <row r="1" spans="1:35">
       <c r="A1" s="2">
-        <v>12.026999</v>
+        <v>11.994846000000001</v>
       </c>
       <c r="B1" s="2">
-        <v>3.4237449999999998</v>
+        <v>3.4145919999999998</v>
       </c>
       <c r="C1" s="2">
-        <v>0.18410099999999999</v>
+        <v>0.18360899999999999</v>
       </c>
       <c r="D1" s="2">
-        <v>7.1387000000000006E-2</v>
+        <v>7.1195999999999995E-2</v>
       </c>
       <c r="E1" s="2">
-        <v>3.1815000000000003E-2</v>
+        <v>3.1730000000000001E-2</v>
       </c>
       <c r="F1" s="2">
-        <v>5.5015000000000001E-2</v>
+        <v>5.4866999999999999E-2</v>
       </c>
       <c r="G1" s="2">
         <v>1.17E-4</v>
@@ -385,43 +385,43 @@
         <v>0</v>
       </c>
       <c r="J1" s="2">
-        <v>0.11765299999999999</v>
+        <v>0.117338</v>
       </c>
       <c r="K1" s="2">
-        <v>1.1789999999999999E-3</v>
+        <v>1.176E-3</v>
       </c>
       <c r="L1" s="2">
-        <v>5.633E-3</v>
+        <v>5.6179999999999997E-3</v>
       </c>
       <c r="M1" s="2">
-        <v>2.3869999999999998E-3</v>
+        <v>2.3809999999999999E-3</v>
       </c>
       <c r="N1" s="2">
-        <v>7.2499999999999995E-4</v>
+        <v>7.2300000000000001E-4</v>
       </c>
       <c r="O1" s="2">
         <v>0</v>
       </c>
       <c r="P1" s="2">
-        <v>1.3209999999999999E-3</v>
+        <v>1.3179999999999999E-3</v>
       </c>
       <c r="Q1" s="2">
-        <v>0.63055600000000001</v>
+        <v>0.62896600000000003</v>
       </c>
       <c r="R1" s="2">
-        <v>3.4359999999999998E-3</v>
+        <v>3.4269999999999999E-3</v>
       </c>
       <c r="S1" s="2">
-        <v>0.108932</v>
+        <v>0.108657</v>
       </c>
       <c r="T1" s="2">
-        <v>3.0409999999999999E-3</v>
+        <v>3.0339999999999998E-3</v>
       </c>
       <c r="U1" s="2">
-        <v>4.1229999999999999E-3</v>
+        <v>4.1130000000000003E-3</v>
       </c>
       <c r="V1" s="2">
-        <v>2.2769999999999999E-3</v>
+        <v>2.2720000000000001E-3</v>
       </c>
       <c r="W1" s="2">
         <v>3.6600000000000001E-4</v>
@@ -433,22 +433,22 @@
         <v>0</v>
       </c>
       <c r="Z1" s="2">
-        <v>5.8650000000000004E-3</v>
+        <v>5.8500000000000002E-3</v>
       </c>
       <c r="AA1" s="2">
         <v>0</v>
       </c>
       <c r="AB1" s="2">
-        <v>1.3190000000000001E-3</v>
+        <v>1.3159999999999999E-3</v>
       </c>
       <c r="AC1" s="2">
         <v>0</v>
       </c>
       <c r="AD1" s="2">
-        <v>2.4000000000000001E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AE1" s="2">
-        <v>0.41075800000000001</v>
+        <v>0.409661</v>
       </c>
       <c r="AF1" s="1"/>
       <c r="AG1" s="1"/>
@@ -457,22 +457,22 @@
     </row>
     <row r="2" spans="1:35">
       <c r="A2" s="2">
-        <v>0.38770500000000002</v>
+        <v>0.38666800000000001</v>
       </c>
       <c r="B2" s="2">
-        <v>2.9267210000000001</v>
+        <v>2.9188969999999999</v>
       </c>
       <c r="C2" s="2">
-        <v>4.7163999999999998E-2</v>
+        <v>4.7038000000000003E-2</v>
       </c>
       <c r="D2" s="2">
-        <v>1.5519E-2</v>
+        <v>1.5478E-2</v>
       </c>
       <c r="E2" s="2">
-        <v>3.2028000000000001E-2</v>
+        <v>3.1941999999999998E-2</v>
       </c>
       <c r="F2" s="2">
-        <v>4.3905E-2</v>
+        <v>4.3788000000000001E-2</v>
       </c>
       <c r="G2" s="2">
         <v>0</v>
@@ -481,49 +481,49 @@
         <v>0</v>
       </c>
       <c r="I2" s="2">
-        <v>2.9E-4</v>
+        <v>2.8899999999999998E-4</v>
       </c>
       <c r="J2" s="2">
-        <v>0.26112200000000002</v>
+        <v>0.26042399999999999</v>
       </c>
       <c r="K2" s="2">
-        <v>1.8710000000000001E-3</v>
+        <v>1.866E-3</v>
       </c>
       <c r="L2" s="2">
-        <v>4.8789999999999997E-3</v>
+        <v>4.8659999999999997E-3</v>
       </c>
       <c r="M2" s="2">
-        <v>1.121E-3</v>
+        <v>1.1180000000000001E-3</v>
       </c>
       <c r="N2" s="2">
-        <v>3.5199999999999999E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="O2" s="2">
         <v>0</v>
       </c>
       <c r="P2" s="2">
-        <v>4.4099999999999999E-4</v>
+        <v>4.4000000000000002E-4</v>
       </c>
       <c r="Q2" s="2">
-        <v>7.6303999999999997E-2</v>
+        <v>7.6110999999999998E-2</v>
       </c>
       <c r="R2" s="2">
-        <v>8.7500000000000002E-4</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="S2" s="2">
-        <v>0.13042300000000001</v>
+        <v>0.13009399999999999</v>
       </c>
       <c r="T2" s="2">
-        <v>1.815E-3</v>
+        <v>1.8109999999999999E-3</v>
       </c>
       <c r="U2" s="2">
         <v>0</v>
       </c>
       <c r="V2" s="2">
-        <v>1.0449999999999999E-3</v>
+        <v>1.042E-3</v>
       </c>
       <c r="W2" s="2">
-        <v>2.9700000000000001E-4</v>
+        <v>2.9599999999999998E-4</v>
       </c>
       <c r="X2" s="2">
         <v>0</v>
@@ -532,13 +532,13 @@
         <v>0</v>
       </c>
       <c r="Z2" s="2">
-        <v>8.9829999999999997E-3</v>
+        <v>8.9599999999999992E-3</v>
       </c>
       <c r="AA2" s="2">
-        <v>1.5679999999999999E-3</v>
+        <v>1.5640000000000001E-3</v>
       </c>
       <c r="AB2" s="2">
-        <v>7.1900000000000002E-4</v>
+        <v>7.1699999999999997E-4</v>
       </c>
       <c r="AC2" s="2">
         <v>0</v>
@@ -547,7 +547,7 @@
         <v>0</v>
       </c>
       <c r="AE2" s="2">
-        <v>0.21177000000000001</v>
+        <v>0.211205</v>
       </c>
       <c r="AF2" s="1"/>
       <c r="AG2" s="1"/>
@@ -556,37 +556,37 @@
     </row>
     <row r="3" spans="1:35">
       <c r="A3" s="2">
-        <v>1.4959999999999999E-3</v>
+        <v>1.4920000000000001E-3</v>
       </c>
       <c r="B3" s="2">
         <v>0</v>
       </c>
       <c r="C3" s="2">
-        <v>1.664979</v>
+        <v>1.660528</v>
       </c>
       <c r="D3" s="2">
-        <v>2.2799999999999999E-3</v>
+        <v>2.274E-3</v>
       </c>
       <c r="E3" s="2">
-        <v>0.26414700000000002</v>
+        <v>0.26344099999999998</v>
       </c>
       <c r="F3" s="2">
-        <v>1.951E-3</v>
+        <v>1.946E-3</v>
       </c>
       <c r="G3" s="2">
-        <v>5.3489999999999996E-3</v>
+        <v>5.3350000000000003E-3</v>
       </c>
       <c r="H3" s="2">
         <v>0</v>
       </c>
       <c r="I3" s="2">
-        <v>1.2960000000000001E-3</v>
+        <v>1.2930000000000001E-3</v>
       </c>
       <c r="J3" s="2">
         <v>0</v>
       </c>
       <c r="K3" s="2">
-        <v>1.6913999999999998E-2</v>
+        <v>1.6868999999999999E-2</v>
       </c>
       <c r="L3" s="2">
         <v>0</v>
@@ -601,25 +601,25 @@
         <v>0</v>
       </c>
       <c r="P3" s="2">
-        <v>8.4749999999999999E-3</v>
+        <v>8.4530000000000004E-3</v>
       </c>
       <c r="Q3" s="2">
-        <v>5.326E-3</v>
+        <v>5.313E-3</v>
       </c>
       <c r="R3" s="2">
-        <v>3.9519999999999998E-3</v>
+        <v>3.9420000000000002E-3</v>
       </c>
       <c r="S3" s="2">
         <v>0</v>
       </c>
       <c r="T3" s="2">
-        <v>3.2745000000000003E-2</v>
+        <v>3.2661999999999997E-2</v>
       </c>
       <c r="U3" s="2">
-        <v>1.0280000000000001E-3</v>
+        <v>1.0250000000000001E-3</v>
       </c>
       <c r="V3" s="2">
-        <v>8.6440000000000006E-3</v>
+        <v>8.6219999999999995E-3</v>
       </c>
       <c r="W3" s="2">
         <v>0</v>
@@ -628,16 +628,16 @@
         <v>0</v>
       </c>
       <c r="Y3" s="2">
-        <v>6.5399999999999996E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="Z3" s="2">
         <v>0</v>
       </c>
       <c r="AA3" s="2">
-        <v>1.6559999999999999E-3</v>
+        <v>1.6509999999999999E-3</v>
       </c>
       <c r="AB3" s="2">
-        <v>2.4000000000000001E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AC3" s="2">
         <v>0</v>
@@ -646,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="2">
-        <v>1.2699999999999999E-2</v>
+        <v>1.2666E-2</v>
       </c>
       <c r="AF3" s="1"/>
       <c r="AG3" s="1"/>
@@ -655,31 +655,31 @@
     </row>
     <row r="4" spans="1:35">
       <c r="A4" s="2">
-        <v>4.9799999999999996E-4</v>
+        <v>4.9700000000000005E-4</v>
       </c>
       <c r="B4" s="2">
-        <v>2.6819999999999999E-3</v>
+        <v>2.6749999999999999E-3</v>
       </c>
       <c r="C4" s="2">
-        <v>7.0299999999999998E-3</v>
+        <v>7.012E-3</v>
       </c>
       <c r="D4" s="2">
-        <v>0.90019499999999997</v>
+        <v>0.89778899999999995</v>
       </c>
       <c r="E4" s="2">
-        <v>3.6999999999999999E-4</v>
+        <v>3.6900000000000002E-4</v>
       </c>
       <c r="F4" s="2">
-        <v>0.39141599999999999</v>
+        <v>0.39036999999999999</v>
       </c>
       <c r="G4" s="2">
-        <v>4.2810000000000001E-3</v>
+        <v>4.2700000000000004E-3</v>
       </c>
       <c r="H4" s="2">
-        <v>1.7639999999999999E-3</v>
+        <v>1.7589999999999999E-3</v>
       </c>
       <c r="I4" s="2">
-        <v>2.4499999999999999E-4</v>
+        <v>2.4399999999999999E-4</v>
       </c>
       <c r="J4" s="2">
         <v>0</v>
@@ -688,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="2">
-        <v>2.5107999999999998E-2</v>
+        <v>2.5041000000000001E-2</v>
       </c>
       <c r="M4" s="2">
         <v>0</v>
@@ -703,25 +703,25 @@
         <v>0</v>
       </c>
       <c r="Q4" s="2">
-        <v>3.4218999999999999E-2</v>
+        <v>3.4132999999999997E-2</v>
       </c>
       <c r="R4" s="2">
         <v>0</v>
       </c>
       <c r="S4" s="2">
-        <v>1.3762E-2</v>
+        <v>1.3727E-2</v>
       </c>
       <c r="T4" s="2">
-        <v>2.0799999999999998E-3</v>
+        <v>2.0739999999999999E-3</v>
       </c>
       <c r="U4" s="2">
-        <v>2.7274E-2</v>
+        <v>2.7205E-2</v>
       </c>
       <c r="V4" s="2">
-        <v>1.3940000000000001E-3</v>
+        <v>1.3910000000000001E-3</v>
       </c>
       <c r="W4" s="2">
-        <v>7.4780000000000003E-3</v>
+        <v>7.4590000000000004E-3</v>
       </c>
       <c r="X4" s="2">
         <v>0</v>
@@ -730,13 +730,13 @@
         <v>0</v>
       </c>
       <c r="Z4" s="2">
-        <v>1.3079999999999999E-3</v>
+        <v>1.304E-3</v>
       </c>
       <c r="AA4" s="2">
         <v>0</v>
       </c>
       <c r="AB4" s="2">
-        <v>3.8299999999999999E-4</v>
+        <v>3.8200000000000002E-4</v>
       </c>
       <c r="AC4" s="2">
         <v>0</v>
@@ -745,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="AE4" s="2">
-        <v>3.5987999999999999E-2</v>
+        <v>3.5893000000000001E-2</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -760,34 +760,34 @@
         <v>0</v>
       </c>
       <c r="C5" s="2">
-        <v>6.9403999999999993E-2</v>
+        <v>6.9218000000000002E-2</v>
       </c>
       <c r="D5" s="2">
-        <v>8.3299999999999997E-4</v>
+        <v>8.3100000000000003E-4</v>
       </c>
       <c r="E5" s="2">
-        <v>0.29631299999999999</v>
+        <v>0.29552099999999998</v>
       </c>
       <c r="F5" s="2">
-        <v>8.6200000000000003E-4</v>
+        <v>8.5999999999999998E-4</v>
       </c>
       <c r="G5" s="2">
-        <v>2.9580000000000001E-3</v>
+        <v>2.9499999999999999E-3</v>
       </c>
       <c r="H5" s="2">
         <v>0</v>
       </c>
       <c r="I5" s="2">
-        <v>2.1410000000000001E-3</v>
+        <v>2.1350000000000002E-3</v>
       </c>
       <c r="J5" s="2">
         <v>0</v>
       </c>
       <c r="K5" s="2">
-        <v>2.3719E-2</v>
+        <v>2.3656E-2</v>
       </c>
       <c r="L5" s="2">
-        <v>6.38E-4</v>
+        <v>6.3699999999999998E-4</v>
       </c>
       <c r="M5" s="2">
         <v>0</v>
@@ -802,22 +802,22 @@
         <v>0</v>
       </c>
       <c r="Q5" s="2">
-        <v>9.3000000000000005E-4</v>
+        <v>9.2800000000000001E-4</v>
       </c>
       <c r="R5" s="2">
-        <v>3.483E-3</v>
+        <v>3.4740000000000001E-3</v>
       </c>
       <c r="S5" s="2">
-        <v>3.7800000000000003E-4</v>
+        <v>3.77E-4</v>
       </c>
       <c r="T5" s="2">
-        <v>5.3E-3</v>
+        <v>5.287E-3</v>
       </c>
       <c r="U5" s="2">
         <v>0</v>
       </c>
       <c r="V5" s="2">
-        <v>1.2848999999999999E-2</v>
+        <v>1.2815999999999999E-2</v>
       </c>
       <c r="W5" s="2">
         <v>0</v>
@@ -826,13 +826,13 @@
         <v>0</v>
       </c>
       <c r="Y5" s="2">
-        <v>6.96E-4</v>
+        <v>6.9399999999999996E-4</v>
       </c>
       <c r="Z5" s="2">
         <v>0</v>
       </c>
       <c r="AA5" s="2">
-        <v>2.209E-3</v>
+        <v>2.2039999999999998E-3</v>
       </c>
       <c r="AB5" s="2">
         <v>0</v>
@@ -844,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="AE5" s="2">
-        <v>1.0580000000000001E-2</v>
+        <v>1.0552000000000001E-2</v>
       </c>
       <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
@@ -856,19 +856,19 @@
         <v>0</v>
       </c>
       <c r="B6" s="2">
-        <v>1.34E-4</v>
+        <v>1.3300000000000001E-4</v>
       </c>
       <c r="C6" s="2">
         <v>1.2E-4</v>
       </c>
       <c r="D6" s="2">
-        <v>2.7503E-2</v>
+        <v>2.7428999999999999E-2</v>
       </c>
       <c r="E6" s="2">
-        <v>1.498E-3</v>
+        <v>1.4940000000000001E-3</v>
       </c>
       <c r="F6" s="2">
-        <v>0.172067</v>
+        <v>0.17160700000000001</v>
       </c>
       <c r="G6" s="2">
         <v>0</v>
@@ -877,19 +877,19 @@
         <v>0</v>
       </c>
       <c r="I6" s="2">
-        <v>6.0300000000000002E-4</v>
+        <v>6.0099999999999997E-4</v>
       </c>
       <c r="J6" s="2">
-        <v>3.4000000000000002E-4</v>
+        <v>3.39E-4</v>
       </c>
       <c r="K6" s="2">
         <v>0</v>
       </c>
       <c r="L6" s="2">
-        <v>3.1287000000000002E-2</v>
+        <v>3.1203000000000002E-2</v>
       </c>
       <c r="M6" s="2">
-        <v>3.7399999999999998E-4</v>
+        <v>3.7300000000000001E-4</v>
       </c>
       <c r="N6" s="2">
         <v>0</v>
@@ -907,19 +907,19 @@
         <v>0</v>
       </c>
       <c r="S6" s="2">
-        <v>4.7800000000000004E-3</v>
+        <v>4.7679999999999997E-3</v>
       </c>
       <c r="T6" s="2">
         <v>0</v>
       </c>
       <c r="U6" s="2">
-        <v>2.1210000000000001E-3</v>
+        <v>2.1159999999999998E-3</v>
       </c>
       <c r="V6" s="2">
         <v>0</v>
       </c>
       <c r="W6" s="2">
-        <v>2.2190000000000001E-3</v>
+        <v>2.2130000000000001E-3</v>
       </c>
       <c r="X6" s="2">
         <v>0</v>
@@ -928,10 +928,10 @@
         <v>0</v>
       </c>
       <c r="Z6" s="2">
-        <v>1.207E-3</v>
+        <v>1.204E-3</v>
       </c>
       <c r="AA6" s="2">
-        <v>6.5399999999999996E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AB6" s="2">
         <v>0</v>
@@ -943,7 +943,7 @@
         <v>0</v>
       </c>
       <c r="AE6" s="2">
-        <v>1.7634E-2</v>
+        <v>1.7586999999999998E-2</v>
       </c>
       <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
@@ -958,7 +958,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="2">
-        <v>3.5199999999999999E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="D7" s="2">
         <v>0</v>
@@ -970,13 +970,13 @@
         <v>0</v>
       </c>
       <c r="G7" s="2">
-        <v>1.2645E-2</v>
+        <v>1.2612E-2</v>
       </c>
       <c r="H7" s="2">
         <v>0</v>
       </c>
       <c r="I7" s="2">
-        <v>3.6879999999999999E-3</v>
+        <v>3.6779999999999998E-3</v>
       </c>
       <c r="J7" s="2">
         <v>0</v>
@@ -1015,13 +1015,13 @@
         <v>0</v>
       </c>
       <c r="V7" s="2">
-        <v>2.5330000000000001E-3</v>
+        <v>2.5270000000000002E-3</v>
       </c>
       <c r="W7" s="2">
         <v>0</v>
       </c>
       <c r="X7" s="2">
-        <v>2.9700000000000001E-4</v>
+        <v>2.9599999999999998E-4</v>
       </c>
       <c r="Y7" s="2">
         <v>0</v>
@@ -1042,7 +1042,7 @@
         <v>0</v>
       </c>
       <c r="AE7" s="2">
-        <v>1.4159999999999999E-3</v>
+        <v>1.4120000000000001E-3</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
@@ -1072,7 +1072,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="2">
-        <v>1.7830000000000001E-3</v>
+        <v>1.7780000000000001E-3</v>
       </c>
       <c r="I8" s="2">
         <v>0</v>
@@ -1141,7 +1141,7 @@
         <v>0</v>
       </c>
       <c r="AE8" s="2">
-        <v>1.776E-3</v>
+        <v>1.771E-3</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -1174,7 +1174,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="2">
-        <v>1.364E-3</v>
+        <v>1.3600000000000001E-3</v>
       </c>
       <c r="J9" s="2">
         <v>0</v>
@@ -1204,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="S9" s="2">
-        <v>3.7800000000000003E-4</v>
+        <v>3.77E-4</v>
       </c>
       <c r="T9" s="2">
         <v>0</v>
@@ -1240,7 +1240,7 @@
         <v>0</v>
       </c>
       <c r="AE9" s="2">
-        <v>3.5199999999999999E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="AF9" s="1"/>
       <c r="AG9" s="1"/>
@@ -1249,22 +1249,22 @@
     </row>
     <row r="10" spans="1:35">
       <c r="A10" s="2">
-        <v>9.0860000000000003E-3</v>
+        <v>9.0620000000000006E-3</v>
       </c>
       <c r="B10" s="2">
-        <v>0.10488699999999999</v>
+        <v>0.104606</v>
       </c>
       <c r="C10" s="2">
-        <v>5.4510000000000001E-3</v>
+        <v>5.4359999999999999E-3</v>
       </c>
       <c r="D10" s="2">
-        <v>1.916E-3</v>
+        <v>1.9109999999999999E-3</v>
       </c>
       <c r="E10" s="2">
-        <v>1.2840000000000001E-2</v>
+        <v>1.2806E-2</v>
       </c>
       <c r="F10" s="2">
-        <v>8.5990000000000007E-3</v>
+        <v>8.5760000000000003E-3</v>
       </c>
       <c r="G10" s="2">
         <v>0</v>
@@ -1276,13 +1276,13 @@
         <v>0</v>
       </c>
       <c r="J10" s="2">
-        <v>0.108443</v>
+        <v>0.108153</v>
       </c>
       <c r="K10" s="2">
-        <v>1.1789999999999999E-3</v>
+        <v>1.176E-3</v>
       </c>
       <c r="L10" s="2">
-        <v>5.0099999999999997E-3</v>
+        <v>4.9969999999999997E-3</v>
       </c>
       <c r="M10" s="2">
         <v>0</v>
@@ -1297,13 +1297,13 @@
         <v>0</v>
       </c>
       <c r="Q10" s="2">
-        <v>5.6080000000000001E-3</v>
+        <v>5.5929999999999999E-3</v>
       </c>
       <c r="R10" s="2">
-        <v>4.0000000000000002E-4</v>
+        <v>3.9899999999999999E-4</v>
       </c>
       <c r="S10" s="2">
-        <v>1.2872E-2</v>
+        <v>1.2839E-2</v>
       </c>
       <c r="T10" s="2">
         <v>0</v>
@@ -1312,10 +1312,10 @@
         <v>0</v>
       </c>
       <c r="V10" s="2">
-        <v>4.4099999999999999E-4</v>
+        <v>4.4000000000000002E-4</v>
       </c>
       <c r="W10" s="2">
-        <v>2.5099999999999998E-4</v>
+        <v>2.5000000000000001E-4</v>
       </c>
       <c r="X10" s="2">
         <v>0</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="2">
-        <v>4.8240000000000002E-3</v>
+        <v>4.8120000000000003E-3</v>
       </c>
       <c r="AA10" s="2">
         <v>0</v>
@@ -1339,7 +1339,7 @@
         <v>0</v>
       </c>
       <c r="AE10" s="2">
-        <v>9.9618999999999999E-2</v>
+        <v>9.9352999999999997E-2</v>
       </c>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
@@ -1354,16 +1354,16 @@
         <v>0</v>
       </c>
       <c r="C11" s="2">
-        <v>1.1130000000000001E-3</v>
+        <v>1.1100000000000001E-3</v>
       </c>
       <c r="D11" s="2">
         <v>0</v>
       </c>
       <c r="E11" s="2">
-        <v>8.5970000000000005E-3</v>
+        <v>8.574E-3</v>
       </c>
       <c r="F11" s="2">
-        <v>6.8099999999999996E-4</v>
+        <v>6.7900000000000002E-4</v>
       </c>
       <c r="G11" s="2">
         <v>0</v>
@@ -1378,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="2">
-        <v>5.7460000000000002E-3</v>
+        <v>5.731E-3</v>
       </c>
       <c r="L11" s="2">
         <v>0</v>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="P11" s="2">
-        <v>4.5199999999999998E-4</v>
+        <v>4.5100000000000001E-4</v>
       </c>
       <c r="Q11" s="2">
         <v>0</v>
@@ -1411,7 +1411,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="2">
-        <v>6.9700000000000003E-4</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W11" s="2">
         <v>0</v>
@@ -1426,7 +1426,7 @@
         <v>0</v>
       </c>
       <c r="AA11" s="2">
-        <v>5.5400000000000002E-4</v>
+        <v>5.5199999999999997E-4</v>
       </c>
       <c r="AB11" s="2">
         <v>0</v>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AE11" s="2">
-        <v>2.4629999999999999E-3</v>
+        <v>2.4559999999999998E-3</v>
       </c>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
@@ -1456,13 +1456,13 @@
         <v>0</v>
       </c>
       <c r="D12" s="2">
-        <v>4.6999999999999999E-4</v>
+        <v>4.6799999999999999E-4</v>
       </c>
       <c r="E12" s="2">
         <v>0</v>
       </c>
       <c r="F12" s="2">
-        <v>5.3790000000000001E-3</v>
+        <v>5.3639999999999998E-3</v>
       </c>
       <c r="G12" s="2">
         <v>0</v>
@@ -1480,7 +1480,7 @@
         <v>0</v>
       </c>
       <c r="L12" s="2">
-        <v>2.5539999999999998E-3</v>
+        <v>2.5469999999999998E-3</v>
       </c>
       <c r="M12" s="2">
         <v>0</v>
@@ -1537,7 +1537,7 @@
         <v>0</v>
       </c>
       <c r="AE12" s="2">
-        <v>2.8319999999999999E-3</v>
+        <v>2.8240000000000001E-3</v>
       </c>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
@@ -1549,13 +1549,13 @@
         <v>0</v>
       </c>
       <c r="B13" s="2">
-        <v>1.34E-4</v>
+        <v>1.3300000000000001E-4</v>
       </c>
       <c r="C13" s="2">
         <v>0</v>
       </c>
       <c r="D13" s="2">
-        <v>1.3029999999999999E-3</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="E13" s="2">
         <v>0</v>
@@ -1582,13 +1582,13 @@
         <v>0</v>
       </c>
       <c r="M13" s="2">
-        <v>5.2352000000000003E-2</v>
+        <v>5.2212000000000001E-2</v>
       </c>
       <c r="N13" s="2">
         <v>0</v>
       </c>
       <c r="O13" s="2">
-        <v>6.992E-3</v>
+        <v>6.973E-3</v>
       </c>
       <c r="P13" s="2">
         <v>0</v>
@@ -1630,13 +1630,13 @@
         <v>0</v>
       </c>
       <c r="AC13" s="2">
-        <v>7.1900000000000002E-4</v>
+        <v>7.1699999999999997E-4</v>
       </c>
       <c r="AD13" s="2">
         <v>0</v>
       </c>
       <c r="AE13" s="2">
-        <v>1.768E-3</v>
+        <v>1.763E-3</v>
       </c>
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
@@ -1684,7 +1684,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="2">
-        <v>1.405E-3</v>
+        <v>1.4009999999999999E-3</v>
       </c>
       <c r="O14" s="2">
         <v>0</v>
@@ -1780,13 +1780,13 @@
         <v>0</v>
       </c>
       <c r="M15" s="2">
-        <v>1.1709999999999999E-3</v>
+        <v>1.168E-3</v>
       </c>
       <c r="N15" s="2">
         <v>0</v>
       </c>
       <c r="O15" s="2">
-        <v>7.0200000000000004E-4</v>
+        <v>7.0100000000000002E-4</v>
       </c>
       <c r="P15" s="2">
         <v>0</v>
@@ -1828,13 +1828,13 @@
         <v>0</v>
       </c>
       <c r="AC15" s="2">
-        <v>2.4000000000000001E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AD15" s="2">
         <v>0</v>
       </c>
       <c r="AE15" s="2">
-        <v>7.1199999999999996E-4</v>
+        <v>7.1000000000000002E-4</v>
       </c>
       <c r="AF15" s="1"/>
       <c r="AG15" s="1"/>
@@ -1843,19 +1843,19 @@
     </row>
     <row r="16" spans="1:35">
       <c r="A16" s="2">
-        <v>5.1500000000000005E-4</v>
+        <v>5.1400000000000003E-4</v>
       </c>
       <c r="B16" s="2">
-        <v>9.9299999999999996E-4</v>
+        <v>9.8999999999999999E-4</v>
       </c>
       <c r="C16" s="2">
-        <v>0.14616899999999999</v>
+        <v>0.14577799999999999</v>
       </c>
       <c r="D16" s="2">
-        <v>8.3299999999999997E-4</v>
+        <v>8.3100000000000003E-4</v>
       </c>
       <c r="E16" s="2">
-        <v>1.5174999999999999E-2</v>
+        <v>1.5134E-2</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
@@ -1867,13 +1867,13 @@
         <v>0</v>
       </c>
       <c r="I16" s="2">
-        <v>2.9E-4</v>
+        <v>2.8899999999999998E-4</v>
       </c>
       <c r="J16" s="2">
         <v>0</v>
       </c>
       <c r="K16" s="2">
-        <v>8.8000000000000003E-4</v>
+        <v>8.7799999999999998E-4</v>
       </c>
       <c r="L16" s="2">
         <v>0</v>
@@ -1882,31 +1882,31 @@
         <v>0</v>
       </c>
       <c r="N16" s="2">
-        <v>3.7399999999999998E-4</v>
+        <v>3.7300000000000001E-4</v>
       </c>
       <c r="O16" s="2">
         <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>1.2677020000000001</v>
+        <v>1.2645040000000001</v>
       </c>
       <c r="Q16" s="2">
-        <v>4.0489999999999996E-3</v>
+        <v>4.0390000000000001E-3</v>
       </c>
       <c r="R16" s="2">
-        <v>0.26593099999999997</v>
+        <v>0.26526</v>
       </c>
       <c r="S16" s="2">
-        <v>3.6000000000000002E-4</v>
+        <v>3.59E-4</v>
       </c>
       <c r="T16" s="2">
-        <v>9.0329999999999994E-3</v>
+        <v>9.0100000000000006E-3</v>
       </c>
       <c r="U16" s="2">
         <v>0</v>
       </c>
       <c r="V16" s="2">
-        <v>3.9379999999999997E-3</v>
+        <v>3.9280000000000001E-3</v>
       </c>
       <c r="W16" s="2">
         <v>0</v>
@@ -1915,16 +1915,16 @@
         <v>0</v>
       </c>
       <c r="Y16" s="2">
-        <v>9.0620000000000006E-3</v>
+        <v>9.0390000000000002E-3</v>
       </c>
       <c r="Z16" s="2">
-        <v>6.5399999999999996E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AA16" s="2">
         <v>0</v>
       </c>
       <c r="AB16" s="2">
-        <v>2.4000000000000001E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AC16" s="2">
         <v>0</v>
@@ -1933,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="AE16" s="2">
-        <v>3.1688000000000001E-2</v>
+        <v>3.1607999999999997E-2</v>
       </c>
       <c r="AF16" s="1"/>
       <c r="AG16" s="1"/>
@@ -1942,25 +1942,25 @@
     </row>
     <row r="17" spans="1:35">
       <c r="A17" s="2">
-        <v>1.6160000000000001E-2</v>
+        <v>1.6115999999999998E-2</v>
       </c>
       <c r="B17" s="2">
-        <v>1.8540000000000001E-2</v>
+        <v>1.8489999999999999E-2</v>
       </c>
       <c r="C17" s="2">
-        <v>8.0549999999999997E-3</v>
+        <v>8.0330000000000002E-3</v>
       </c>
       <c r="D17" s="2">
-        <v>0.113506</v>
+        <v>0.113202</v>
       </c>
       <c r="E17" s="2">
-        <v>1.867E-3</v>
+        <v>1.8619999999999999E-3</v>
       </c>
       <c r="F17" s="2">
-        <v>5.8821999999999999E-2</v>
+        <v>5.8665000000000002E-2</v>
       </c>
       <c r="G17" s="2">
-        <v>2.8410000000000002E-3</v>
+        <v>2.833E-3</v>
       </c>
       <c r="H17" s="2">
         <v>0</v>
@@ -1969,16 +1969,16 @@
         <v>0</v>
       </c>
       <c r="J17" s="2">
-        <v>1.6169999999999999E-3</v>
+        <v>1.6119999999999999E-3</v>
       </c>
       <c r="K17" s="2">
         <v>0</v>
       </c>
       <c r="L17" s="2">
-        <v>2.9350000000000001E-3</v>
+        <v>2.9269999999999999E-3</v>
       </c>
       <c r="M17" s="2">
-        <v>4.6799999999999999E-4</v>
+        <v>4.6700000000000002E-4</v>
       </c>
       <c r="N17" s="2">
         <v>0</v>
@@ -1987,28 +1987,28 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>8.3999999999999995E-3</v>
+        <v>8.3789999999999993E-3</v>
       </c>
       <c r="Q17" s="2">
-        <v>3.7176960000000001</v>
+        <v>3.7083170000000001</v>
       </c>
       <c r="R17" s="2">
-        <v>1.0120000000000001E-3</v>
+        <v>1.0089999999999999E-3</v>
       </c>
       <c r="S17" s="2">
-        <v>0.72534699999999996</v>
+        <v>0.72351699999999997</v>
       </c>
       <c r="T17" s="2">
-        <v>2.1432E-2</v>
+        <v>2.1378000000000001E-2</v>
       </c>
       <c r="U17" s="2">
-        <v>9.554E-3</v>
+        <v>9.5300000000000003E-3</v>
       </c>
       <c r="V17" s="2">
-        <v>4.7869999999999996E-3</v>
+        <v>4.7739999999999996E-3</v>
       </c>
       <c r="W17" s="2">
-        <v>2.4369999999999999E-3</v>
+        <v>2.431E-3</v>
       </c>
       <c r="X17" s="2">
         <v>0</v>
@@ -2017,22 +2017,22 @@
         <v>0</v>
       </c>
       <c r="Z17" s="2">
-        <v>3.5784999999999997E-2</v>
+        <v>3.5693999999999997E-2</v>
       </c>
       <c r="AA17" s="2">
         <v>0</v>
       </c>
       <c r="AB17" s="2">
-        <v>1.8450000000000001E-3</v>
+        <v>1.8400000000000001E-3</v>
       </c>
       <c r="AC17" s="2">
-        <v>7.6499999999999995E-4</v>
+        <v>7.6300000000000001E-4</v>
       </c>
       <c r="AD17" s="2">
-        <v>3.8299999999999999E-4</v>
+        <v>3.8200000000000002E-4</v>
       </c>
       <c r="AE17" s="2">
-        <v>3.3009999999999998E-2</v>
+        <v>3.2925999999999997E-2</v>
       </c>
       <c r="AF17" s="1"/>
       <c r="AG17" s="1"/>
@@ -2044,19 +2044,19 @@
         <v>0</v>
       </c>
       <c r="B18" s="2">
-        <v>2.1580000000000002E-3</v>
+        <v>2.1519999999999998E-3</v>
       </c>
       <c r="C18" s="2">
-        <v>2.0181999999999999E-2</v>
+        <v>2.0128E-2</v>
       </c>
       <c r="D18" s="2">
         <v>0</v>
       </c>
       <c r="E18" s="2">
-        <v>4.7701E-2</v>
+        <v>4.7573999999999998E-2</v>
       </c>
       <c r="F18" s="2">
-        <v>1.1119999999999999E-3</v>
+        <v>1.109E-3</v>
       </c>
       <c r="G18" s="2">
         <v>0</v>
@@ -2071,7 +2071,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="2">
-        <v>1.6169999999999999E-3</v>
+        <v>1.6119999999999999E-3</v>
       </c>
       <c r="L18" s="2">
         <v>0</v>
@@ -2086,25 +2086,25 @@
         <v>0</v>
       </c>
       <c r="P18" s="2">
-        <v>6.0437999999999999E-2</v>
+        <v>6.0284999999999998E-2</v>
       </c>
       <c r="Q18" s="2">
         <v>5.5000000000000002E-5</v>
       </c>
       <c r="R18" s="2">
-        <v>0.36191499999999999</v>
+        <v>0.36100199999999999</v>
       </c>
       <c r="S18" s="2">
-        <v>3.8349999999999999E-3</v>
+        <v>3.826E-3</v>
       </c>
       <c r="T18" s="2">
-        <v>2.5600000000000002E-3</v>
+        <v>2.5539999999999998E-3</v>
       </c>
       <c r="U18" s="2">
         <v>0</v>
       </c>
       <c r="V18" s="2">
-        <v>2.0920000000000001E-3</v>
+        <v>2.0860000000000002E-3</v>
       </c>
       <c r="W18" s="2">
         <v>0</v>
@@ -2113,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="Y18" s="2">
-        <v>4.0016999999999997E-2</v>
+        <v>3.9916E-2</v>
       </c>
       <c r="Z18" s="2">
         <v>0</v>
@@ -2131,7 +2131,7 @@
         <v>0</v>
       </c>
       <c r="AE18" s="2">
-        <v>3.2399999999999998E-2</v>
+        <v>3.2318E-2</v>
       </c>
       <c r="AF18" s="1"/>
       <c r="AG18" s="1"/>
@@ -2140,43 +2140,43 @@
     </row>
     <row r="19" spans="1:35">
       <c r="A19" s="2">
-        <v>5.0299999999999997E-4</v>
+        <v>5.0199999999999995E-4</v>
       </c>
       <c r="B19" s="2">
-        <v>7.6E-3</v>
+        <v>7.5799999999999999E-3</v>
       </c>
       <c r="C19" s="2">
-        <v>1.1130000000000001E-3</v>
+        <v>1.1100000000000001E-3</v>
       </c>
       <c r="D19" s="2">
-        <v>2.6391999999999999E-2</v>
+        <v>2.6321000000000001E-2</v>
       </c>
       <c r="E19" s="2">
-        <v>9.2299999999999999E-4</v>
+        <v>9.2000000000000003E-4</v>
       </c>
       <c r="F19" s="2">
-        <v>5.4149999999999997E-2</v>
+        <v>5.4004999999999997E-2</v>
       </c>
       <c r="G19" s="2">
-        <v>3.7919999999999998E-3</v>
+        <v>3.7820000000000002E-3</v>
       </c>
       <c r="H19" s="2">
-        <v>6.4800000000000003E-4</v>
+        <v>6.4599999999999998E-4</v>
       </c>
       <c r="I19" s="2">
-        <v>7.1599999999999995E-4</v>
+        <v>7.1400000000000001E-4</v>
       </c>
       <c r="J19" s="2">
-        <v>3.4000000000000002E-4</v>
+        <v>3.39E-4</v>
       </c>
       <c r="K19" s="2">
         <v>0</v>
       </c>
       <c r="L19" s="2">
-        <v>6.4429999999999999E-3</v>
+        <v>6.4260000000000003E-3</v>
       </c>
       <c r="M19" s="2">
-        <v>3.7399999999999998E-4</v>
+        <v>3.7300000000000001E-4</v>
       </c>
       <c r="N19" s="2">
         <v>0</v>
@@ -2185,28 +2185,28 @@
         <v>0</v>
       </c>
       <c r="P19" s="2">
-        <v>8.9099999999999997E-4</v>
+        <v>8.8900000000000003E-4</v>
       </c>
       <c r="Q19" s="2">
-        <v>0.15104699999999999</v>
+        <v>0.15066599999999999</v>
       </c>
       <c r="R19" s="2">
-        <v>3.0360000000000001E-3</v>
+        <v>3.0279999999999999E-3</v>
       </c>
       <c r="S19" s="2">
-        <v>0.71881600000000001</v>
+        <v>0.71700200000000003</v>
       </c>
       <c r="T19" s="2">
-        <v>6.1339999999999997E-3</v>
+        <v>6.1180000000000002E-3</v>
       </c>
       <c r="U19" s="2">
-        <v>4.9969999999999997E-3</v>
+        <v>4.9849999999999998E-3</v>
       </c>
       <c r="V19" s="2">
-        <v>6.7140000000000003E-3</v>
+        <v>6.6969999999999998E-3</v>
       </c>
       <c r="W19" s="2">
-        <v>6.3E-3</v>
+        <v>6.2839999999999997E-3</v>
       </c>
       <c r="X19" s="2">
         <v>0</v>
@@ -2215,22 +2215,22 @@
         <v>0</v>
       </c>
       <c r="Z19" s="2">
-        <v>7.0707999999999993E-2</v>
+        <v>7.0529999999999995E-2</v>
       </c>
       <c r="AA19" s="2">
-        <v>1.207E-3</v>
+        <v>1.204E-3</v>
       </c>
       <c r="AB19" s="2">
-        <v>4.8000000000000001E-4</v>
+        <v>4.7800000000000002E-4</v>
       </c>
       <c r="AC19" s="2">
-        <v>2.4000000000000001E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AD19" s="2">
-        <v>3.8299999999999999E-4</v>
+        <v>3.8200000000000002E-4</v>
       </c>
       <c r="AE19" s="2">
-        <v>3.4117000000000001E-2</v>
+        <v>3.4029999999999998E-2</v>
       </c>
       <c r="AF19" s="1"/>
       <c r="AG19" s="1"/>
@@ -2245,31 +2245,31 @@
         <v>0</v>
       </c>
       <c r="C20" s="2">
-        <v>5.4450000000000002E-3</v>
+        <v>5.4299999999999999E-3</v>
       </c>
       <c r="D20" s="2">
-        <v>4.6999999999999999E-4</v>
+        <v>4.6799999999999999E-4</v>
       </c>
       <c r="E20" s="2">
-        <v>5.5400000000000002E-4</v>
+        <v>5.53E-4</v>
       </c>
       <c r="F20" s="2">
         <v>0</v>
       </c>
       <c r="G20" s="2">
-        <v>9.5580000000000005E-3</v>
+        <v>9.5329999999999998E-3</v>
       </c>
       <c r="H20" s="2">
         <v>0</v>
       </c>
       <c r="I20" s="2">
-        <v>1.2509999999999999E-3</v>
+        <v>1.248E-3</v>
       </c>
       <c r="J20" s="2">
         <v>0</v>
       </c>
       <c r="K20" s="2">
-        <v>6.38E-4</v>
+        <v>6.3699999999999998E-4</v>
       </c>
       <c r="L20" s="2">
         <v>0</v>
@@ -2284,25 +2284,25 @@
         <v>0</v>
       </c>
       <c r="P20" s="2">
-        <v>9.01E-4</v>
+        <v>8.9899999999999995E-4</v>
       </c>
       <c r="Q20" s="2">
-        <v>9.9799999999999997E-4</v>
+        <v>9.9599999999999992E-4</v>
       </c>
       <c r="R20" s="2">
         <v>4.0000000000000003E-5</v>
       </c>
       <c r="S20" s="2">
-        <v>7.67E-4</v>
+        <v>7.6499999999999995E-4</v>
       </c>
       <c r="T20" s="2">
-        <v>0.11144900000000001</v>
+        <v>0.111168</v>
       </c>
       <c r="U20" s="2">
         <v>0</v>
       </c>
       <c r="V20" s="2">
-        <v>4.2251999999999998E-2</v>
+        <v>4.2146000000000003E-2</v>
       </c>
       <c r="W20" s="2">
         <v>3.6600000000000001E-4</v>
@@ -2317,7 +2317,7 @@
         <v>0</v>
       </c>
       <c r="AA20" s="2">
-        <v>2.209E-3</v>
+        <v>2.2039999999999998E-3</v>
       </c>
       <c r="AB20" s="2">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="AE20" s="2">
-        <v>3.2260000000000001E-3</v>
+        <v>3.2169999999999998E-3</v>
       </c>
       <c r="AF20" s="1"/>
       <c r="AG20" s="1"/>
@@ -2347,19 +2347,19 @@
         <v>0</v>
       </c>
       <c r="D21" s="2">
-        <v>7.2800000000000002E-4</v>
+        <v>7.2599999999999997E-4</v>
       </c>
       <c r="E21" s="2">
         <v>0</v>
       </c>
       <c r="F21" s="2">
-        <v>1.0330000000000001E-3</v>
+        <v>1.0300000000000001E-3</v>
       </c>
       <c r="G21" s="2">
-        <v>9.19E-4</v>
+        <v>9.1600000000000004E-4</v>
       </c>
       <c r="H21" s="2">
-        <v>5.8E-4</v>
+        <v>5.7899999999999998E-4</v>
       </c>
       <c r="I21" s="2">
         <v>0</v>
@@ -2392,19 +2392,19 @@
         <v>0</v>
       </c>
       <c r="S21" s="2">
-        <v>7.67E-4</v>
+        <v>7.6499999999999995E-4</v>
       </c>
       <c r="T21" s="2">
-        <v>2.5600000000000002E-3</v>
+        <v>2.5539999999999998E-3</v>
       </c>
       <c r="U21" s="2">
-        <v>4.0236000000000001E-2</v>
+        <v>4.0134000000000003E-2</v>
       </c>
       <c r="V21" s="2">
-        <v>1.057E-3</v>
+        <v>1.0549999999999999E-3</v>
       </c>
       <c r="W21" s="2">
-        <v>1.6404999999999999E-2</v>
+        <v>1.6362999999999999E-2</v>
       </c>
       <c r="X21" s="2">
         <v>0</v>
@@ -2419,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="AB21" s="2">
-        <v>2.4000000000000001E-4</v>
+        <v>2.3900000000000001E-4</v>
       </c>
       <c r="AC21" s="2">
         <v>0</v>
@@ -2428,7 +2428,7 @@
         <v>0</v>
       </c>
       <c r="AE21" s="2">
-        <v>6.0990000000000003E-3</v>
+        <v>6.084E-3</v>
       </c>
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
@@ -2455,13 +2455,13 @@
         <v>0</v>
       </c>
       <c r="G22" s="2">
-        <v>9.19E-4</v>
+        <v>9.1600000000000004E-4</v>
       </c>
       <c r="H22" s="2">
         <v>0</v>
       </c>
       <c r="I22" s="2">
-        <v>2.3700000000000001E-3</v>
+        <v>2.3630000000000001E-3</v>
       </c>
       <c r="J22" s="2">
         <v>0</v>
@@ -2494,13 +2494,13 @@
         <v>0</v>
       </c>
       <c r="T22" s="2">
-        <v>2.4399999999999999E-3</v>
+        <v>2.434E-3</v>
       </c>
       <c r="U22" s="2">
         <v>0</v>
       </c>
       <c r="V22" s="2">
-        <v>2.0145E-2</v>
+        <v>2.0094999999999998E-2</v>
       </c>
       <c r="W22" s="2">
         <v>0</v>
@@ -2515,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="AA22" s="2">
-        <v>3.1110000000000001E-3</v>
+        <v>3.1029999999999999E-3</v>
       </c>
       <c r="AB22" s="2">
         <v>0</v>
@@ -2527,7 +2527,7 @@
         <v>0</v>
       </c>
       <c r="AE22" s="2">
-        <v>1.8010000000000001E-3</v>
+        <v>1.797E-3</v>
       </c>
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
@@ -2545,7 +2545,7 @@
         <v>0</v>
       </c>
       <c r="D23" s="2">
-        <v>4.6999999999999999E-4</v>
+        <v>4.6799999999999999E-4</v>
       </c>
       <c r="E23" s="2">
         <v>0</v>
@@ -2569,7 +2569,7 @@
         <v>0</v>
       </c>
       <c r="L23" s="2">
-        <v>6.38E-4</v>
+        <v>6.3699999999999998E-4</v>
       </c>
       <c r="M23" s="2">
         <v>0</v>
@@ -2593,7 +2593,7 @@
         <v>0</v>
       </c>
       <c r="T23" s="2">
-        <v>3.7300000000000001E-4</v>
+        <v>3.7199999999999999E-4</v>
       </c>
       <c r="U23" s="2">
         <v>1.2E-4</v>
@@ -2602,7 +2602,7 @@
         <v>0</v>
       </c>
       <c r="W23" s="2">
-        <v>3.222E-3</v>
+        <v>3.2139999999999998E-3</v>
       </c>
       <c r="X23" s="2">
         <v>0</v>
@@ -2626,7 +2626,7 @@
         <v>0</v>
       </c>
       <c r="AE23" s="2">
-        <v>2.8479999999999998E-3</v>
+        <v>2.8410000000000002E-3</v>
       </c>
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
@@ -2740,13 +2740,13 @@
         <v>0</v>
       </c>
       <c r="C25" s="2">
-        <v>1.047E-3</v>
+        <v>1.044E-3</v>
       </c>
       <c r="D25" s="2">
         <v>0</v>
       </c>
       <c r="E25" s="2">
-        <v>8.5749999999999993E-3</v>
+        <v>8.5520000000000006E-3</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -2764,7 +2764,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="2">
-        <v>3.4000000000000002E-4</v>
+        <v>3.39E-4</v>
       </c>
       <c r="L25" s="2">
         <v>0</v>
@@ -2779,16 +2779,16 @@
         <v>0</v>
       </c>
       <c r="P25" s="2">
-        <v>4.4000000000000002E-4</v>
+        <v>4.3800000000000002E-4</v>
       </c>
       <c r="Q25" s="2">
         <v>0</v>
       </c>
       <c r="R25" s="2">
-        <v>1.5552E-2</v>
+        <v>1.5512E-2</v>
       </c>
       <c r="S25" s="2">
-        <v>7.67E-4</v>
+        <v>7.6499999999999995E-4</v>
       </c>
       <c r="T25" s="2">
         <v>0</v>
@@ -2797,7 +2797,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="2">
-        <v>2.8930000000000002E-3</v>
+        <v>2.8860000000000001E-3</v>
       </c>
       <c r="W25" s="2">
         <v>0</v>
@@ -2806,13 +2806,13 @@
         <v>0</v>
       </c>
       <c r="Y25" s="2">
-        <v>1.5006E-2</v>
+        <v>1.4968E-2</v>
       </c>
       <c r="Z25" s="2">
-        <v>3.6000000000000002E-4</v>
+        <v>3.59E-4</v>
       </c>
       <c r="AA25" s="2">
-        <v>3.6000000000000002E-4</v>
+        <v>3.59E-4</v>
       </c>
       <c r="AB25" s="2">
         <v>0</v>
@@ -2824,7 +2824,7 @@
         <v>0</v>
       </c>
       <c r="AE25" s="2">
-        <v>1.0054E-2</v>
+        <v>1.0028E-2</v>
       </c>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
@@ -2839,16 +2839,16 @@
         <v>0</v>
       </c>
       <c r="C26" s="2">
-        <v>9.9299999999999996E-4</v>
+        <v>9.8999999999999999E-4</v>
       </c>
       <c r="D26" s="2">
-        <v>8.3299999999999997E-4</v>
+        <v>8.3100000000000003E-4</v>
       </c>
       <c r="E26" s="2">
         <v>0</v>
       </c>
       <c r="F26" s="2">
-        <v>2.9940000000000001E-3</v>
+        <v>2.9859999999999999E-3</v>
       </c>
       <c r="G26" s="2">
         <v>1.17E-4</v>
@@ -2860,19 +2860,19 @@
         <v>0</v>
       </c>
       <c r="J26" s="2">
-        <v>1.3179999999999999E-3</v>
+        <v>1.315E-3</v>
       </c>
       <c r="K26" s="2">
         <v>0</v>
       </c>
       <c r="L26" s="2">
-        <v>2.3579999999999999E-3</v>
+        <v>2.3519999999999999E-3</v>
       </c>
       <c r="M26" s="2">
         <v>0</v>
       </c>
       <c r="N26" s="2">
-        <v>6.0800000000000003E-4</v>
+        <v>6.0599999999999998E-4</v>
       </c>
       <c r="O26" s="2">
         <v>0</v>
@@ -2881,25 +2881,25 @@
         <v>0</v>
       </c>
       <c r="Q26" s="2">
-        <v>8.7500000000000002E-4</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="R26" s="2">
-        <v>8.7500000000000002E-4</v>
+        <v>8.7299999999999997E-4</v>
       </c>
       <c r="S26" s="2">
-        <v>1.8658999999999999E-2</v>
+        <v>1.8612E-2</v>
       </c>
       <c r="T26" s="2">
-        <v>9.6199999999999996E-4</v>
+        <v>9.59E-4</v>
       </c>
       <c r="U26" s="2">
         <v>0</v>
       </c>
       <c r="V26" s="2">
-        <v>8.83E-4</v>
+        <v>8.8099999999999995E-4</v>
       </c>
       <c r="W26" s="2">
-        <v>1.4660000000000001E-3</v>
+        <v>1.462E-3</v>
       </c>
       <c r="X26" s="2">
         <v>0</v>
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="2">
-        <v>1.4531000000000001E-2</v>
+        <v>1.4494E-2</v>
       </c>
       <c r="AA26" s="2">
         <v>0</v>
@@ -2923,7 +2923,7 @@
         <v>0</v>
       </c>
       <c r="AE26" s="2">
-        <v>8.9560000000000004E-3</v>
+        <v>8.933E-3</v>
       </c>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
@@ -2956,7 +2956,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="2">
-        <v>2.9E-4</v>
+        <v>2.8899999999999998E-4</v>
       </c>
       <c r="J27" s="2">
         <v>0</v>
@@ -2995,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="V27" s="2">
-        <v>6.9700000000000003E-4</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W27" s="2">
         <v>0</v>
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="AA27" s="2">
-        <v>6.5399999999999996E-4</v>
+        <v>6.5200000000000002E-4</v>
       </c>
       <c r="AB27" s="2">
         <v>0</v>
@@ -3070,7 +3070,7 @@
         <v>0</v>
       </c>
       <c r="N28" s="2">
-        <v>6.0800000000000003E-4</v>
+        <v>6.0599999999999998E-4</v>
       </c>
       <c r="O28" s="2">
         <v>0</v>
@@ -3088,13 +3088,13 @@
         <v>0</v>
       </c>
       <c r="T28" s="2">
-        <v>4.8099999999999998E-4</v>
+        <v>4.8000000000000001E-4</v>
       </c>
       <c r="U28" s="2">
         <v>0</v>
       </c>
       <c r="V28" s="2">
-        <v>6.9700000000000003E-4</v>
+        <v>6.9499999999999998E-4</v>
       </c>
       <c r="W28" s="2">
         <v>0</v>
@@ -3112,16 +3112,16 @@
         <v>0</v>
       </c>
       <c r="AB28" s="2">
-        <v>5.7540000000000004E-3</v>
+        <v>5.7400000000000003E-3</v>
       </c>
       <c r="AC28" s="2">
         <v>0</v>
       </c>
       <c r="AD28" s="2">
-        <v>7.6499999999999995E-4</v>
+        <v>7.6300000000000001E-4</v>
       </c>
       <c r="AE28" s="2">
-        <v>7.0399999999999998E-4</v>
+        <v>7.0200000000000004E-4</v>
       </c>
       <c r="AF28" s="1"/>
       <c r="AG28" s="1"/>
@@ -3214,13 +3214,13 @@
         <v>0</v>
       </c>
       <c r="AC29" s="2">
-        <v>4.8000000000000001E-4</v>
+        <v>4.7800000000000002E-4</v>
       </c>
       <c r="AD29" s="2">
         <v>0</v>
       </c>
       <c r="AE29" s="2">
-        <v>3.5199999999999999E-4</v>
+        <v>3.5100000000000002E-4</v>
       </c>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>

</xml_diff>

<commit_message>
print chi2 for THStack plot fit
</commit_message>
<xml_diff>
--- a/Belle2/efficiency_data.xlsx
+++ b/Belle2/efficiency_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwpark\Desktop\git\Belle2_script\Belle2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7ADD60-1D84-46E7-B56E-940017F5F899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A674EB38-D9D5-4907-AFC3-F31A8661FF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>